<commit_message>
fix: bind the login queries, add csrf and regenerate the session id
index.php built its login query from $_REQUEST, so a username ending in
' -- or ' OR '1'='1 removed the password check and logged in as the first
active user. Prepared statement with both values bound now; the rules for
who may log in are unchanged.

admin_multi_logins.php had the same query and also echoed it, password
included, to the page. Bound and the echo removed.

Both pages: csrf + form token on the post, session id regenerated and
tokens dropped on success, failed logins written to the error log. The
login form no longer ships a prefilled username.

Report filter forms left as they are.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1333,17 +1333,47 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>db/bie.sql</t>
+          <t>index.php</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
         </is>
       </c>
       <c r="C52" s="4" t="n"/>
       <c r="D52" s="4" t="n"/>
       <c r="E52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>admin_multi_logins.php</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>db/bie.sql</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="n"/>
+      <c r="D54" s="4" t="n"/>
+      <c r="E54" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: item stock history report runs for all items, newest row first
Leaving the item blank now reports every item for the chosen branch and
date range. fnValidate() was alerting "Item ..!" and the result block was
guarded by item_id != '', so a blank item rendered nothing at all.

On the all-items run an Item column is added between Date and Type, its
name joined from tbl_item_details rather than looked up once per row. The
heading and the no-rows colspans follow the column count instead of being
hardcoded, so the single-item view is unchanged.

Sort is now trans_date DESC, auto_id DESC - latest movement on top. The
item filter is appended to the WHERE only when an item is chosen; branch,
date range, stock_status and trans_qty conditions are untouched.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -801,7 +801,11 @@
           <t>2026-09-23 | Runs from $_REQUEST so the stock list View All link works; query now bound instead of interpolated.</t>
         </is>
       </c>
-      <c r="D17" s="4" t="n"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-02 | Item is optional - blank reports every item for the branch and range, with an Item column added and the name joined in rather than looked up per row. Sort changed to trans_date DESC, auto_id DESC so the latest movement is on top. Heading and empty-state colspans now follow the column count.</t>
+        </is>
+      </c>
       <c r="E17" s="4" t="n"/>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
fix(db): step 7 failed on the server, and the file was not safe to re-run
Step 7 was one UNION ALL whose first branch read information_schema, and
MariaDB then looked for the plain table names in information_schema as
well: #1109 Unknown table 'tbl_user_rights' in information_schema. Split
into five separate queries. Steps 1 to 6 were unaffected - step 7 only
reports.

Two re-run hazards found while fixing it. There is no unique key on
tbl_user_rights (usr_id, mm_id, sm_id), so running the file twice would
have doubled the new rights rows; both grants now skip anyone who already
has the row. The step 4b backup would have failed, or clobbered the first
backup, on a second run; it is CREATE TABLE IF NOT EXISTS now.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -1349,7 +1349,11 @@
           <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
         </is>
       </c>
-      <c r="C52" s="4" t="n"/>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
+        </is>
+      </c>
       <c r="D52" s="4" t="n"/>
       <c r="E52" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
fix: Stock List wrote no cells for Rajapalayam
The branch headers were built by looping mst_branch, so three active
branches gave three headers, but the row loop wrote exactly two cells,
hardcoded to ho_stock and kl_stock. Every row was a cell short of its
header, so the last column had nothing under it and read as merged.

The branch list is now read once into an array and both the header and the
rows walk it, each row taking that branch's own branch_stock_field. A
branch added to mst_branch gets its column with no code change.

Also on this page: an item with no tbl_item_stock row produced no branch
cells at all and now reads 0.000 under each branch, the per-item stock
lookup is bound instead of concatenated, and the no-rows colspan follows
the branch count.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1345,46 +1345,46 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>db/post_upload_051026.sql</t>
+          <t>rpt_all_store_stock_list.php</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
-        </is>
-      </c>
+          <t>2026-10-06 | Branch columns driven from mst_branch. The header looped the branch table but the rows wrote only ho_stock and kl_stock, so Rajapalayam had a header and no cells. An item with no tbl_item_stock row now reads 0.000 instead of dropping its cells, the item lookup is bound, and the empty-state colspan follows the branch count.</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="n"/>
       <c r="D52" s="4" t="n"/>
       <c r="E52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>index.php</t>
+          <t>db/post_upload_051026.sql</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="n"/>
+          <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
+        </is>
+      </c>
       <c r="D53" s="4" t="n"/>
       <c r="E53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>admin_multi_logins.php</t>
+          <t>index.php</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
+          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
         </is>
       </c>
       <c r="C54" s="4" t="n"/>
@@ -1394,17 +1394,32 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>db/bie.sql</t>
+          <t>admin_multi_logins.php</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
         </is>
       </c>
       <c r="C55" s="4" t="n"/>
       <c r="D55" s="4" t="n"/>
       <c r="E55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>db/bie.sql</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="n"/>
+      <c r="D56" s="4" t="n"/>
+      <c r="E56" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: multi UOM price save bound null for min and max discount
The multi UOM rows have never had branch_new_min_discount[] or
branch_new_max_discount[] fields, so the insert bound null into NOT NULL
columns and failed. Now binds the column default 0 when absent. With the
csrf token added earlier, the multi UOM save works for the first time.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -693,7 +693,11 @@
           <t>2026-10-06 | csrf token added to the multi UOM form - its Save and Update were always rejected.</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-06 | Multi UOM insert binds 0 for min / max discount when the row has no such field - it bound null and always failed on the NOT NULL column.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
db: post-upload script for 06-10-26 - principal master columns
Checked bie_db_061026.sql: every change from this work is live. Checking
every INSERT and UPDATE column in the code against that schema found one
gap: mst_principal never had the created_by, created_dtm, modify_by and
modify_dtm columns mst_principal.php writes, so adding or editing a
principal always failed. post_upload_061026.sql adds them.

Changelog: full list of buttons with their own onclick (21 in 10 files,
mst_supplier_approve.php added), each now confirmed to post its name; the
earlier DataTables warning note was the test machine's timezone data and
is withdrawn.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1478,46 +1478,46 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>db/post_upload_051026.sql</t>
+          <t>db/post_upload_061026.sql</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
-        </is>
-      </c>
+          <t>2026-10-06 | New. Checked against bie_db_061026.sql: every earlier change is live; adds the four audit columns mst_principal.php writes but the table never had.</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="n"/>
       <c r="D59" s="4" t="n"/>
       <c r="E59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>index.php</t>
+          <t>db/post_upload_051026.sql</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="n"/>
+          <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
+        </is>
+      </c>
       <c r="D60" s="4" t="n"/>
       <c r="E60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>admin_multi_logins.php</t>
+          <t>index.php</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
+          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
         </is>
       </c>
       <c r="C61" s="4" t="n"/>
@@ -1527,17 +1527,32 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>db/bie.sql</t>
+          <t>admin_multi_logins.php</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
         </is>
       </c>
       <c r="C62" s="4" t="n"/>
       <c r="D62" s="4" t="n"/>
       <c r="E62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>db/bie.sql</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="n"/>
+      <c r="D63" s="4" t="n"/>
+      <c r="E63" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1550,7 +1565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1638,24 +1653,16 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>tbl_user_rights</t>
+          <t>mst_principal</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | sm_id | Signed TINYINT widened to SMALLINT. It stopped at 127, so the rights rows for the new menus (147, 148) were silently clamped to 127 and the menus never showed.</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | mm_id | Signed TINYINT widened to SMALLINT, same reason - it was two main menus away from the same limit.</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | (rows) | Six clamped rows deleted (users 2/6/7, sm_id 127 under main menus 3 and 20); sm_id 147 and 148 granted to whoever holds the parent menu.</t>
-        </is>
-      </c>
+          <t>2026-10-06 | created_by, created_dtm, modify_by, modify_dtm | Added - mst_principal.php writes them on save and update, so both always failed with Unknown column. Existing rows get 0 / NULL.</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
@@ -1669,20 +1676,24 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>tbl_invoice_details</t>
+          <t>tbl_user_rights</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | inv_value, tax_value | 111 rows across 35 invoices rebuilt as net_value / (1 + vat/100); tax_value rebuilt with them. Backup taken as tbl_invoice_details_bkp_051026.</t>
+          <t>2026-10-05 | sm_id | Signed TINYINT widened to SMALLINT. It stopped at 127, so the rights rows for the new menus (147, 148) were silently clamped to 127 and the menus never showed.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | cgst_per, sgst_per, igst_per, cgst_val, sgst_val, igst_val | Optional tidy on the same 111 rows only.</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="n"/>
+          <t>2026-10-05 | mm_id | Signed TINYINT widened to SMALLINT, same reason - it was two main menus away from the same limit.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05 | (rows) | Six clamped rows deleted (users 2/6/7, sm_id 127 under main menus 3 and 20); sm_id 147 and 148 granted to whoever holds the parent menu.</t>
+        </is>
+      </c>
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
@@ -1696,133 +1707,133 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>tbl_stock_flow</t>
+          <t>tbl_invoice_details</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | trans_dir | Added CHAR(1). I = stock in (+), O = stock out (-). Backfilled GRN=I, INV/SALE=O.</t>
+          <t>2026-10-05 | inv_value, tax_value | 111 rows across 35 invoices rebuilt as net_value / (1 + vat/100); tax_value rebuilt with them. Backup taken as tbl_invoice_details_bkp_051026.</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | trans_remarks | Added VARCHAR(255). Reason / narration, mandatory on ADJ rows.</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | stock_field | Added VARCHAR(30). Which tbl_item_stock column was changed. Backfilled from mst_branch.</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | before_qty | INT to DECIMAL(12,3). Was truncating decimal stock.</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | trans_qty | INT to DECIMAL(12,3). Always a positive magnitude, direction is in trans_dir.</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | rcvd_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | after_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | reje_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | pend_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | trans_type | VARCHAR(8) to VARCHAR(10). Values GRN, INV, ADJ, OPEN, RET.</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | idx_sf_item_branch_date | Index added on (item_id, branch_id, trans_date) - what the reports filter on.</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | idx_sf_trans | Index added on (trans_type, trans_id).</t>
-        </is>
-      </c>
+          <t>2026-10-05 | cgst_per, sgst_per, igst_per, cgst_val, sgst_val, igst_val | Optional tidy on the same 111 rows only.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>tbl_stock_adjustment</t>
+          <t>tbl_stock_flow</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (new table) | Header for every manual stock correction. One row per adjustment.</t>
+          <t>2026-09-22 | trans_dir | Added CHAR(1). I = stock in (+), O = stock out (-). Backfilled GRN=I, INV/SALE=O.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | adj_id, adj_refno, adj_slno, adj_finyr | Key and reference number ADJ/nnnn/BIE/&lt;branch&gt;/&lt;finyr&gt;.</t>
+          <t>2026-09-22 | trans_remarks | Added VARCHAR(255). Reason / narration, mandatory on ADJ rows.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | adj_date, branch_id, stock_field, item_id | What was adjusted, where, and which stock column.</t>
+          <t>2026-09-22 | stock_field | Added VARCHAR(30). Which tbl_item_stock column was changed. Backfilled from mst_branch.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | adj_type, adj_qty, before_qty, after_qty | I = increase, D = decrease. adj_qty is always positive.</t>
+          <t>2026-09-22 | before_qty | INT to DECIMAL(12,3). Was truncating decimal stock.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | item_price, adj_reason, adj_status | Reason is mandatory. adj_status 1 = active, 0 = deleted.</t>
+          <t>2026-09-22 | trans_qty | INT to DECIMAL(12,3). Always a positive magnitude, direction is in trans_dir.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | created_by, created_dtm | Who made the adjustment and when.</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="n"/>
-      <c r="K5" s="4" t="n"/>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4" t="n"/>
+          <t>2026-09-22 | rcvd_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | after_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | reje_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | pend_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | trans_type | VARCHAR(8) to VARCHAR(10). Values GRN, INV, ADJ, OPEN, RET.</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | idx_sf_item_branch_date | Index added on (item_id, branch_id, trans_date) - what the reports filter on.</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | idx_sf_trans | Index added on (trans_type, trans_id).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>mst_sub_menu</t>
+          <t>tbl_stock_adjustment</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (row) | sm_id 147, mm_id 20 (Stores) - Stock Adjustment, stock_adjustment.php.</t>
+          <t>2026-09-22 | (new table) | Header for every manual stock correction. One row per adjustment.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 | (row) | sm_id 148, mm_id 3 (Item Masters) - Item Stock List, lst_item_stock.php.</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
+          <t>2026-09-22 | adj_id, adj_refno, adj_slno, adj_finyr | Key and reference number ADJ/nnnn/BIE/&lt;branch&gt;/&lt;finyr&gt;.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | adj_date, branch_id, stock_field, item_id | What was adjusted, where, and which stock column.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | adj_type, adj_qty, before_qty, after_qty | I = increase, D = decrease. adj_qty is always positive.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | item_price, adj_reason, adj_status | Reason is mandatory. adj_status 1 = active, 0 = deleted.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | created_by, created_dtm | Who made the adjustment and when.</t>
+        </is>
+      </c>
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
@@ -1833,17 +1844,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>tbl_user_rights</t>
+          <t>mst_sub_menu</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (rows) | sm_id 147 granted to every user who already has the Stores menu.</t>
+          <t>2026-09-22 | (row) | sm_id 147, mm_id 20 (Stores) - Stock Adjustment, stock_adjustment.php.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 | (rows) | sm_id 148 granted to every user who already has the Item Masters menu.</t>
+          <t>2026-09-23 | (row) | sm_id 148, mm_id 3 (Item Masters) - Item Stock List, lst_item_stock.php.</t>
         </is>
       </c>
       <c r="D7" s="4" t="n"/>
@@ -1860,15 +1871,19 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>tbl_item_stock</t>
+          <t>tbl_user_rights</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (no schema change) | Qty columns are now only written through fnApplyStockMovement(), never directly.</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n"/>
+          <t>2026-09-22 | (rows) | sm_id 147 granted to every user who already has the Stores menu.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 | (rows) | sm_id 148 granted to every user who already has the Item Masters menu.</t>
+        </is>
+      </c>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="4" t="n"/>
       <c r="F8" s="4" t="n"/>
@@ -1883,19 +1898,15 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>tbl_cash_details</t>
+          <t>tbl_item_stock</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Not deleted - old receipts hold cash_id 7 and history screens look the name up without checking status.</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Sales Receipt screen.</t>
-        </is>
-      </c>
+          <t>2026-09-22 | (no schema change) | Qty columns are now only written through fnApplyStockMovement(), never directly.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
@@ -1910,17 +1921,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>mst_cash_details</t>
+          <t>tbl_cash_details</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Same reasoning as tbl_cash_details.</t>
+          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Not deleted - old receipts hold cash_id 7 and history screens look the name up without checking status.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Invoice and Credit screens.</t>
+          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Sales Receipt screen.</t>
         </is>
       </c>
       <c r="D10" s="4" t="n"/>
@@ -1937,15 +1948,19 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>mst_customer_branch_temp</t>
+          <t>mst_cash_details</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. Branch rows live in the page and post back as arrays. Drop with db/drop_temp_tables.sql.</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n"/>
+          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Same reasoning as tbl_cash_details.</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Invoice and Credit screens.</t>
+        </is>
+      </c>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
@@ -1960,12 +1975,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>tbl_item_group_details_temp</t>
+          <t>mst_customer_branch_temp</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. Group items live in the page. Drop with db/drop_temp_tables.sql.</t>
+          <t>2026-10-01 | (whole table) | No longer used. Branch rows live in the page and post back as arrays. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C12" s="4" t="n"/>
@@ -1983,12 +1998,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>tbl_dc_details_temp</t>
+          <t>tbl_item_group_details_temp</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. DC item rows are built in php and posted back as arrays. Drop with db/drop_temp_tables.sql.</t>
+          <t>2026-10-01 | (whole table) | No longer used. Group items live in the page. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C13" s="4" t="n"/>
@@ -2006,12 +2021,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>tbl_package_box_details_temp</t>
+          <t>tbl_dc_details_temp</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. Packing rides on the DC item row as csv hidden fields. Drop with db/drop_temp_tables.sql.</t>
+          <t>2026-10-01 | (whole table) | No longer used. DC item rows are built in php and posted back as arrays. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C14" s="4" t="n"/>
@@ -2029,12 +2044,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>tbl_invoice_details</t>
+          <t>tbl_package_box_details_temp</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30 | inv_value | No schema change. Data repair - rows saved from the invoice edit screen had this zeroed by a bad field mapping. Rebuilt as net_value - tax_value where that agrees with qty x unit_price less discount.</t>
+          <t>2026-10-01 | (whole table) | No longer used. Packing rides on the DC item row as csv hidden fields. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C15" s="4" t="n"/>
@@ -2052,12 +2067,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>tbl_proforma_details</t>
+          <t>tbl_invoice_details</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30 | pro_value | No schema change. Same data repair as tbl_invoice_details.</t>
+          <t>2026-09-30 | inv_value | No schema change. Data repair - rows saved from the invoice edit screen had this zeroed by a bad field mapping. Rebuilt as net_value - tax_value where that agrees with qty x unit_price less discount.</t>
         </is>
       </c>
       <c r="C16" s="4" t="n"/>
@@ -2075,12 +2090,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>tbl_item_details</t>
+          <t>tbl_proforma_details</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | item_curr_stock | No change. Noted as dead - every write to it was already commented out. Branch columns in tbl_item_stock are the live balance.</t>
+          <t>2026-09-30 | pro_value | No schema change. Same data repair as tbl_invoice_details.</t>
         </is>
       </c>
       <c r="C17" s="4" t="n"/>
@@ -2095,6 +2110,29 @@
       <c r="L17" s="4" t="n"/>
       <c r="M17" s="4" t="n"/>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>tbl_item_details</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | item_curr_stock | No change. Noted as dead - every write to it was already commented out. Branch columns in tbl_item_stock are the live balance.</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n"/>
+      <c r="K18" s="4" t="n"/>
+      <c r="L18" s="4" t="n"/>
+      <c r="M18" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: details row counts no longer fatal on PHP 8
Every details save counted posted rows with count($_REQUEST['x']). When the
field arrived as a single value PHP 8 stops with a TypeError; PHP 7 counted
it as one row. fnRowCount('x') returns the row count, or 0 for a missing,
empty or single value; all 109 counts in 20 files use it.

In quotation.php and dc_invoice.php the package dropdown shared the name
pack_id with the package rows pack_id[]. A package picked but not added
replaced the rows: fatal on PHP 8, a junk package row on PHP 7. The
dropdown is now pack_pick; the scripts read it by id.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -471,6 +471,7 @@
     <col width="62" customWidth="1" min="3" max="3"/>
     <col width="62" customWidth="1" min="4" max="4"/>
     <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -499,6 +500,11 @@
           <t>Change 4</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Change 5</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -514,6 +520,7 @@
       <c r="C2" s="4" t="n"/>
       <c r="D2" s="4" t="n"/>
       <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -533,6 +540,7 @@
       </c>
       <c r="D3" s="4" t="n"/>
       <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -548,6 +556,7 @@
       <c r="C4" s="4" t="n"/>
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -567,6 +576,7 @@
       </c>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -589,7 +599,12 @@
           <t>2026-10-06 | New GRN from PO: commit moved above header(); die; - every new GRN was being rolled back while the screen said recorded.</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -617,6 +632,11 @@
           <t>2026-09-30 | Edit view posted quo_value, a column tbl_invoice_details does not have, wiping inv_value to 0. Now posts inv_value.</t>
         </is>
       </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -644,6 +664,11 @@
           <t>2026-09-30 | Edit view posted quo_value, a column tbl_invoice_details does not have, wiping inv_value to 0. Now posts inv_value.</t>
         </is>
       </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -671,6 +696,11 @@
           <t>2026-09-30 | Edit view posted quo_value, a column tbl_invoice_details does not have, wiping inv_value to 0. Now posts inv_value. Percentage charge base read from the raw hidden total instead of the comma-formatted text.</t>
         </is>
       </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8. Package dropdown renamed pack_pick so it cannot replace the pack_id[] rows.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -698,6 +728,11 @@
           <t>2026-10-06 | Multi UOM insert binds 0 for min / max discount when the row has no such field - it bound null and always failed on the NOT NULL column.</t>
         </is>
       </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -717,6 +752,7 @@
       </c>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -732,6 +768,7 @@
       <c r="C12" s="4" t="n"/>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -747,6 +784,7 @@
       <c r="C13" s="4" t="n"/>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -766,6 +804,7 @@
       </c>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -781,6 +820,7 @@
       <c r="C15" s="4" t="n"/>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -796,6 +836,7 @@
       <c r="C16" s="4" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -819,6 +860,7 @@
         </is>
       </c>
       <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -834,6 +876,7 @@
       <c r="C18" s="4" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -849,6 +892,7 @@
       <c r="C19" s="4" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -864,6 +908,7 @@
       <c r="C20" s="4" t="n"/>
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -879,6 +924,7 @@
       <c r="C21" s="4" t="n"/>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -894,6 +940,7 @@
       <c r="C22" s="4" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -913,6 +960,7 @@
       </c>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -932,6 +980,7 @@
       </c>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -944,9 +993,14 @@
           <t>2026-09-24 | CSRF + form token guard on SAVE/UPDATE/ACCOUNTS; try/catch added (handlers had none); transaction with rollback.</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -959,9 +1013,14 @@
           <t>2026-09-24 | CSRF + form token guard on SAVE/UPDATE/FINALIZE; transaction with rollback.</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n"/>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8. Package dropdown renamed pack_pick so it cannot replace the pack_id[] rows.</t>
+        </is>
+      </c>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -979,8 +1038,13 @@
           <t>2026-09-30 | Edit view posted quo_value, a column tbl_proforma_details does not have, wiping pro_value to 0. Now posts pro_value.</t>
         </is>
       </c>
-      <c r="D27" s="4" t="n"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1003,7 +1067,12 @@
           <t>2026-10-06 | Packing keeps its own box type and dispatch qty (hidden pack_box_id / pack_dispatch_qty) and box counts read them, so editing a completed DC no longer zeroes packing.</t>
         </is>
       </c>
-      <c r="E28" s="4" t="n"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1023,6 +1092,7 @@
       </c>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1035,9 +1105,14 @@
           <t>2026-09-24 | CSRF + form token guard on Draft/UPDATE/FINALIZE; transaction with rollback. Commit moved before the redirect that ends the success path.</t>
         </is>
       </c>
-      <c r="C30" s="4" t="n"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1050,9 +1125,14 @@
           <t>2026-09-24 | CSRF + form token guard on SAVE/UPDATE/FINALIZE; transaction with rollback. Commit moved before the redirect that ends the success path.</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1065,9 +1145,14 @@
           <t>2026-09-24 | CSRF + form token guard on SAVE/UPDATE; transaction with rollback.</t>
         </is>
       </c>
-      <c r="C32" s="4" t="n"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1080,9 +1165,14 @@
           <t>2026-09-24 | CSRF + form token guard on SAVE/UPDATE/FINALIZE; transaction with rollback.</t>
         </is>
       </c>
-      <c r="C33" s="4" t="n"/>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="4" t="n"/>
+      <c r="F33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1098,6 +1188,7 @@
       <c r="C34" s="4" t="n"/>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1113,6 +1204,7 @@
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="4" t="n"/>
+      <c r="F35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1125,9 +1217,14 @@
           <t>2026-09-25 | Cash denomination dropdown ordered by value instead of cash_id, so 1/2/5 sit at the top.</t>
         </is>
       </c>
-      <c r="C36" s="4" t="n"/>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1140,9 +1237,14 @@
           <t>2026-09-25 | Cash denomination dropdown ordered by value instead of cash_id.</t>
         </is>
       </c>
-      <c r="C37" s="4" t="n"/>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1158,6 +1260,7 @@
       <c r="C38" s="4" t="n"/>
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="4" t="n"/>
+      <c r="F38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1185,6 +1288,7 @@
           <t>2026-10-06 | Lock rewritten again: no longer wraps form.submit() or cancels a submission, only disables buttons once a submit is under way and drops later clicks. Buttons with their own onclick (Send to Purchase, invoice, direct PO, GRN, credit, Generate PO) were posting without their name.</t>
         </is>
       </c>
+      <c r="F39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1200,6 +1304,7 @@
       <c r="C40" s="4" t="n"/>
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="4" t="n"/>
+      <c r="F40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1215,6 +1320,7 @@
       <c r="C41" s="4" t="n"/>
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1230,6 +1336,7 @@
       <c r="C42" s="4" t="n"/>
       <c r="D42" s="4" t="n"/>
       <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1242,9 +1349,14 @@
           <t>2026-10-01 | Branch rows moved off mst_customer_branch_temp. Existing branches render from mst_customer_branch; save loops the posted br_* arrays; add/edit/remove are DOM only.</t>
         </is>
       </c>
-      <c r="C43" s="4" t="n"/>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="4" t="n"/>
+      <c r="F43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1260,6 +1372,7 @@
       <c r="C44" s="4" t="n"/>
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="4" t="n"/>
+      <c r="F44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1272,9 +1385,14 @@
           <t>2026-10-01 | Group items moved off tbl_item_group_details_temp. Added the trade_items field that fnValidate() read but never existed. Read-only users now post qty and position as hidden fields.</t>
         </is>
       </c>
-      <c r="C45" s="4" t="n"/>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D45" s="4" t="n"/>
       <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1290,6 +1408,7 @@
       <c r="C46" s="4" t="n"/>
       <c r="D46" s="4" t="n"/>
       <c r="E46" s="4" t="n"/>
+      <c r="F46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1305,6 +1424,7 @@
       <c r="C47" s="4" t="n"/>
       <c r="D47" s="4" t="n"/>
       <c r="E47" s="4" t="n"/>
+      <c r="F47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1320,6 +1440,7 @@
       <c r="C48" s="4" t="n"/>
       <c r="D48" s="4" t="n"/>
       <c r="E48" s="4" t="n"/>
+      <c r="F48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1332,9 +1453,14 @@
           <t>2026-10-01 | csrf + rollback. Done by hand: a brace at column zero hid the UPDATE handler's end, and the SAVE handler redirects three ways by employee type so the commit had to go above the whole chain.</t>
         </is>
       </c>
-      <c r="C49" s="4" t="n"/>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D49" s="4" t="n"/>
       <c r="E49" s="4" t="n"/>
+      <c r="F49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1350,6 +1476,7 @@
       <c r="C50" s="4" t="n"/>
       <c r="D50" s="4" t="n"/>
       <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1369,6 +1496,7 @@
       </c>
       <c r="D51" s="4" t="n"/>
       <c r="E51" s="4" t="n"/>
+      <c r="F51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1384,6 +1512,7 @@
       <c r="C52" s="4" t="n"/>
       <c r="D52" s="4" t="n"/>
       <c r="E52" s="4" t="n"/>
+      <c r="F52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1396,9 +1525,14 @@
           <t>2026-10-06 | Paid total read on $conn - a GRN paid in full was marked partly paid.</t>
         </is>
       </c>
-      <c r="C53" s="4" t="n"/>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
+        </is>
+      </c>
       <c r="D53" s="4" t="n"/>
       <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1414,6 +1548,7 @@
       <c r="C54" s="4" t="n"/>
       <c r="D54" s="4" t="n"/>
       <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1429,6 +1564,7 @@
       <c r="C55" s="4" t="n"/>
       <c r="D55" s="4" t="n"/>
       <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1444,6 +1580,7 @@
       <c r="C56" s="4" t="n"/>
       <c r="D56" s="4" t="n"/>
       <c r="E56" s="4" t="n"/>
+      <c r="F56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1459,6 +1596,7 @@
       <c r="C57" s="4" t="n"/>
       <c r="D57" s="4" t="n"/>
       <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1474,85 +1612,123 @@
       <c r="C58" s="4" t="n"/>
       <c r="D58" s="4" t="n"/>
       <c r="E58" s="4" t="n"/>
+      <c r="F58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>db/post_upload_061026.sql</t>
+          <t>spare_mapping.php</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>2026-10-06 | New. Checked against bie_db_061026.sql: every earlier change is live; adds the four audit columns mst_principal.php writes but the table never had.</t>
+          <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
       <c r="C59" s="4" t="n"/>
       <c r="D59" s="4" t="n"/>
       <c r="E59" s="4" t="n"/>
+      <c r="F59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>db/post_upload_051026.sql</t>
+          <t>inc/common/functions.php</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
-        </is>
-      </c>
+          <t>2026-10-07 | fnRowCount() added - posted row count, 0 for a missing or single value.</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="n"/>
       <c r="D60" s="4" t="n"/>
       <c r="E60" s="4" t="n"/>
+      <c r="F60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>index.php</t>
+          <t>db/post_upload_061026.sql</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
+          <t>2026-10-06 | New. Checked against bie_db_061026.sql: every earlier change is live; adds the four audit columns mst_principal.php writes but the table never had.</t>
         </is>
       </c>
       <c r="C61" s="4" t="n"/>
       <c r="D61" s="4" t="n"/>
       <c r="E61" s="4" t="n"/>
+      <c r="F61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>admin_multi_logins.php</t>
+          <t>db/post_upload_051026.sql</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="n"/>
+          <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
+        </is>
+      </c>
       <c r="D62" s="4" t="n"/>
       <c r="E62" s="4" t="n"/>
+      <c r="F62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>db/bie.sql</t>
+          <t>index.php</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
         </is>
       </c>
       <c r="C63" s="4" t="n"/>
       <c r="D63" s="4" t="n"/>
       <c r="E63" s="4" t="n"/>
+      <c r="F63" s="4" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>admin_multi_logins.php</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="n"/>
+      <c r="D64" s="4" t="n"/>
+      <c r="E64" s="4" t="n"/>
+      <c r="F64" s="4" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>db/bie.sql</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="n"/>
+      <c r="D65" s="4" t="n"/>
+      <c r="E65" s="4" t="n"/>
+      <c r="F65" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
perf: item search boxes answer in milliseconds
One letter in the Quotation item box took 8.6 s: every match came back
(2,865 items), each with five more queries, and the session stayed open so
each keystroke's search queued behind the last. Typing "cp-7" showed the
list after 8.3 s although "cp-7" alone took 19 ms.

item_search_lib.php returns the best 30 matches in one query, code prefix
first, and the stock fields for those items in one more, first stock row
per item as before. The session is released as soon as the branch is
read and the typed text is bound. Quotation and Store Indent use it;
Repair Indent and Spare Mapping release the session early.

Old against new for 15 terms on both pages, branch 1 and 2: every
suggestion identical field for field. One letter now 9 ms.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1649,12 +1649,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>db/post_upload_061026.sql</t>
+          <t>inc/auto/item_search_lib.php</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>2026-10-06 | New. Checked against bie_db_061026.sql: every earlier change is live; adds the four audit columns mst_principal.php writes but the table never had.</t>
+          <t>2026-10-07 | New. Shared item search: best 30 matches in one query, stock fields for those items in one more, branch column names checked against tbl_item_stock.</t>
         </is>
       </c>
       <c r="C61" s="4" t="n"/>
@@ -1665,19 +1665,15 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>db/post_upload_051026.sql</t>
+          <t>inc/auto/select_quotation_items.php</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
-        </is>
-      </c>
+          <t>2026-10-07 | Rewritten on item_search_lib - one letter went from 8.6 s and 2,865 items to 9 ms and the best 30; session released early, text bound.</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="n"/>
       <c r="D62" s="4" t="n"/>
       <c r="E62" s="4" t="n"/>
       <c r="F62" s="4" t="n"/>
@@ -1685,12 +1681,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>index.php</t>
+          <t>inc/auto/select_store_indent_items.php</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
+          <t>2026-10-07 | Rewritten on item_search_lib - one letter went from 5 s to 8 ms; session released early, text bound.</t>
         </is>
       </c>
       <c r="C63" s="4" t="n"/>
@@ -1701,12 +1697,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>admin_multi_logins.php</t>
+          <t>inc/auto/select_repair_indent_items.php</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
+          <t>2026-10-07 | Session released straight away so keystrokes are not queued.</t>
         </is>
       </c>
       <c r="C64" s="4" t="n"/>
@@ -1717,18 +1713,102 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>db/bie.sql</t>
+          <t>inc/cis_ajax/select_spare_mapping_items.php</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+          <t>2026-10-07 | Session released straight away; typed text bound.</t>
         </is>
       </c>
       <c r="C65" s="4" t="n"/>
       <c r="D65" s="4" t="n"/>
       <c r="E65" s="4" t="n"/>
       <c r="F65" s="4" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>db/post_upload_061026.sql</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-06 | New. Checked against bie_db_061026.sql: every earlier change is live; adds the four audit columns mst_principal.php writes but the table never had.</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="n"/>
+      <c r="D66" s="4" t="n"/>
+      <c r="E66" s="4" t="n"/>
+      <c r="F66" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>db/post_upload_051026.sql</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="n"/>
+      <c r="E67" s="4" t="n"/>
+      <c r="F67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>index.php</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="n"/>
+      <c r="D68" s="4" t="n"/>
+      <c r="E68" s="4" t="n"/>
+      <c r="F68" s="4" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>admin_multi_logins.php</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="n"/>
+      <c r="D69" s="4" t="n"/>
+      <c r="E69" s="4" t="n"/>
+      <c r="F69" s="4" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>db/bie.sql</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="n"/>
+      <c r="D70" s="4" t="n"/>
+      <c r="E70" s="4" t="n"/>
+      <c r="F70" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Item master: All branch option, principal code in dropdown, min/max discount on new item
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -750,7 +750,11 @@
           <t>2026-09-24 | CSRF + form token guard on SAVE/UPDATE; transaction with rollback.</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-12 | Branch dropdown gets All and is saved on a new item (All = every active branch, e.g. 1,2,3); it was ignored before and every item saved as branch 1. Principal shows Name - Code. Min / Max Discount on new item only, saved to each branch's min/max discount column in tbl_item_stock; min above max is refused.</t>
+        </is>
+      </c>
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
SPAC price list import script (4,702 items)
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1653,12 +1653,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>inc/auto/item_search_lib.php</t>
+          <t>db/import_spac_price_list_121026.sql</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>2026-10-07 | New. Shared item search: best 30 matches in one query, stock fields for those items in one more, branch column names checked against tbl_item_stock.</t>
+          <t>2026-10-12 | New. One-time import of the SPAC price list (4,702 items) - adds missing categories and HSN codes, items for all branches, stock rows with price, discount and min/max discount. Safe to run twice.</t>
         </is>
       </c>
       <c r="C61" s="4" t="n"/>
@@ -1669,12 +1669,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>inc/auto/select_quotation_items.php</t>
+          <t>inc/auto/item_search_lib.php</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>2026-10-07 | Rewritten on item_search_lib - one letter went from 8.6 s and 2,865 items to 9 ms and the best 30; session released early, text bound.</t>
+          <t>2026-10-07 | New. Shared item search: best 30 matches in one query, stock fields for those items in one more, branch column names checked against tbl_item_stock.</t>
         </is>
       </c>
       <c r="C62" s="4" t="n"/>
@@ -1685,12 +1685,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>inc/auto/select_store_indent_items.php</t>
+          <t>inc/auto/select_quotation_items.php</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>2026-10-07 | Rewritten on item_search_lib - one letter went from 5 s to 8 ms; session released early, text bound.</t>
+          <t>2026-10-07 | Rewritten on item_search_lib - one letter went from 8.6 s and 2,865 items to 9 ms and the best 30; session released early, text bound.</t>
         </is>
       </c>
       <c r="C63" s="4" t="n"/>
@@ -1701,12 +1701,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>inc/auto/select_repair_indent_items.php</t>
+          <t>inc/auto/select_store_indent_items.php</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>2026-10-07 | Session released straight away so keystrokes are not queued.</t>
+          <t>2026-10-07 | Rewritten on item_search_lib - one letter went from 5 s to 8 ms; session released early, text bound.</t>
         </is>
       </c>
       <c r="C64" s="4" t="n"/>
@@ -1717,12 +1717,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>inc/cis_ajax/select_spare_mapping_items.php</t>
+          <t>inc/auto/select_repair_indent_items.php</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>2026-10-07 | Session released straight away; typed text bound.</t>
+          <t>2026-10-07 | Session released straight away so keystrokes are not queued.</t>
         </is>
       </c>
       <c r="C65" s="4" t="n"/>
@@ -1733,12 +1733,12 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>db/post_upload_061026.sql</t>
+          <t>inc/cis_ajax/select_spare_mapping_items.php</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>2026-10-06 | New. Checked against bie_db_061026.sql: every earlier change is live; adds the four audit columns mst_principal.php writes but the table never had.</t>
+          <t>2026-10-07 | Session released straight away; typed text bound.</t>
         </is>
       </c>
       <c r="C66" s="4" t="n"/>
@@ -1749,19 +1749,15 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>db/post_upload_051026.sql</t>
+          <t>db/post_upload_061026.sql</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
-        </is>
-      </c>
+          <t>2026-10-06 | New. Checked against bie_db_061026.sql: every earlier change is live; adds the four audit columns mst_principal.php writes but the table never had.</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="n"/>
       <c r="D67" s="4" t="n"/>
       <c r="E67" s="4" t="n"/>
       <c r="F67" s="4" t="n"/>
@@ -1769,15 +1765,19 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>index.php</t>
+          <t>db/post_upload_051026.sql</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="n"/>
+          <t>2026-10-05 | New. Everything to run on the server after the file upload, checked against bie_db_051026.sql: widen tbl_user_rights.sm_id, clear the six clamped rights rows, grant sm_id 147/148, repair 111 zeroed invoice line amounts, drop the four temp tables.</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05 | Step 7 split into five queries - as one UNION starting from information_schema, MariaDB looked for the plain tables there too (#1109). Step 3 now skips rights rows that already exist and step 4b keeps an existing backup, so the whole file is safe to run twice.</t>
+        </is>
+      </c>
       <c r="D68" s="4" t="n"/>
       <c r="E68" s="4" t="n"/>
       <c r="F68" s="4" t="n"/>
@@ -1785,12 +1785,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>admin_multi_logins.php</t>
+          <t>index.php</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
+          <t>2026-10-01 | Login query was concatenated from $_REQUEST so the password check could be commented out - now a prepared statement with both values bound. csrf + form token on the post, session id regenerated and tokens dropped on success, failed logins written to the error log, prefilled admin@bie.com removed, autocomplete attributes added.</t>
         </is>
       </c>
       <c r="C69" s="4" t="n"/>
@@ -1801,18 +1801,34 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>db/bie.sql</t>
+          <t>admin_multi_logins.php</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+          <t>2026-10-01 | Same concatenated login query, bound now. Removed the echo that printed the query with the password in it to the page. csrf + form token, session id regenerated on success. Its no-hash password compare left as it was - that changes who can use the screen.</t>
         </is>
       </c>
       <c r="C70" s="4" t="n"/>
       <c r="D70" s="4" t="n"/>
       <c r="E70" s="4" t="n"/>
       <c r="F70" s="4" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>db/bie.sql</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | Base dump updated - 2000 inactive, 1/2/5 added to tbl_cash_details and mst_cash_details.</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="n"/>
+      <c r="D71" s="4" t="n"/>
+      <c r="E71" s="4" t="n"/>
+      <c r="F71" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1825,7 +1841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1913,12 +1929,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>mst_principal</t>
+          <t>mst_category</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-06 | created_by, created_dtm, modify_by, modify_dtm | Added - mst_principal.php writes them on save and update, so both always failed with Unknown column. Existing rows get 0 / NULL.</t>
+          <t>2026-10-12 | (rows) | SPAC import adds AIR GUN, FRL, TUBING. Sheet FITTING mapped to the existing FITTINGS.</t>
         </is>
       </c>
       <c r="C2" s="4" t="n"/>
@@ -1936,24 +1952,16 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>tbl_user_rights</t>
+          <t>mst_hsn</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | sm_id | Signed TINYINT widened to SMALLINT. It stopped at 127, so the rights rows for the new menus (147, 148) were silently clamped to 127 and the menus never showed.</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | mm_id | Signed TINYINT widened to SMALLINT, same reason - it was two main menus away from the same limit.</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | (rows) | Six clamped rows deleted (users 2/6/7, sm_id 127 under main menus 3 and 20); sm_id 147 and 148 granted to whoever holds the parent menu.</t>
-        </is>
-      </c>
+          <t>2026-10-12 | (rows) | SPAC import adds 39173290, 39174000, 40169390, 84678910, 84812000, 85045090, 85365090, 85444999 at 18% (9 + 9).</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
@@ -1967,19 +1975,15 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>tbl_invoice_details</t>
+          <t>tbl_item_details / tbl_item_stock</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | inv_value, tax_value | 111 rows across 35 invoices rebuilt as net_value / (1 + vat/100); tax_value rebuilt with them. Backup taken as tbl_invoice_details_bkp_051026.</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | cgst_per, sgst_per, igst_per, cgst_val, sgst_val, igst_val | Optional tidy on the same 111 rows only.</t>
-        </is>
-      </c>
+          <t>2026-10-12 | (rows) | SPAC import adds 4,702 items (principal SPAC, Pneumatic, Trading, branches 1,2,3) and one stock row each.</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n"/>
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="4" t="n"/>
@@ -1994,106 +1998,50 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>tbl_stock_flow</t>
+          <t>mst_principal</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | trans_dir | Added CHAR(1). I = stock in (+), O = stock out (-). Backfilled GRN=I, INV/SALE=O.</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | trans_remarks | Added VARCHAR(255). Reason / narration, mandatory on ADJ rows.</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | stock_field | Added VARCHAR(30). Which tbl_item_stock column was changed. Backfilled from mst_branch.</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | before_qty | INT to DECIMAL(12,3). Was truncating decimal stock.</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | trans_qty | INT to DECIMAL(12,3). Always a positive magnitude, direction is in trans_dir.</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | rcvd_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | after_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | reje_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | pend_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | trans_type | VARCHAR(8) to VARCHAR(10). Values GRN, INV, ADJ, OPEN, RET.</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | idx_sf_item_branch_date | Index added on (item_id, branch_id, trans_date) - what the reports filter on.</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | idx_sf_trans | Index added on (trans_type, trans_id).</t>
-        </is>
-      </c>
+          <t>2026-10-06 | created_by, created_dtm, modify_by, modify_dtm | Added - mst_principal.php writes them on save and update, so both always failed with Unknown column. Existing rows get 0 / NULL.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>tbl_stock_adjustment</t>
+          <t>tbl_user_rights</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (new table) | Header for every manual stock correction. One row per adjustment.</t>
+          <t>2026-10-05 | sm_id | Signed TINYINT widened to SMALLINT. It stopped at 127, so the rights rows for the new menus (147, 148) were silently clamped to 127 and the menus never showed.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | adj_id, adj_refno, adj_slno, adj_finyr | Key and reference number ADJ/nnnn/BIE/&lt;branch&gt;/&lt;finyr&gt;.</t>
+          <t>2026-10-05 | mm_id | Signed TINYINT widened to SMALLINT, same reason - it was two main menus away from the same limit.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | adj_date, branch_id, stock_field, item_id | What was adjusted, where, and which stock column.</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | adj_type, adj_qty, before_qty, after_qty | I = increase, D = decrease. adj_qty is always positive.</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | item_price, adj_reason, adj_status | Reason is mandatory. adj_status 1 = active, 0 = deleted.</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | created_by, created_dtm | Who made the adjustment and when.</t>
-        </is>
-      </c>
+          <t>2026-10-05 | (rows) | Six clamped rows deleted (users 2/6/7, sm_id 127 under main menus 3 and 20); sm_id 147 and 148 granted to whoever holds the parent menu.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
@@ -2104,17 +2052,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>mst_sub_menu</t>
+          <t>tbl_invoice_details</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (row) | sm_id 147, mm_id 20 (Stores) - Stock Adjustment, stock_adjustment.php.</t>
+          <t>2026-10-05 | inv_value, tax_value | 111 rows across 35 invoices rebuilt as net_value / (1 + vat/100); tax_value rebuilt with them. Backup taken as tbl_invoice_details_bkp_051026.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 | (row) | sm_id 148, mm_id 3 (Item Masters) - Item Stock List, lst_item_stock.php.</t>
+          <t>2026-10-05 | cgst_per, sgst_per, igst_per, cgst_val, sgst_val, igst_val | Optional tidy on the same 111 rows only.</t>
         </is>
       </c>
       <c r="D7" s="4" t="n"/>
@@ -2131,46 +2079,106 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>tbl_user_rights</t>
+          <t>tbl_stock_flow</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (rows) | sm_id 147 granted to every user who already has the Stores menu.</t>
+          <t>2026-09-22 | trans_dir | Added CHAR(1). I = stock in (+), O = stock out (-). Backfilled GRN=I, INV/SALE=O.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 | (rows) | sm_id 148 granted to every user who already has the Item Masters menu.</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
-      <c r="I8" s="4" t="n"/>
-      <c r="J8" s="4" t="n"/>
-      <c r="K8" s="4" t="n"/>
-      <c r="L8" s="4" t="n"/>
-      <c r="M8" s="4" t="n"/>
+          <t>2026-09-22 | trans_remarks | Added VARCHAR(255). Reason / narration, mandatory on ADJ rows.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | stock_field | Added VARCHAR(30). Which tbl_item_stock column was changed. Backfilled from mst_branch.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | before_qty | INT to DECIMAL(12,3). Was truncating decimal stock.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | trans_qty | INT to DECIMAL(12,3). Always a positive magnitude, direction is in trans_dir.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | rcvd_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | after_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | reje_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | pend_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | trans_type | VARCHAR(8) to VARCHAR(10). Values GRN, INV, ADJ, OPEN, RET.</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | idx_sf_item_branch_date | Index added on (item_id, branch_id, trans_date) - what the reports filter on.</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | idx_sf_trans | Index added on (trans_type, trans_id).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>tbl_item_stock</t>
+          <t>tbl_stock_adjustment</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (no schema change) | Qty columns are now only written through fnApplyStockMovement(), never directly.</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
+          <t>2026-09-22 | (new table) | Header for every manual stock correction. One row per adjustment.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | adj_id, adj_refno, adj_slno, adj_finyr | Key and reference number ADJ/nnnn/BIE/&lt;branch&gt;/&lt;finyr&gt;.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | adj_date, branch_id, stock_field, item_id | What was adjusted, where, and which stock column.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | adj_type, adj_qty, before_qty, after_qty | I = increase, D = decrease. adj_qty is always positive.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | item_price, adj_reason, adj_status | Reason is mandatory. adj_status 1 = active, 0 = deleted.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | created_by, created_dtm | Who made the adjustment and when.</t>
+        </is>
+      </c>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="4" t="n"/>
       <c r="J9" s="4" t="n"/>
@@ -2181,17 +2189,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>tbl_cash_details</t>
+          <t>mst_sub_menu</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Not deleted - old receipts hold cash_id 7 and history screens look the name up without checking status.</t>
+          <t>2026-09-22 | (row) | sm_id 147, mm_id 20 (Stores) - Stock Adjustment, stock_adjustment.php.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Sales Receipt screen.</t>
+          <t>2026-09-23 | (row) | sm_id 148, mm_id 3 (Item Masters) - Item Stock List, lst_item_stock.php.</t>
         </is>
       </c>
       <c r="D10" s="4" t="n"/>
@@ -2208,17 +2216,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>mst_cash_details</t>
+          <t>tbl_user_rights</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Same reasoning as tbl_cash_details.</t>
+          <t>2026-09-22 | (rows) | sm_id 147 granted to every user who already has the Stores menu.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Invoice and Credit screens.</t>
+          <t>2026-09-23 | (rows) | sm_id 148 granted to every user who already has the Item Masters menu.</t>
         </is>
       </c>
       <c r="D11" s="4" t="n"/>
@@ -2235,12 +2243,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>mst_customer_branch_temp</t>
+          <t>tbl_item_stock</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. Branch rows live in the page and post back as arrays. Drop with db/drop_temp_tables.sql.</t>
+          <t>2026-09-22 | (no schema change) | Qty columns are now only written through fnApplyStockMovement(), never directly.</t>
         </is>
       </c>
       <c r="C12" s="4" t="n"/>
@@ -2258,15 +2266,19 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>tbl_item_group_details_temp</t>
+          <t>tbl_cash_details</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. Group items live in the page. Drop with db/drop_temp_tables.sql.</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="n"/>
+          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Not deleted - old receipts hold cash_id 7 and history screens look the name up without checking status.</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Sales Receipt screen.</t>
+        </is>
+      </c>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
@@ -2281,15 +2293,19 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>tbl_dc_details_temp</t>
+          <t>mst_cash_details</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. DC item rows are built in php and posted back as arrays. Drop with db/drop_temp_tables.sql.</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="n"/>
+          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Same reasoning as tbl_cash_details.</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Invoice and Credit screens.</t>
+        </is>
+      </c>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
@@ -2304,12 +2320,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>tbl_package_box_details_temp</t>
+          <t>mst_customer_branch_temp</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. Packing rides on the DC item row as csv hidden fields. Drop with db/drop_temp_tables.sql.</t>
+          <t>2026-10-01 | (whole table) | No longer used. Branch rows live in the page and post back as arrays. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C15" s="4" t="n"/>
@@ -2327,12 +2343,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>tbl_invoice_details</t>
+          <t>tbl_item_group_details_temp</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30 | inv_value | No schema change. Data repair - rows saved from the invoice edit screen had this zeroed by a bad field mapping. Rebuilt as net_value - tax_value where that agrees with qty x unit_price less discount.</t>
+          <t>2026-10-01 | (whole table) | No longer used. Group items live in the page. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C16" s="4" t="n"/>
@@ -2350,12 +2366,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>tbl_proforma_details</t>
+          <t>tbl_dc_details_temp</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30 | pro_value | No schema change. Same data repair as tbl_invoice_details.</t>
+          <t>2026-10-01 | (whole table) | No longer used. DC item rows are built in php and posted back as arrays. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C17" s="4" t="n"/>
@@ -2373,12 +2389,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>tbl_item_details</t>
+          <t>tbl_package_box_details_temp</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | item_curr_stock | No change. Noted as dead - every write to it was already commented out. Branch columns in tbl_item_stock are the live balance.</t>
+          <t>2026-10-01 | (whole table) | No longer used. Packing rides on the DC item row as csv hidden fields. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C18" s="4" t="n"/>
@@ -2393,6 +2409,75 @@
       <c r="L18" s="4" t="n"/>
       <c r="M18" s="4" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>tbl_invoice_details</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30 | inv_value | No schema change. Data repair - rows saved from the invoice edit screen had this zeroed by a bad field mapping. Rebuilt as net_value - tax_value where that agrees with qty x unit_price less discount.</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="n"/>
+      <c r="K19" s="4" t="n"/>
+      <c r="L19" s="4" t="n"/>
+      <c r="M19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>tbl_proforma_details</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30 | pro_value | No schema change. Same data repair as tbl_invoice_details.</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
+      <c r="M20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>tbl_item_details</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | item_curr_stock | No change. Noted as dead - every write to it was already commented out. Branch columns in tbl_item_stock are the live balance.</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="n"/>
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="n"/>
+      <c r="M21" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Approve/verify/reject checked on the server; modal session, ajax csrf prefilter and _userid fixes
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -472,6 +472,7 @@
     <col width="62" customWidth="1" min="4" max="4"/>
     <col width="62" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -505,6 +506,11 @@
           <t>Change 5</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Change 6</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -521,6 +527,7 @@
       <c r="D2" s="4" t="n"/>
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -541,6 +548,7 @@
       <c r="D3" s="4" t="n"/>
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -557,6 +565,7 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -577,6 +586,7 @@
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -605,6 +615,7 @@
         </is>
       </c>
       <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -637,6 +648,7 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
+      <c r="G7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -669,6 +681,7 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
+      <c r="G8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -701,6 +714,7 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8. Package dropdown renamed pack_pick so it cannot replace the pack_id[] rows.</t>
         </is>
       </c>
+      <c r="G9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -733,6 +747,11 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | updated_by from _user_id (was empty).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -755,8 +774,13 @@
           <t>2026-10-12 | Branch dropdown gets All and is saved on a new item (All = every active branch, e.g. 1,2,3); it was ignored before and every item saved as branch 1. Principal shows Name - Code. Min / Max Discount on new item only, saved to each branch's min/max discount column in tbl_item_stock; min above max is refused.</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | _userid replaced by _user_id - the admin price-required check never ran.</t>
+        </is>
+      </c>
       <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -773,6 +797,7 @@
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -789,6 +814,7 @@
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -809,6 +835,7 @@
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -825,6 +852,7 @@
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
+      <c r="G15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -841,6 +869,7 @@
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -865,6 +894,7 @@
       </c>
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
+      <c r="G17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -881,6 +911,7 @@
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -897,6 +928,7 @@
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -913,6 +945,7 @@
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -929,6 +962,7 @@
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -945,6 +979,7 @@
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -965,6 +1000,7 @@
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
+      <c r="G23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -982,9 +1018,14 @@
           <t>2026-09-24 | Loads csrf.php and db_txn.php.</t>
         </is>
       </c>
-      <c r="D24" s="4" t="n"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Loads access.php.</t>
+        </is>
+      </c>
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1005,6 +1046,7 @@
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1025,6 +1067,7 @@
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1049,6 +1092,7 @@
       </c>
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1076,7 +1120,12 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
-      <c r="F28" s="4" t="n"/>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | dc_verify_by from _user_id - _userid is never set at login, so it was always empty.</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1094,9 +1143,14 @@
           <t>2026-10-06 | Prepared qty read on $conn - a complete PO went to admin as partial.</t>
         </is>
       </c>
-      <c r="D29" s="4" t="n"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | modify_by from _user_id (was empty).</t>
+        </is>
+      </c>
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1117,6 +1171,7 @@
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1137,6 +1192,7 @@
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1157,6 +1213,7 @@
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1177,6 +1234,7 @@
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
+      <c r="G33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1193,6 +1251,7 @@
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1209,6 +1268,7 @@
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
+      <c r="G35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1229,6 +1289,7 @@
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1249,6 +1310,7 @@
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1265,6 +1327,7 @@
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="n"/>
+      <c r="G38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1292,7 +1355,12 @@
           <t>2026-10-06 | Lock rewritten again: no longer wraps form.submit() or cancels a submission, only disables buttons once a submit is under way and drops later clicks. Buttons with their own onclick (Send to Purchase, invoice, direct PO, GRN, credit, Generate PO) were posting without their name.</t>
         </is>
       </c>
-      <c r="F39" s="4" t="n"/>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Csrf token attached in $.ajaxPrefilter - pages passing their own beforeSend dropped the ajaxSetup hook, so their posts had no token.</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1309,6 +1377,7 @@
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1325,6 +1394,7 @@
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="4" t="n"/>
+      <c r="G41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1341,6 +1411,7 @@
       <c r="D42" s="4" t="n"/>
       <c r="E42" s="4" t="n"/>
       <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1361,6 +1432,7 @@
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="4" t="n"/>
       <c r="F43" s="4" t="n"/>
+      <c r="G43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1377,6 +1449,7 @@
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="4" t="n"/>
       <c r="F44" s="4" t="n"/>
+      <c r="G44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1397,6 +1470,7 @@
       <c r="D45" s="4" t="n"/>
       <c r="E45" s="4" t="n"/>
       <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1413,6 +1487,7 @@
       <c r="D46" s="4" t="n"/>
       <c r="E46" s="4" t="n"/>
       <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1429,6 +1504,7 @@
       <c r="D47" s="4" t="n"/>
       <c r="E47" s="4" t="n"/>
       <c r="F47" s="4" t="n"/>
+      <c r="G47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1445,6 +1521,7 @@
       <c r="D48" s="4" t="n"/>
       <c r="E48" s="4" t="n"/>
       <c r="F48" s="4" t="n"/>
+      <c r="G48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1465,6 +1542,7 @@
       <c r="D49" s="4" t="n"/>
       <c r="E49" s="4" t="n"/>
       <c r="F49" s="4" t="n"/>
+      <c r="G49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1481,6 +1559,7 @@
       <c r="D50" s="4" t="n"/>
       <c r="E50" s="4" t="n"/>
       <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1501,6 +1580,7 @@
       <c r="D51" s="4" t="n"/>
       <c r="E51" s="4" t="n"/>
       <c r="F51" s="4" t="n"/>
+      <c r="G51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1517,6 +1597,7 @@
       <c r="D52" s="4" t="n"/>
       <c r="E52" s="4" t="n"/>
       <c r="F52" s="4" t="n"/>
+      <c r="G52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1534,9 +1615,14 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
-      <c r="D53" s="4" t="n"/>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | _userid replaced by _user_id - the admin Edit amount button never showed for anyone.</t>
+        </is>
+      </c>
       <c r="E53" s="4" t="n"/>
       <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1553,6 +1639,7 @@
       <c r="D54" s="4" t="n"/>
       <c r="E54" s="4" t="n"/>
       <c r="F54" s="4" t="n"/>
+      <c r="G54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1569,6 +1656,7 @@
       <c r="D55" s="4" t="n"/>
       <c r="E55" s="4" t="n"/>
       <c r="F55" s="4" t="n"/>
+      <c r="G55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1581,10 +1669,15 @@
           <t>2026-10-06 | Loads csrf and txn helpers itself - opened on its own it died on csrf_fields().</t>
         </is>
       </c>
-      <c r="C56" s="4" t="n"/>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Starts its own session when posted directly - credit approval failed since 2026-10-01. Allowed for the credit-approval tile users; approver saved as the user, was always 1.</t>
+        </is>
+      </c>
       <c r="D56" s="4" t="n"/>
       <c r="E56" s="4" t="n"/>
       <c r="F56" s="4" t="n"/>
+      <c r="G56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1597,10 +1690,15 @@
           <t>2026-10-06 | Loads csrf and txn helpers itself - opened on its own it died on csrf_fields().</t>
         </is>
       </c>
-      <c r="C57" s="4" t="n"/>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Starts its own session when posted directly - every cancel failed the csrf check since 2026-10-01. Cancel allowed for admin only (the link); cancelled-by is the user, was always 1.</t>
+        </is>
+      </c>
       <c r="D57" s="4" t="n"/>
       <c r="E57" s="4" t="n"/>
       <c r="F57" s="4" t="n"/>
+      <c r="G57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1613,10 +1711,15 @@
           <t>2026-10-06 | Loads csrf and txn helpers itself - opened on its own it died on csrf_fields().</t>
         </is>
       </c>
-      <c r="C58" s="4" t="n"/>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Starts its own session when posted directly - every cancel failed since 2026-10-01. Allowed for admin or head office (the link); cancelled-by is the user, was always 1.</t>
+        </is>
+      </c>
       <c r="D58" s="4" t="n"/>
       <c r="E58" s="4" t="n"/>
       <c r="F58" s="4" t="n"/>
+      <c r="G58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1633,6 +1736,7 @@
       <c r="D59" s="4" t="n"/>
       <c r="E59" s="4" t="n"/>
       <c r="F59" s="4" t="n"/>
+      <c r="G59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1649,6 +1753,7 @@
       <c r="D60" s="4" t="n"/>
       <c r="E60" s="4" t="n"/>
       <c r="F60" s="4" t="n"/>
+      <c r="G60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1665,6 +1770,7 @@
       <c r="D61" s="4" t="n"/>
       <c r="E61" s="4" t="n"/>
       <c r="F61" s="4" t="n"/>
+      <c r="G61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1681,6 +1787,7 @@
       <c r="D62" s="4" t="n"/>
       <c r="E62" s="4" t="n"/>
       <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1697,6 +1804,7 @@
       <c r="D63" s="4" t="n"/>
       <c r="E63" s="4" t="n"/>
       <c r="F63" s="4" t="n"/>
+      <c r="G63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1713,6 +1821,7 @@
       <c r="D64" s="4" t="n"/>
       <c r="E64" s="4" t="n"/>
       <c r="F64" s="4" t="n"/>
+      <c r="G64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1729,6 +1838,7 @@
       <c r="D65" s="4" t="n"/>
       <c r="E65" s="4" t="n"/>
       <c r="F65" s="4" t="n"/>
+      <c r="G65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1745,6 +1855,7 @@
       <c r="D66" s="4" t="n"/>
       <c r="E66" s="4" t="n"/>
       <c r="F66" s="4" t="n"/>
+      <c r="G66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1761,6 +1872,7 @@
       <c r="D67" s="4" t="n"/>
       <c r="E67" s="4" t="n"/>
       <c r="F67" s="4" t="n"/>
+      <c r="G67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1781,6 +1893,7 @@
       <c r="D68" s="4" t="n"/>
       <c r="E68" s="4" t="n"/>
       <c r="F68" s="4" t="n"/>
+      <c r="G68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1797,6 +1910,7 @@
       <c r="D69" s="4" t="n"/>
       <c r="E69" s="4" t="n"/>
       <c r="F69" s="4" t="n"/>
+      <c r="G69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -1813,6 +1927,7 @@
       <c r="D70" s="4" t="n"/>
       <c r="E70" s="4" t="n"/>
       <c r="F70" s="4" t="n"/>
+      <c r="G70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -1829,6 +1944,211 @@
       <c r="D71" s="4" t="n"/>
       <c r="E71" s="4" t="n"/>
       <c r="F71" s="4" t="n"/>
+      <c r="G71" s="4" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>inc/common/access.php</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | New. fnAccessDenied, fnAjaxGuard (login + csrf), fnUserHasMenu, fnTaskUserListed - server-side checks for approve / verify / reject.</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="n"/>
+      <c r="D72" s="4" t="n"/>
+      <c r="E72" s="4" t="n"/>
+      <c r="F72" s="4" t="n"/>
+      <c r="G72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_po_approval.php</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Login + csrf + approver check (admin, as the button); remarks and id bound instead of pasted into the sql.</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="n"/>
+      <c r="D73" s="4" t="n"/>
+      <c r="E73" s="4" t="n"/>
+      <c r="F73" s="4" t="n"/>
+      <c r="G73" s="4" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_purchase_return_approval.php</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Login + csrf + approver check (admin - the list is an admin-only menu); remarks and id bound.</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="n"/>
+      <c r="D74" s="4" t="n"/>
+      <c r="E74" s="4" t="n"/>
+      <c r="F74" s="4" t="n"/>
+      <c r="G74" s="4" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_quo_approval.php</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Login + csrf + approver check: admin or the quotation's branch, as the button.</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="n"/>
+      <c r="D75" s="4" t="n"/>
+      <c r="E75" s="4" t="n"/>
+      <c r="F75" s="4" t="n"/>
+      <c r="G75" s="4" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_so_approval.php</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Login + csrf + approver check (admin, as the button).</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="n"/>
+      <c r="D76" s="4" t="n"/>
+      <c r="E76" s="4" t="n"/>
+      <c r="F76" s="4" t="n"/>
+      <c r="G76" s="4" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_dc_approval.php</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Login + csrf + approver check: admin or the DC's branch, as the button.</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="n"/>
+      <c r="D77" s="4" t="n"/>
+      <c r="E77" s="4" t="n"/>
+      <c r="F77" s="4" t="n"/>
+      <c r="G77" s="4" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_sales_repair_status.php</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Login + csrf + check (admin, as the buttons).</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="n"/>
+      <c r="D78" s="4" t="n"/>
+      <c r="E78" s="4" t="n"/>
+      <c r="F78" s="4" t="n"/>
+      <c r="G78" s="4" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_so_pay_status.php</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Login + csrf + check: holders of the Sales Order in Accounts menu. Verifier saved from _user_id - it was always empty.</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="n"/>
+      <c r="D79" s="4" t="n"/>
+      <c r="E79" s="4" t="n"/>
+      <c r="F79" s="4" t="n"/>
+      <c r="G79" s="4" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>so_verify.php</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Csrf + check: holders of the Sales Order in Accounts menu; so_id bound.</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="n"/>
+      <c r="D80" s="4" t="n"/>
+      <c r="E80" s="4" t="n"/>
+      <c r="F80" s="4" t="n"/>
+      <c r="G80" s="4" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>mst_supplier_approve.php</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Csrf token on the form + approver check (admin, the only user shown the link).</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="n"/>
+      <c r="D81" s="4" t="n"/>
+      <c r="E81" s="4" t="n"/>
+      <c r="F81" s="4" t="n"/>
+      <c r="G81" s="4" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>branch_wise_item_update.php</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Update allowed for admin at head office or the item-approval users; updated_by from _user_id (was empty).</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="n"/>
+      <c r="D82" s="4" t="n"/>
+      <c r="E82" s="4" t="n"/>
+      <c r="F82" s="4" t="n"/>
+      <c r="G82" s="4" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>po_prepare_print.php</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | modify_by from _user_id (was empty).</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="n"/>
+      <c r="D83" s="4" t="n"/>
+      <c r="E83" s="4" t="n"/>
+      <c r="F83" s="4" t="n"/>
+      <c r="G83" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Task Settings: creator / verifier / approver / viewer rules moved from code into mst_task and tbl_task_assign
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,11 @@
           <t>2026-10-13 | _userid replaced by _user_id - the admin price-required check never ran.</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Price block check uses Task Settings (ITEM C) - was user 1; both branches show it.</t>
+        </is>
+      </c>
       <c r="G11" s="4" t="n"/>
     </row>
     <row r="12">
@@ -1064,7 +1068,11 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8. Package dropdown renamed pack_pick so it cannot replace the pack_id[] rows.</t>
         </is>
       </c>
-      <c r="D26" s="4" t="n"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Named approver from Task Settings (QUOTATION A, else admin) - was tbl_task_user 1.</t>
+        </is>
+      </c>
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
@@ -1168,7 +1176,11 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
-      <c r="D30" s="4" t="n"/>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Named approver from Task Settings (PURCHASE_ORDER A, else admin) - was tbl_task_user 1.</t>
+        </is>
+      </c>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="n"/>
@@ -1189,7 +1201,11 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
-      <c r="D31" s="4" t="n"/>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Named approver from Task Settings (STORE_INDENT A, else admin) - was tbl_task_user 1.</t>
+        </is>
+      </c>
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
       <c r="G31" s="4" t="n"/>
@@ -1620,7 +1636,11 @@
           <t>2026-10-13 | _userid replaced by _user_id - the admin Edit amount button never showed for anyone.</t>
         </is>
       </c>
-      <c r="E53" s="4" t="n"/>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Edit paid amount for approvers in Task Settings (GRN_PAYMENT A) - was admin.</t>
+        </is>
+      </c>
       <c r="F53" s="4" t="n"/>
       <c r="G53" s="4" t="n"/>
     </row>
@@ -1674,7 +1694,11 @@
           <t>2026-10-13 | Starts its own session when posted directly - credit approval failed since 2026-10-01. Allowed for the credit-approval tile users; approver saved as the user, was always 1.</t>
         </is>
       </c>
-      <c r="D56" s="4" t="n"/>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Credit approval for approvers in Task Settings (CREDIT_SALES A).</t>
+        </is>
+      </c>
       <c r="E56" s="4" t="n"/>
       <c r="F56" s="4" t="n"/>
       <c r="G56" s="4" t="n"/>
@@ -1695,7 +1719,11 @@
           <t>2026-10-13 | Starts its own session when posted directly - every cancel failed the csrf check since 2026-10-01. Cancel allowed for admin only (the link); cancelled-by is the user, was always 1.</t>
         </is>
       </c>
-      <c r="D57" s="4" t="n"/>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Cancel for approvers in Task Settings (SALES_ORDER A).</t>
+        </is>
+      </c>
       <c r="E57" s="4" t="n"/>
       <c r="F57" s="4" t="n"/>
       <c r="G57" s="4" t="n"/>
@@ -1716,7 +1744,11 @@
           <t>2026-10-13 | Starts its own session when posted directly - every cancel failed since 2026-10-01. Allowed for admin or head office (the link); cancelled-by is the user, was always 1.</t>
         </is>
       </c>
-      <c r="D58" s="4" t="n"/>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Cancel for approvers in Task Settings (GRN A).</t>
+        </is>
+      </c>
       <c r="E58" s="4" t="n"/>
       <c r="F58" s="4" t="n"/>
       <c r="G58" s="4" t="n"/>
@@ -1957,7 +1989,11 @@
           <t>2026-10-13 | New. fnAccessDenied, fnAjaxGuard (login + csrf), fnUserHasMenu, fnTaskUserListed - server-side checks for approve / verify / reject.</t>
         </is>
       </c>
-      <c r="C72" s="4" t="n"/>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | fnTaskCan(code, role, branch), fnTaskIsAdmin, fnTaskDefaultUser; rows read once per request. fnUserHasMenu / fnTaskUserListed removed.</t>
+        </is>
+      </c>
       <c r="D72" s="4" t="n"/>
       <c r="E72" s="4" t="n"/>
       <c r="F72" s="4" t="n"/>
@@ -1974,7 +2010,11 @@
           <t>2026-10-13 | Login + csrf + approver check (admin, as the button); remarks and id bound instead of pasted into the sql.</t>
         </is>
       </c>
-      <c r="C73" s="4" t="n"/>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approver from Task Settings (PURCHASE_ORDER A).</t>
+        </is>
+      </c>
       <c r="D73" s="4" t="n"/>
       <c r="E73" s="4" t="n"/>
       <c r="F73" s="4" t="n"/>
@@ -1991,7 +2031,11 @@
           <t>2026-10-13 | Login + csrf + approver check (admin - the list is an admin-only menu); remarks and id bound.</t>
         </is>
       </c>
-      <c r="C74" s="4" t="n"/>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approver from Task Settings (PURCHASE_RETURN A).</t>
+        </is>
+      </c>
       <c r="D74" s="4" t="n"/>
       <c r="E74" s="4" t="n"/>
       <c r="F74" s="4" t="n"/>
@@ -2008,7 +2052,11 @@
           <t>2026-10-13 | Login + csrf + approver check: admin or the quotation's branch, as the button.</t>
         </is>
       </c>
-      <c r="C75" s="4" t="n"/>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approver from Task Settings (QUOTATION A, per branch).</t>
+        </is>
+      </c>
       <c r="D75" s="4" t="n"/>
       <c r="E75" s="4" t="n"/>
       <c r="F75" s="4" t="n"/>
@@ -2025,7 +2073,11 @@
           <t>2026-10-13 | Login + csrf + approver check (admin, as the button).</t>
         </is>
       </c>
-      <c r="C76" s="4" t="n"/>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approver from Task Settings (SALES_ORDER A).</t>
+        </is>
+      </c>
       <c r="D76" s="4" t="n"/>
       <c r="E76" s="4" t="n"/>
       <c r="F76" s="4" t="n"/>
@@ -2042,7 +2094,11 @@
           <t>2026-10-13 | Login + csrf + approver check: admin or the DC's branch, as the button.</t>
         </is>
       </c>
-      <c r="C77" s="4" t="n"/>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approver from Task Settings (DC A, per branch).</t>
+        </is>
+      </c>
       <c r="D77" s="4" t="n"/>
       <c r="E77" s="4" t="n"/>
       <c r="F77" s="4" t="n"/>
@@ -2059,7 +2115,11 @@
           <t>2026-10-13 | Login + csrf + check (admin, as the buttons).</t>
         </is>
       </c>
-      <c r="C78" s="4" t="n"/>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Send for approval / approve from Task Settings (SALES_REPAIR V / A).</t>
+        </is>
+      </c>
       <c r="D78" s="4" t="n"/>
       <c r="E78" s="4" t="n"/>
       <c r="F78" s="4" t="n"/>
@@ -2076,7 +2136,11 @@
           <t>2026-10-13 | Login + csrf + check: holders of the Sales Order in Accounts menu. Verifier saved from _user_id - it was always empty.</t>
         </is>
       </c>
-      <c r="C79" s="4" t="n"/>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Verifier from Task Settings (SALES_RECEIPT V) - was the Sales Order in Accounts menu.</t>
+        </is>
+      </c>
       <c r="D79" s="4" t="n"/>
       <c r="E79" s="4" t="n"/>
       <c r="F79" s="4" t="n"/>
@@ -2093,7 +2157,11 @@
           <t>2026-10-13 | Csrf + check: holders of the Sales Order in Accounts menu; so_id bound.</t>
         </is>
       </c>
-      <c r="C80" s="4" t="n"/>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Verifier from Task Settings (SALES_RECEIPT V) - was the Sales Order in Accounts menu.</t>
+        </is>
+      </c>
       <c r="D80" s="4" t="n"/>
       <c r="E80" s="4" t="n"/>
       <c r="F80" s="4" t="n"/>
@@ -2110,7 +2178,11 @@
           <t>2026-10-13 | Csrf token on the form + approver check (admin, the only user shown the link).</t>
         </is>
       </c>
-      <c r="C81" s="4" t="n"/>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approver from Task Settings (SUPPLIER A).</t>
+        </is>
+      </c>
       <c r="D81" s="4" t="n"/>
       <c r="E81" s="4" t="n"/>
       <c r="F81" s="4" t="n"/>
@@ -2127,7 +2199,11 @@
           <t>2026-10-13 | Update allowed for admin at head office or the item-approval users; updated_by from _user_id (was empty).</t>
         </is>
       </c>
-      <c r="C82" s="4" t="n"/>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Item creators and approvers from Task Settings (ITEM C / A).</t>
+        </is>
+      </c>
       <c r="D82" s="4" t="n"/>
       <c r="E82" s="4" t="n"/>
       <c r="F82" s="4" t="n"/>
@@ -2149,6 +2225,873 @@
       <c r="E83" s="4" t="n"/>
       <c r="F83" s="4" t="n"/>
       <c r="G83" s="4" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>attendance_report_ot.php</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Salary issue button for approvers in Task Settings (SALARY A) - was admin.</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="n"/>
+      <c r="D84" s="4" t="n"/>
+      <c r="E84" s="4" t="n"/>
+      <c r="F84" s="4" t="n"/>
+      <c r="G84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>attendance_report_pf.php</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Salary issue button for approvers in Task Settings (SALARY A) - was admin.</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="n"/>
+      <c r="D85" s="4" t="n"/>
+      <c r="E85" s="4" t="n"/>
+      <c r="F85" s="4" t="n"/>
+      <c r="G85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>attendance_report_withoutpf.php</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Salary issue button for approvers in Task Settings (SALARY A) - was admin.</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="n"/>
+      <c r="D86" s="4" t="n"/>
+      <c r="E86" s="4" t="n"/>
+      <c r="F86" s="4" t="n"/>
+      <c r="G86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>dc_list.php</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (DC W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="n"/>
+      <c r="D87" s="4" t="n"/>
+      <c r="E87" s="4" t="n"/>
+      <c r="F87" s="4" t="n"/>
+      <c r="G87" s="4" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>dc_print.php</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approve / reject for approvers in Task Settings (DC A) - was admin or the DC's branch.</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="n"/>
+      <c r="D88" s="4" t="n"/>
+      <c r="E88" s="4" t="n"/>
+      <c r="F88" s="4" t="n"/>
+      <c r="G88" s="4" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>employee_advance.php</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (EMPLOYEE W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="n"/>
+      <c r="D89" s="4" t="n"/>
+      <c r="E89" s="4" t="n"/>
+      <c r="F89" s="4" t="n"/>
+      <c r="G89" s="4" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>employee_debit_note.php</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (EMPLOYEE W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="n"/>
+      <c r="D90" s="4" t="n"/>
+      <c r="E90" s="4" t="n"/>
+      <c r="F90" s="4" t="n"/>
+      <c r="G90" s="4" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>employee_salary.php</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (EMPLOYEE W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="n"/>
+      <c r="D91" s="4" t="n"/>
+      <c r="E91" s="4" t="n"/>
+      <c r="F91" s="4" t="n"/>
+      <c r="G91" s="4" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>grn_list.php</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (GRN W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="n"/>
+      <c r="D92" s="4" t="n"/>
+      <c r="E92" s="4" t="n"/>
+      <c r="F92" s="4" t="n"/>
+      <c r="G92" s="4" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>grn_payment_details.php</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (GRN_PAYMENT W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="n"/>
+      <c r="D93" s="4" t="n"/>
+      <c r="E93" s="4" t="n"/>
+      <c r="F93" s="4" t="n"/>
+      <c r="G93" s="4" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>home.php</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Dashboard tiles shown to all-branch approvers of each task (PO, supplier, quotation, credit sales, new item, GRN payment) - were the tbl_task_user ids.</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="n"/>
+      <c r="D94" s="4" t="n"/>
+      <c r="E94" s="4" t="n"/>
+      <c r="F94" s="4" t="n"/>
+      <c r="G94" s="4" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxDclist.php</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (DC W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="n"/>
+      <c r="D95" s="4" t="n"/>
+      <c r="E95" s="4" t="n"/>
+      <c r="F95" s="4" t="n"/>
+      <c r="G95" s="4" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxEmployeeAdvance.php</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="n"/>
+      <c r="D96" s="4" t="n"/>
+      <c r="E96" s="4" t="n"/>
+      <c r="F96" s="4" t="n"/>
+      <c r="G96" s="4" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxEmployeeDebit.php</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="n"/>
+      <c r="D97" s="4" t="n"/>
+      <c r="E97" s="4" t="n"/>
+      <c r="F97" s="4" t="n"/>
+      <c r="G97" s="4" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxEmployeeSalarySet.php</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="n"/>
+      <c r="D98" s="4" t="n"/>
+      <c r="E98" s="4" t="n"/>
+      <c r="F98" s="4" t="n"/>
+      <c r="G98" s="4" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxEmployeeWorkDetsList.php</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="n"/>
+      <c r="D99" s="4" t="n"/>
+      <c r="E99" s="4" t="n"/>
+      <c r="F99" s="4" t="n"/>
+      <c r="G99" s="4" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxEmployeelist.php</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="n"/>
+      <c r="D100" s="4" t="n"/>
+      <c r="E100" s="4" t="n"/>
+      <c r="F100" s="4" t="n"/>
+      <c r="G100" s="4" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxGrnList.php</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (GRN W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="n"/>
+      <c r="D101" s="4" t="n"/>
+      <c r="E101" s="4" t="n"/>
+      <c r="F101" s="4" t="n"/>
+      <c r="G101" s="4" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxGrnPaymentList.php</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (GRN_PAYMENT W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="n"/>
+      <c r="D102" s="4" t="n"/>
+      <c r="E102" s="4" t="n"/>
+      <c r="F102" s="4" t="n"/>
+      <c r="G102" s="4" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxInvoiceList.php</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (INVOICE W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="n"/>
+      <c r="D103" s="4" t="n"/>
+      <c r="E103" s="4" t="n"/>
+      <c r="F103" s="4" t="n"/>
+      <c r="G103" s="4" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxItemDetailsList.php</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Edit / price / branch / delete links for creators in Task Settings (ITEM C) - was admin at head office.</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="n"/>
+      <c r="D104" s="4" t="n"/>
+      <c r="E104" s="4" t="n"/>
+      <c r="F104" s="4" t="n"/>
+      <c r="G104" s="4" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxLabourList.php</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="n"/>
+      <c r="D105" s="4" t="n"/>
+      <c r="E105" s="4" t="n"/>
+      <c r="F105" s="4" t="n"/>
+      <c r="G105" s="4" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxPoList.php</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Edit links for creators in Task Settings (PURCHASE_ORDER C) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="n"/>
+      <c r="D106" s="4" t="n"/>
+      <c r="E106" s="4" t="n"/>
+      <c r="F106" s="4" t="n"/>
+      <c r="G106" s="4" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxPoPrepareList.php</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (PO_PREPARE W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="n"/>
+      <c r="D107" s="4" t="n"/>
+      <c r="E107" s="4" t="n"/>
+      <c r="F107" s="4" t="n"/>
+      <c r="G107" s="4" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxPurchaseReturnList.php</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | GRN cancel link for approvers in Task Settings (GRN A) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="n"/>
+      <c r="D108" s="4" t="n"/>
+      <c r="E108" s="4" t="n"/>
+      <c r="F108" s="4" t="n"/>
+      <c r="G108" s="4" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxQuotationlist.php</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (QUOTATION W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="n"/>
+      <c r="D109" s="4" t="n"/>
+      <c r="E109" s="4" t="n"/>
+      <c r="F109" s="4" t="n"/>
+      <c r="G109" s="4" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxReceiptlist.php</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (SALES_RECEIPT W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="n"/>
+      <c r="D110" s="4" t="n"/>
+      <c r="E110" s="4" t="n"/>
+      <c r="F110" s="4" t="n"/>
+      <c r="G110" s="4" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxSaleslist.php</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Cancel link for approvers in Task Settings (SALES_ORDER A) - was admin.</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="n"/>
+      <c r="D111" s="4" t="n"/>
+      <c r="E111" s="4" t="n"/>
+      <c r="F111" s="4" t="n"/>
+      <c r="G111" s="4" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxStaffList.php</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C112" s="4" t="n"/>
+      <c r="D112" s="4" t="n"/>
+      <c r="E112" s="4" t="n"/>
+      <c r="F112" s="4" t="n"/>
+      <c r="G112" s="4" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxSupplierList.php</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (SUPPLIER W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="n"/>
+      <c r="D113" s="4" t="n"/>
+      <c r="E113" s="4" t="n"/>
+      <c r="F113" s="4" t="n"/>
+      <c r="G113" s="4" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajax_SiList.php</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | All branches for viewers in Task Settings (STORE_INDENT W) - was admin or head office.</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="n"/>
+      <c r="D114" s="4" t="n"/>
+      <c r="E114" s="4" t="n"/>
+      <c r="F114" s="4" t="n"/>
+      <c r="G114" s="4" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>invoice_list.php</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (INVOICE W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="n"/>
+      <c r="D115" s="4" t="n"/>
+      <c r="E115" s="4" t="n"/>
+      <c r="F115" s="4" t="n"/>
+      <c r="G115" s="4" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>lst_direct_po.php</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | New PO button for creators and branch filter for viewers in Task Settings - were head office.</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="n"/>
+      <c r="D116" s="4" t="n"/>
+      <c r="E116" s="4" t="n"/>
+      <c r="F116" s="4" t="n"/>
+      <c r="G116" s="4" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>lst_employee.php</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (EMPLOYEE W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="n"/>
+      <c r="D117" s="4" t="n"/>
+      <c r="E117" s="4" t="n"/>
+      <c r="F117" s="4" t="n"/>
+      <c r="G117" s="4" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>lst_labour.php</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (EMPLOYEE W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="n"/>
+      <c r="D118" s="4" t="n"/>
+      <c r="E118" s="4" t="n"/>
+      <c r="F118" s="4" t="n"/>
+      <c r="G118" s="4" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>lst_quotation.php</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (QUOTATION W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="n"/>
+      <c r="D119" s="4" t="n"/>
+      <c r="E119" s="4" t="n"/>
+      <c r="F119" s="4" t="n"/>
+      <c r="G119" s="4" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>lst_sales_order.php</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (SALES_ORDER W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="n"/>
+      <c r="D120" s="4" t="n"/>
+      <c r="E120" s="4" t="n"/>
+      <c r="F120" s="4" t="n"/>
+      <c r="G120" s="4" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>lst_sales_receipt.php</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (SALES_RECEIPT W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="n"/>
+      <c r="D121" s="4" t="n"/>
+      <c r="E121" s="4" t="n"/>
+      <c r="F121" s="4" t="n"/>
+      <c r="G121" s="4" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>lst_staff.php</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (EMPLOYEE W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="n"/>
+      <c r="D122" s="4" t="n"/>
+      <c r="E122" s="4" t="n"/>
+      <c r="F122" s="4" t="n"/>
+      <c r="G122" s="4" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>lst_supplier.php</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (SUPPLIER W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="n"/>
+      <c r="D123" s="4" t="n"/>
+      <c r="E123" s="4" t="n"/>
+      <c r="F123" s="4" t="n"/>
+      <c r="G123" s="4" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>po_prepare_list.php</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (PO_PREPARE W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="n"/>
+      <c r="D124" s="4" t="n"/>
+      <c r="E124" s="4" t="n"/>
+      <c r="F124" s="4" t="n"/>
+      <c r="G124" s="4" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>po_print.php</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approve / reject for approvers in Task Settings (PURCHASE_ORDER A) - was admin.</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="n"/>
+      <c r="D125" s="4" t="n"/>
+      <c r="E125" s="4" t="n"/>
+      <c r="F125" s="4" t="n"/>
+      <c r="G125" s="4" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>print_quotation.php</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approve / reject for approvers in Task Settings (QUOTATION A) - was admin or the quotation's branch.</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="n"/>
+      <c r="D126" s="4" t="n"/>
+      <c r="E126" s="4" t="n"/>
+      <c r="F126" s="4" t="n"/>
+      <c r="G126" s="4" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>print_sales_order.php</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approve / reject for approvers in Task Settings (SALES_ORDER A) - was admin.</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="n"/>
+      <c r="D127" s="4" t="n"/>
+      <c r="E127" s="4" t="n"/>
+      <c r="F127" s="4" t="n"/>
+      <c r="G127" s="4" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>purchase_return_list.php</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (PURCHASE_RETURN W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="n"/>
+      <c r="D128" s="4" t="n"/>
+      <c r="E128" s="4" t="n"/>
+      <c r="F128" s="4" t="n"/>
+      <c r="G128" s="4" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>purchase_return_view.php</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approve / reject only for approvers in Task Settings (PURCHASE_RETURN A) - was anyone opening the page.</t>
+        </is>
+      </c>
+      <c r="C129" s="4" t="n"/>
+      <c r="D129" s="4" t="n"/>
+      <c r="E129" s="4" t="n"/>
+      <c r="F129" s="4" t="n"/>
+      <c r="G129" s="4" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>rpt_so_stock_list_branchwise.php</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Update location for creators in Task Settings (STOCK_LOCATION C) - was users 1 and 9.</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="n"/>
+      <c r="D130" s="4" t="n"/>
+      <c r="E130" s="4" t="n"/>
+      <c r="F130" s="4" t="n"/>
+      <c r="G130" s="4" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>sales_repair_print.php</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Send for approval (SALES_REPAIR V) and approve (SALES_REPAIR A) from Task Settings - were admin.</t>
+        </is>
+      </c>
+      <c r="C131" s="4" t="n"/>
+      <c r="D131" s="4" t="n"/>
+      <c r="E131" s="4" t="n"/>
+      <c r="F131" s="4" t="n"/>
+      <c r="G131" s="4" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>store_indent_list.php</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Branch filter for viewers in Task Settings (STORE_INDENT W) - was head office.</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="n"/>
+      <c r="D132" s="4" t="n"/>
+      <c r="E132" s="4" t="n"/>
+      <c r="F132" s="4" t="n"/>
+      <c r="G132" s="4" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>db/post_upload_131026.sql</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | New. Creates mst_task and tbl_task_assign, adds the 18 tasks, starting rows that give everyone exactly the access the code gave, and the Task Settings menu. Safe to run again.</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="n"/>
+      <c r="D133" s="4" t="n"/>
+      <c r="E133" s="4" t="n"/>
+      <c r="F133" s="4" t="n"/>
+      <c r="G133" s="4" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>mst_task.php</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | New. Settings &gt; Task Settings (admin only): add a task, tick the roles it uses, add many users per role with a branch or All, edit or deactivate a task; list shows who holds each role.</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="n"/>
+      <c r="D134" s="4" t="n"/>
+      <c r="E134" s="4" t="n"/>
+      <c r="F134" s="4" t="n"/>
+      <c r="G134" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2161,7 +3104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2249,12 +3192,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>mst_category</t>
+          <t>mst_task</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12 | (rows) | SPAC import adds AIR GUN, FRL, TUBING. Sheet FITTING mapped to the existing FITTINGS.</t>
+          <t>2026-10-13 | (new table) | One row per task: code checked by the screens, name, module, roles used (C V A W), note, status.</t>
         </is>
       </c>
       <c r="C2" s="4" t="n"/>
@@ -2272,12 +3215,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>mst_hsn</t>
+          <t>tbl_task_assign</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12 | (rows) | SPAC import adds 39173290, 39174000, 40169390, 84678910, 84812000, 85045090, 85365090, 85444999 at 18% (9 + 9).</t>
+          <t>2026-10-13 | (new table) | One row per task / role / user / branch (0 = all). Starting rows reproduce the old coded rules: head office users view every branch and create POs, branch users approve their branch's quotations and DCs, accounts confirms payments.</t>
         </is>
       </c>
       <c r="C3" s="4" t="n"/>
@@ -2295,12 +3238,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>tbl_item_details / tbl_item_stock</t>
+          <t>mst_sub_menu</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-12 | (rows) | SPAC import adds 4,702 items (principal SPAC, Pneumatic, Trading, branches 1,2,3) and one stock row each.</t>
+          <t>2026-10-13 | (row) | Settings &gt; Task Settings (mst_task.php).</t>
         </is>
       </c>
       <c r="C4" s="4" t="n"/>
@@ -2318,12 +3261,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>mst_principal</t>
+          <t>tbl_task_user</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-06 | created_by, created_dtm, modify_by, modify_dtm | Added - mst_principal.php writes them on save and update, so both always failed with Unknown column. Existing rows get 0 / NULL.</t>
+          <t>2026-10-13 | (no longer read) | Its user lists are copied into tbl_task_assign by the 13-10-26 script; can be dropped once the new files are live.</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -2341,24 +3284,16 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>tbl_user_rights</t>
+          <t>mst_category</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | sm_id | Signed TINYINT widened to SMALLINT. It stopped at 127, so the rights rows for the new menus (147, 148) were silently clamped to 127 and the menus never showed.</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | mm_id | Signed TINYINT widened to SMALLINT, same reason - it was two main menus away from the same limit.</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | (rows) | Six clamped rows deleted (users 2/6/7, sm_id 127 under main menus 3 and 20); sm_id 147 and 148 granted to whoever holds the parent menu.</t>
-        </is>
-      </c>
+          <t>2026-10-12 | (rows) | SPAC import adds AIR GUN, FRL, TUBING. Sheet FITTING mapped to the existing FITTINGS.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
@@ -2372,19 +3307,15 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>tbl_invoice_details</t>
+          <t>mst_hsn</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05 | inv_value, tax_value | 111 rows across 35 invoices rebuilt as net_value / (1 + vat/100); tax_value rebuilt with them. Backup taken as tbl_invoice_details_bkp_051026.</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-05 | cgst_per, sgst_per, igst_per, cgst_val, sgst_val, igst_val | Optional tidy on the same 111 rows only.</t>
-        </is>
-      </c>
+          <t>2026-10-12 | (rows) | SPAC import adds 39173290, 39174000, 40169390, 84678910, 84812000, 85045090, 85365090, 85444999 at 18% (9 + 9).</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
@@ -2399,106 +3330,42 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>tbl_stock_flow</t>
+          <t>tbl_item_details / tbl_item_stock</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | trans_dir | Added CHAR(1). I = stock in (+), O = stock out (-). Backfilled GRN=I, INV/SALE=O.</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | trans_remarks | Added VARCHAR(255). Reason / narration, mandatory on ADJ rows.</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | stock_field | Added VARCHAR(30). Which tbl_item_stock column was changed. Backfilled from mst_branch.</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | before_qty | INT to DECIMAL(12,3). Was truncating decimal stock.</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | trans_qty | INT to DECIMAL(12,3). Always a positive magnitude, direction is in trans_dir.</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | rcvd_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | after_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | reje_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | pend_qty | INT to DECIMAL(12,3).</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | trans_type | VARCHAR(8) to VARCHAR(10). Values GRN, INV, ADJ, OPEN, RET.</t>
-        </is>
-      </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | idx_sf_item_branch_date | Index added on (item_id, branch_id, trans_date) - what the reports filter on.</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | idx_sf_trans | Index added on (trans_type, trans_id).</t>
-        </is>
-      </c>
+          <t>2026-10-12 | (rows) | SPAC import adds 4,702 items (principal SPAC, Pneumatic, Trading, branches 1,2,3) and one stock row each.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="4" t="n"/>
+      <c r="L8" s="4" t="n"/>
+      <c r="M8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>tbl_stock_adjustment</t>
+          <t>mst_principal</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (new table) | Header for every manual stock correction. One row per adjustment.</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | adj_id, adj_refno, adj_slno, adj_finyr | Key and reference number ADJ/nnnn/BIE/&lt;branch&gt;/&lt;finyr&gt;.</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | adj_date, branch_id, stock_field, item_id | What was adjusted, where, and which stock column.</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | adj_type, adj_qty, before_qty, after_qty | I = increase, D = decrease. adj_qty is always positive.</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | item_price, adj_reason, adj_status | Reason is mandatory. adj_status 1 = active, 0 = deleted.</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-22 | created_by, created_dtm | Who made the adjustment and when.</t>
-        </is>
-      </c>
+          <t>2026-10-06 | created_by, created_dtm, modify_by, modify_dtm | Added - mst_principal.php writes them on save and update, so both always failed with Unknown column. Existing rows get 0 / NULL.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="4" t="n"/>
       <c r="J9" s="4" t="n"/>
@@ -2509,20 +3376,24 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>mst_sub_menu</t>
+          <t>tbl_user_rights</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (row) | sm_id 147, mm_id 20 (Stores) - Stock Adjustment, stock_adjustment.php.</t>
+          <t>2026-10-05 | sm_id | Signed TINYINT widened to SMALLINT. It stopped at 127, so the rights rows for the new menus (147, 148) were silently clamped to 127 and the menus never showed.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 | (row) | sm_id 148, mm_id 3 (Item Masters) - Item Stock List, lst_item_stock.php.</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="n"/>
+          <t>2026-10-05 | mm_id | Signed TINYINT widened to SMALLINT, same reason - it was two main menus away from the same limit.</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05 | (rows) | Six clamped rows deleted (users 2/6/7, sm_id 127 under main menus 3 and 20); sm_id 147 and 148 granted to whoever holds the parent menu.</t>
+        </is>
+      </c>
       <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
@@ -2536,17 +3407,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>tbl_user_rights</t>
+          <t>tbl_invoice_details</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (rows) | sm_id 147 granted to every user who already has the Stores menu.</t>
+          <t>2026-10-05 | inv_value, tax_value | 111 rows across 35 invoices rebuilt as net_value / (1 + vat/100); tax_value rebuilt with them. Backup taken as tbl_invoice_details_bkp_051026.</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 | (rows) | sm_id 148 granted to every user who already has the Item Masters menu.</t>
+          <t>2026-10-05 | cgst_per, sgst_per, igst_per, cgst_val, sgst_val, igst_val | Optional tidy on the same 111 rows only.</t>
         </is>
       </c>
       <c r="D11" s="4" t="n"/>
@@ -2563,46 +3434,106 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>tbl_item_stock</t>
+          <t>tbl_stock_flow</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | (no schema change) | Qty columns are now only written through fnApplyStockMovement(), never directly.</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
-      <c r="K12" s="4" t="n"/>
-      <c r="L12" s="4" t="n"/>
-      <c r="M12" s="4" t="n"/>
+          <t>2026-09-22 | trans_dir | Added CHAR(1). I = stock in (+), O = stock out (-). Backfilled GRN=I, INV/SALE=O.</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | trans_remarks | Added VARCHAR(255). Reason / narration, mandatory on ADJ rows.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | stock_field | Added VARCHAR(30). Which tbl_item_stock column was changed. Backfilled from mst_branch.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | before_qty | INT to DECIMAL(12,3). Was truncating decimal stock.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | trans_qty | INT to DECIMAL(12,3). Always a positive magnitude, direction is in trans_dir.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | rcvd_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | after_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | reje_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | pend_qty | INT to DECIMAL(12,3).</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | trans_type | VARCHAR(8) to VARCHAR(10). Values GRN, INV, ADJ, OPEN, RET.</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | idx_sf_item_branch_date | Index added on (item_id, branch_id, trans_date) - what the reports filter on.</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | idx_sf_trans | Index added on (trans_type, trans_id).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>tbl_cash_details</t>
+          <t>tbl_stock_adjustment</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Not deleted - old receipts hold cash_id 7 and history screens look the name up without checking status.</t>
+          <t>2026-09-22 | (new table) | Header for every manual stock correction. One row per adjustment.</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Sales Receipt screen.</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
+          <t>2026-09-22 | adj_id, adj_refno, adj_slno, adj_finyr | Key and reference number ADJ/nnnn/BIE/&lt;branch&gt;/&lt;finyr&gt;.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | adj_date, branch_id, stock_field, item_id | What was adjusted, where, and which stock column.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | adj_type, adj_qty, before_qty, after_qty | I = increase, D = decrease. adj_qty is always positive.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | item_price, adj_reason, adj_status | Reason is mandatory. adj_status 1 = active, 0 = deleted.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | created_by, created_dtm | Who made the adjustment and when.</t>
+        </is>
+      </c>
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="4" t="n"/>
       <c r="J13" s="4" t="n"/>
@@ -2613,17 +3544,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>mst_cash_details</t>
+          <t>mst_sub_menu</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Same reasoning as tbl_cash_details.</t>
+          <t>2026-09-22 | (row) | sm_id 147, mm_id 20 (Stores) - Stock Adjustment, stock_adjustment.php.</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Invoice and Credit screens.</t>
+          <t>2026-09-23 | (row) | sm_id 148, mm_id 3 (Item Masters) - Item Stock List, lst_item_stock.php.</t>
         </is>
       </c>
       <c r="D14" s="4" t="n"/>
@@ -2640,15 +3571,19 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>mst_customer_branch_temp</t>
+          <t>tbl_user_rights</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. Branch rows live in the page and post back as arrays. Drop with db/drop_temp_tables.sql.</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="n"/>
+          <t>2026-09-22 | (rows) | sm_id 147 granted to every user who already has the Stores menu.</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23 | (rows) | sm_id 148 granted to every user who already has the Item Masters menu.</t>
+        </is>
+      </c>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
@@ -2663,12 +3598,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>tbl_item_group_details_temp</t>
+          <t>tbl_item_stock</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. Group items live in the page. Drop with db/drop_temp_tables.sql.</t>
+          <t>2026-09-22 | (no schema change) | Qty columns are now only written through fnApplyStockMovement(), never directly.</t>
         </is>
       </c>
       <c r="C16" s="4" t="n"/>
@@ -2686,15 +3621,19 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>tbl_dc_details_temp</t>
+          <t>tbl_cash_details</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. DC item rows are built in php and posted back as arrays. Drop with db/drop_temp_tables.sql.</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="n"/>
+          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Not deleted - old receipts hold cash_id 7 and history screens look the name up without checking status.</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Sales Receipt screen.</t>
+        </is>
+      </c>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
@@ -2709,15 +3648,19 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>tbl_package_box_details_temp</t>
+          <t>mst_cash_details</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01 | (whole table) | No longer used. Packing rides on the DC item row as csv hidden fields. Drop with db/drop_temp_tables.sql.</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="n"/>
+          <t>2026-09-25 | cash_status | 2000.00 set to 0 (retired). Same reasoning as tbl_cash_details.</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 | (rows) | Added cash_id 8 = 1.00, 9 = 2.00, 10 = 5.00, all active. Used by the Invoice and Credit screens.</t>
+        </is>
+      </c>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
@@ -2732,12 +3675,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>tbl_invoice_details</t>
+          <t>mst_customer_branch_temp</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30 | inv_value | No schema change. Data repair - rows saved from the invoice edit screen had this zeroed by a bad field mapping. Rebuilt as net_value - tax_value where that agrees with qty x unit_price less discount.</t>
+          <t>2026-10-01 | (whole table) | No longer used. Branch rows live in the page and post back as arrays. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C19" s="4" t="n"/>
@@ -2755,12 +3698,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>tbl_proforma_details</t>
+          <t>tbl_item_group_details_temp</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>2026-09-30 | pro_value | No schema change. Same data repair as tbl_invoice_details.</t>
+          <t>2026-10-01 | (whole table) | No longer used. Group items live in the page. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C20" s="4" t="n"/>
@@ -2778,12 +3721,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>tbl_item_details</t>
+          <t>tbl_dc_details_temp</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-22 | item_curr_stock | No change. Noted as dead - every write to it was already commented out. Branch columns in tbl_item_stock are the live balance.</t>
+          <t>2026-10-01 | (whole table) | No longer used. DC item rows are built in php and posted back as arrays. Drop with db/drop_temp_tables.sql.</t>
         </is>
       </c>
       <c r="C21" s="4" t="n"/>
@@ -2798,6 +3741,98 @@
       <c r="L21" s="4" t="n"/>
       <c r="M21" s="4" t="n"/>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>tbl_package_box_details_temp</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-01 | (whole table) | No longer used. Packing rides on the DC item row as csv hidden fields. Drop with db/drop_temp_tables.sql.</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
+      <c r="J22" s="4" t="n"/>
+      <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="n"/>
+      <c r="M22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>tbl_invoice_details</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30 | inv_value | No schema change. Data repair - rows saved from the invoice edit screen had this zeroed by a bad field mapping. Rebuilt as net_value - tax_value where that agrees with qty x unit_price less discount.</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
+      <c r="J23" s="4" t="n"/>
+      <c r="K23" s="4" t="n"/>
+      <c r="L23" s="4" t="n"/>
+      <c r="M23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>tbl_proforma_details</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30 | pro_value | No schema change. Same data repair as tbl_invoice_details.</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
+      <c r="J24" s="4" t="n"/>
+      <c r="K24" s="4" t="n"/>
+      <c r="L24" s="4" t="n"/>
+      <c r="M24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>tbl_item_details</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22 | item_curr_stock | No change. Noted as dead - every write to it was already commented out. Branch columns in tbl_item_stock are the live balance.</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
+      <c r="I25" s="4" t="n"/>
+      <c r="J25" s="4" t="n"/>
+      <c r="K25" s="4" t="n"/>
+      <c r="L25" s="4" t="n"/>
+      <c r="M25" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Dashboard tiles: supplier, quotation and GRN payment counts match the pages they open
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G134"/>
+  <dimension ref="A1:G135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2407,7 +2407,11 @@
           <t>2026-10-13 | Dashboard tiles shown to all-branch approvers of each task (PO, supplier, quotation, credit sales, new item, GRN payment) - were the tbl_task_user ids.</t>
         </is>
       </c>
-      <c r="C94" s="4" t="n"/>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | GRN Payment Pending tile counts what its page lists (bill and payment both not done) - it counted bill only.</t>
+        </is>
+      </c>
       <c r="D94" s="4" t="n"/>
       <c r="E94" s="4" t="n"/>
       <c r="F94" s="4" t="n"/>
@@ -2900,7 +2904,11 @@
           <t>2026-10-13 | Branch filter for viewers in Task Settings (SUPPLIER W) - was head office.</t>
         </is>
       </c>
-      <c r="C123" s="4" t="n"/>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Opened from the Supplier InApproval tile the branch filter starts at All - it showed head office only, so a pending Kerala supplier was counted but not listed.</t>
+        </is>
+      </c>
       <c r="D123" s="4" t="n"/>
       <c r="E123" s="4" t="n"/>
       <c r="F123" s="4" t="n"/>
@@ -3092,6 +3100,23 @@
       <c r="E134" s="4" t="n"/>
       <c r="F134" s="4" t="n"/>
       <c r="G134" s="4" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>lst_quo_approval.php</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Deleted quotations (quo_status 0) left out, as the dashboard tile does.</t>
+        </is>
+      </c>
+      <c r="C135" s="4" t="n"/>
+      <c r="D135" s="4" t="n"/>
+      <c r="E135" s="4" t="n"/>
+      <c r="F135" s="4" t="n"/>
+      <c r="G135" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Dashboard tiles for every verify / approve job, counted for the user's branches; sales order approve and payment confirm open to all users as before
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G135"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1027,7 +1027,11 @@
           <t>2026-10-13 | Loads access.php.</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n"/>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Loads task_queues.php.</t>
+        </is>
+      </c>
       <c r="F24" s="4" t="n"/>
       <c r="G24" s="4" t="n"/>
     </row>
@@ -1302,7 +1306,11 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
-      <c r="D36" s="4" t="n"/>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Mark as credit follows Sales Order in Accounts verifier - showed to every user (every user holds it to begin with).</t>
+        </is>
+      </c>
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
@@ -1724,7 +1732,11 @@
           <t>2026-10-13 | Cancel for approvers in Task Settings (SALES_ORDER A).</t>
         </is>
       </c>
-      <c r="E57" s="4" t="n"/>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Cancel checked against SO_CANCEL.</t>
+        </is>
+      </c>
       <c r="F57" s="4" t="n"/>
       <c r="G57" s="4" t="n"/>
     </row>
@@ -1994,7 +2006,11 @@
           <t>2026-10-13 | fnTaskCan(code, role, branch), fnTaskIsAdmin, fnTaskDefaultUser; rows read once per request. fnUserHasMenu / fnTaskUserListed removed.</t>
         </is>
       </c>
-      <c r="D72" s="4" t="n"/>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | fnTaskBranches - the branches a user holds a role for.</t>
+        </is>
+      </c>
       <c r="E72" s="4" t="n"/>
       <c r="F72" s="4" t="n"/>
       <c r="G72" s="4" t="n"/>
@@ -2412,7 +2428,11 @@
           <t>2026-10-13 | GRN Payment Pending tile counts what its page lists (bill and payment both not done) - it counted bill only.</t>
         </is>
       </c>
-      <c r="D94" s="4" t="n"/>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Tiles built from task_queues.php: every verify / approve job the user holds, any branch; count limited to their branches.</t>
+        </is>
+      </c>
       <c r="E94" s="4" t="n"/>
       <c r="F94" s="4" t="n"/>
       <c r="G94" s="4" t="n"/>
@@ -2700,7 +2720,11 @@
           <t>2026-10-13 | Cancel link for approvers in Task Settings (SALES_ORDER A) - was admin.</t>
         </is>
       </c>
-      <c r="C111" s="4" t="n"/>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Cancel link moved to its own task SO_CANCEL (admin) - approve and cancel are different people.</t>
+        </is>
+      </c>
       <c r="D111" s="4" t="n"/>
       <c r="E111" s="4" t="n"/>
       <c r="F111" s="4" t="n"/>
@@ -2734,7 +2758,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (SUPPLIER W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C113" s="4" t="n"/>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Tile mode: pending suppliers of the user's approver branches; status filter cast to int.</t>
+        </is>
+      </c>
       <c r="D113" s="4" t="n"/>
       <c r="E113" s="4" t="n"/>
       <c r="F113" s="4" t="n"/>
@@ -2909,7 +2937,11 @@
           <t>2026-10-13 | Opened from the Supplier InApproval tile the branch filter starts at All - it showed head office only, so a pending Kerala supplier was counted but not listed.</t>
         </is>
       </c>
-      <c r="D123" s="4" t="n"/>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | From the tile it lists the pending suppliers of the branches the user approves for.</t>
+        </is>
+      </c>
       <c r="E123" s="4" t="n"/>
       <c r="F123" s="4" t="n"/>
       <c r="G123" s="4" t="n"/>
@@ -2976,7 +3008,11 @@
           <t>2026-10-13 | Approve / reject for approvers in Task Settings (SALES_ORDER A) - was admin.</t>
         </is>
       </c>
-      <c r="C127" s="4" t="n"/>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Approve / reject buttons follow Sales Order approver - they showed to every user (every user holds it to begin with).</t>
+        </is>
+      </c>
       <c r="D127" s="4" t="n"/>
       <c r="E127" s="4" t="n"/>
       <c r="F127" s="4" t="n"/>
@@ -3078,7 +3114,11 @@
           <t>2026-10-13 | New. Creates mst_task and tbl_task_assign, adds the 18 tasks, starting rows that give everyone exactly the access the code gave, and the Task Settings menu. Safe to run again.</t>
         </is>
       </c>
-      <c r="C133" s="4" t="n"/>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Second block: SO_CANCEL task; sales order approver and payment verifier for every user (head office all branches, others own) - the buttons had no check. Runs once, also where the first version ran.</t>
+        </is>
+      </c>
       <c r="D133" s="4" t="n"/>
       <c r="E133" s="4" t="n"/>
       <c r="F133" s="4" t="n"/>
@@ -3112,11 +3152,117 @@
           <t>2026-10-13 | Deleted quotations (quo_status 0) left out, as the dashboard tile does.</t>
         </is>
       </c>
-      <c r="C135" s="4" t="n"/>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | List limited to the branches the user approves for, same rule as the tile.</t>
+        </is>
+      </c>
       <c r="D135" s="4" t="n"/>
       <c r="E135" s="4" t="n"/>
       <c r="F135" s="4" t="n"/>
       <c r="G135" s="4" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>inc/common/task_queues.php</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | New. One definition per dashboard tile: task / role, waiting rule, branch column, page it opens; count and page share it.</t>
+        </is>
+      </c>
+      <c r="C136" s="4" t="n"/>
+      <c r="D136" s="4" t="n"/>
+      <c r="E136" s="4" t="n"/>
+      <c r="F136" s="4" t="n"/>
+      <c r="G136" s="4" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>lst_pending.php</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | New. Waiting list behind the new tiles (sales order, payment, DC, purchase return, repair) with an Open link; only for holders of the job, their branches.</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="n"/>
+      <c r="D137" s="4" t="n"/>
+      <c r="E137" s="4" t="n"/>
+      <c r="F137" s="4" t="n"/>
+      <c r="G137" s="4" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>lst_direct_po_approval.php</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | List limited to the branches the user approves for, same rule as the tile.</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="n"/>
+      <c r="D138" s="4" t="n"/>
+      <c r="E138" s="4" t="n"/>
+      <c r="F138" s="4" t="n"/>
+      <c r="G138" s="4" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>lst_so_approval.php</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | List limited to the branches the user approves for, same rule as the tile.</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="n"/>
+      <c r="D139" s="4" t="n"/>
+      <c r="E139" s="4" t="n"/>
+      <c r="F139" s="4" t="n"/>
+      <c r="G139" s="4" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>lst_item_approval.php</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | List only for item approvers, same rule as the tile.</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="n"/>
+      <c r="D140" s="4" t="n"/>
+      <c r="E140" s="4" t="n"/>
+      <c r="F140" s="4" t="n"/>
+      <c r="G140" s="4" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>grn_payment_details_pending.php</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | List limited to the branches the user approves for, same rule as the tile.</t>
+        </is>
+      </c>
+      <c r="C141" s="4" t="n"/>
+      <c r="D141" s="4" t="n"/>
+      <c r="E141" s="4" t="n"/>
+      <c r="F141" s="4" t="n"/>
+      <c r="G141" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3248,7 +3394,11 @@
           <t>2026-10-13 | (new table) | One row per task / role / user / branch (0 = all). Starting rows reproduce the old coded rules: head office users view every branch and create POs, branch users approve their branch's quotations and DCs, accounts confirms payments.</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | (rows) | Sales order approver and payment verifier: every user (head office all branches, others own branch). New task SO_CANCEL for cancel (admin).</t>
+        </is>
+      </c>
       <c r="D3" s="4" t="n"/>
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>

</xml_diff>

<commit_message>
Critical: delete endpoint locked down; Task Settings branch fixes, approval state checks, attendance branch filter
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1077,7 +1077,11 @@
           <t>2026-10-13 | Named approver from Task Settings (QUOTATION A, else admin) - was tbl_task_user 1.</t>
         </is>
       </c>
-      <c r="E26" s="4" t="n"/>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Named approver may be a holder for the quotation's branch.</t>
+        </is>
+      </c>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
     </row>
@@ -1185,7 +1189,11 @@
           <t>2026-10-13 | Named approver from Task Settings (PURCHASE_ORDER A, else admin) - was tbl_task_user 1.</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Named approver may be a holder for the PO's branch.</t>
+        </is>
+      </c>
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="n"/>
     </row>
@@ -1210,7 +1218,11 @@
           <t>2026-10-13 | Named approver from Task Settings (STORE_INDENT A, else admin) - was tbl_task_user 1.</t>
         </is>
       </c>
-      <c r="E31" s="4" t="n"/>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Named approver may be a holder for the indent's branch.</t>
+        </is>
+      </c>
       <c r="F31" s="4" t="n"/>
       <c r="G31" s="4" t="n"/>
     </row>
@@ -1707,7 +1719,11 @@
           <t>2026-10-13 | Credit approval for approvers in Task Settings (CREDIT_SALES A).</t>
         </is>
       </c>
-      <c r="E56" s="4" t="n"/>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Only a sales order waiting for credit approval.</t>
+        </is>
+      </c>
       <c r="F56" s="4" t="n"/>
       <c r="G56" s="4" t="n"/>
     </row>
@@ -2011,7 +2027,11 @@
           <t>2026-10-13 | fnTaskBranches - the branches a user holds a role for.</t>
         </is>
       </c>
-      <c r="E72" s="4" t="n"/>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Named approver: All-branch holder, then the document's branch, else admin.</t>
+        </is>
+      </c>
       <c r="F72" s="4" t="n"/>
       <c r="G72" s="4" t="n"/>
     </row>
@@ -2031,7 +2051,11 @@
           <t>2026-10-13 | Approver from Task Settings (PURCHASE_ORDER A).</t>
         </is>
       </c>
-      <c r="D73" s="4" t="n"/>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Only a PO in approval can be approved / rejected; otherwise 'not waiting'.</t>
+        </is>
+      </c>
       <c r="E73" s="4" t="n"/>
       <c r="F73" s="4" t="n"/>
       <c r="G73" s="4" t="n"/>
@@ -2052,7 +2076,11 @@
           <t>2026-10-13 | Approver from Task Settings (PURCHASE_RETURN A).</t>
         </is>
       </c>
-      <c r="D74" s="4" t="n"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Only a return sent and not decided.</t>
+        </is>
+      </c>
       <c r="E74" s="4" t="n"/>
       <c r="F74" s="4" t="n"/>
       <c r="G74" s="4" t="n"/>
@@ -2073,7 +2101,11 @@
           <t>2026-10-13 | Approver from Task Settings (QUOTATION A, per branch).</t>
         </is>
       </c>
-      <c r="D75" s="4" t="n"/>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Only a quotation sent and not decided.</t>
+        </is>
+      </c>
       <c r="E75" s="4" t="n"/>
       <c r="F75" s="4" t="n"/>
       <c r="G75" s="4" t="n"/>
@@ -2094,7 +2126,11 @@
           <t>2026-10-13 | Approver from Task Settings (SALES_ORDER A).</t>
         </is>
       </c>
-      <c r="D76" s="4" t="n"/>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Only a verified, open sales order.</t>
+        </is>
+      </c>
       <c r="E76" s="4" t="n"/>
       <c r="F76" s="4" t="n"/>
       <c r="G76" s="4" t="n"/>
@@ -2115,7 +2151,11 @@
           <t>2026-10-13 | Approver from Task Settings (DC A, per branch).</t>
         </is>
       </c>
-      <c r="D77" s="4" t="n"/>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Only a DC sent and not decided.</t>
+        </is>
+      </c>
       <c r="E77" s="4" t="n"/>
       <c r="F77" s="4" t="n"/>
       <c r="G77" s="4" t="n"/>
@@ -2136,7 +2176,11 @@
           <t>2026-10-13 | Send for approval / approve from Task Settings (SALES_REPAIR V / A).</t>
         </is>
       </c>
-      <c r="D78" s="4" t="n"/>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Repair's branch (company_id) passed; send / approve only in the right state.</t>
+        </is>
+      </c>
       <c r="E78" s="4" t="n"/>
       <c r="F78" s="4" t="n"/>
       <c r="G78" s="4" t="n"/>
@@ -2253,7 +2297,11 @@
           <t>2026-10-13 | Salary issue button for approvers in Task Settings (SALARY A) - was admin.</t>
         </is>
       </c>
-      <c r="C84" s="4" t="n"/>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Issue button checked against the employee's branch.</t>
+        </is>
+      </c>
       <c r="D84" s="4" t="n"/>
       <c r="E84" s="4" t="n"/>
       <c r="F84" s="4" t="n"/>
@@ -2270,7 +2318,11 @@
           <t>2026-10-13 | Salary issue button for approvers in Task Settings (SALARY A) - was admin.</t>
         </is>
       </c>
-      <c r="C85" s="4" t="n"/>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Issue button checked against the employee's branch.</t>
+        </is>
+      </c>
       <c r="D85" s="4" t="n"/>
       <c r="E85" s="4" t="n"/>
       <c r="F85" s="4" t="n"/>
@@ -2287,7 +2339,11 @@
           <t>2026-10-13 | Salary issue button for approvers in Task Settings (SALARY A) - was admin.</t>
         </is>
       </c>
-      <c r="C86" s="4" t="n"/>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Issue button checked against the employee's branch.</t>
+        </is>
+      </c>
       <c r="D86" s="4" t="n"/>
       <c r="E86" s="4" t="n"/>
       <c r="F86" s="4" t="n"/>
@@ -2516,7 +2572,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C99" s="4" t="n"/>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Own branch only without the Employee viewer role - every branch showed.</t>
+        </is>
+      </c>
       <c r="D99" s="4" t="n"/>
       <c r="E99" s="4" t="n"/>
       <c r="F99" s="4" t="n"/>
@@ -2830,7 +2890,11 @@
           <t>2026-10-13 | Branch filter for viewers in Task Settings (EMPLOYEE W) - was head office.</t>
         </is>
       </c>
-      <c r="C117" s="4" t="n"/>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Ajax url matches the file name case - broke on case-sensitive servers.</t>
+        </is>
+      </c>
       <c r="D117" s="4" t="n"/>
       <c r="E117" s="4" t="n"/>
       <c r="F117" s="4" t="n"/>
@@ -3080,7 +3144,11 @@
           <t>2026-10-13 | Send for approval (SALES_REPAIR V) and approve (SALES_REPAIR A) from Task Settings - were admin.</t>
         </is>
       </c>
-      <c r="C131" s="4" t="n"/>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Buttons checked against the repair's branch (company_id).</t>
+        </is>
+      </c>
       <c r="D131" s="4" t="n"/>
       <c r="E131" s="4" t="n"/>
       <c r="F131" s="4" t="n"/>
@@ -3135,7 +3203,11 @@
           <t>2026-10-13 | New. Settings &gt; Task Settings (admin only): add a task, tick the roles it uses, add many users per role with a branch or All, edit or deactivate a task; list shows who holds each role.</t>
         </is>
       </c>
-      <c r="C134" s="4" t="n"/>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Unknown user / branch ids refused; Item and Stock Location rows always All branches.</t>
+        </is>
+      </c>
       <c r="D134" s="4" t="n"/>
       <c r="E134" s="4" t="n"/>
       <c r="F134" s="4" t="n"/>
@@ -3173,7 +3245,11 @@
           <t>2026-10-13 | New. One definition per dashboard tile: task / role, waiting rule, branch column, page it opens; count and page share it.</t>
         </is>
       </c>
-      <c r="C136" s="4" t="n"/>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Sales repair tiles counted by the repair's branch.</t>
+        </is>
+      </c>
       <c r="D136" s="4" t="n"/>
       <c r="E136" s="4" t="n"/>
       <c r="F136" s="4" t="n"/>
@@ -3263,6 +3339,40 @@
       <c r="E141" s="4" t="n"/>
       <c r="F141" s="4" t="n"/>
       <c r="G141" s="4" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_delete_records.php</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | CRITICAL: login + csrf, only the 24 table / column pairs the delete links use, status forced to 0, id bound - it took table, column and value from the post with no login.</t>
+        </is>
+      </c>
+      <c r="C142" s="4" t="n"/>
+      <c r="D142" s="4" t="n"/>
+      <c r="E142" s="4" t="n"/>
+      <c r="F142" s="4" t="n"/>
+      <c r="G142" s="4" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>issue_salary.php</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13 | Csrf + salary approver for the employee's branch on the server - only the button was hidden.</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="n"/>
+      <c r="D143" s="4" t="n"/>
+      <c r="E143" s="4" t="n"/>
+      <c r="F143" s="4" t="n"/>
+      <c r="G143" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Invoice report: customer branch from cus_branch_id, not our branch_id
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G143"/>
+  <dimension ref="A1:G144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3373,6 +3373,23 @@
       <c r="E143" s="4" t="n"/>
       <c r="F143" s="4" t="n"/>
       <c r="G143" s="4" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>invoice_report.php</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14 | Customer branch read from cus_branch_id - it used branch_id (our branch), so every invoice showed customer branch 1 or 2, even for customers without a branch.</t>
+        </is>
+      </c>
+      <c r="C144" s="4" t="n"/>
+      <c r="D144" s="4" t="n"/>
+      <c r="E144" s="4" t="n"/>
+      <c r="F144" s="4" t="n"/>
+      <c r="G144" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Login check needs user and branch; item details popup needs a login (live error log)
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G144"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1809,7 +1809,11 @@
           <t>2026-10-07 | fnRowCount() added - posted row count, 0 for a missing or single value.</t>
         </is>
       </c>
-      <c r="C60" s="4" t="n"/>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14 | fnIsLoggedIn(); isAdmin also needs the user id and branch - a session with only _user=crm_user (another app on the server) opened pages with no user or branch.</t>
+        </is>
+      </c>
       <c r="D60" s="4" t="n"/>
       <c r="E60" s="4" t="n"/>
       <c r="F60" s="4" t="n"/>
@@ -3390,6 +3394,23 @@
       <c r="E144" s="4" t="n"/>
       <c r="F144" s="4" t="n"/>
       <c r="G144" s="4" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/modal_items_dets.php</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14 | Login needed - it answered without one (prices / stock) and logged sql errors for an empty branch.</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="n"/>
+      <c r="D145" s="4" t="n"/>
+      <c r="E145" s="4" t="n"/>
+      <c r="F145" s="4" t="n"/>
+      <c r="G145" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Revoke for a wrong approve / verify (Task Settings role R, admin only to begin with)
- Revoker role (R) on the 10 tasks with an approve / verify step; db/post_upload_151026.sql widens
  mst_task.task_roles, adds tbl_revoke_log, adds no user rows
- One revoke call (inc/cis_ajax/jquery_revoke.php) with per-form rules in inc/common/revoke.php:
  required state, blockers (GRN / sales order / DC / invoice / proforma / requote made on top),
  state it returns to, log row with old values and reason - all in one transaction
- Revoke button where approve / verify was: PO, quotation, sales order, DC, purchase return,
  sales repair (both steps), supplier, payment confirm / mark as credit, credit approval, salary issue
- Approve / verify never moves stock, so revoke never touches stock; it is refused once stock-moving
  documents exist on top
- EPF text file only takes issued salaries
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G145"/>
+  <dimension ref="A1:G150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1032,7 +1032,11 @@
           <t>2026-10-13 | Loads task_queues.php.</t>
         </is>
       </c>
-      <c r="F24" s="4" t="n"/>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Loads revoke.php.</t>
+        </is>
+      </c>
       <c r="G24" s="4" t="n"/>
     </row>
     <row r="25">
@@ -1323,7 +1327,11 @@
           <t>2026-10-13 | Mark as credit follows Sales Order in Accounts verifier - showed to every user (every user holds it to begin with).</t>
         </is>
       </c>
-      <c r="E36" s="4" t="n"/>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke payment confirm / mark as credit (SALES_RECEIPT R) - back to payment pending; revoke credit approval (CREDIT_SALES R) - back to credit requested. Each only before the next step is approved.</t>
+        </is>
+      </c>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
     </row>
@@ -1396,7 +1404,11 @@
           <t>2026-10-13 | Csrf token attached in $.ajaxPrefilter - pages passing their own beforeSend dropped the ajaxSetup hook, so their posts had no token.</t>
         </is>
       </c>
-      <c r="G39" s="4" t="n"/>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Loads js/revoke.js.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2247,7 +2259,11 @@
           <t>2026-10-13 | Approver from Task Settings (SUPPLIER A).</t>
         </is>
       </c>
-      <c r="D81" s="4" t="n"/>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke (SUPPLIER R) on an approved supplier - back to not approved; refused once used in a PO / GRN / return.</t>
+        </is>
+      </c>
       <c r="E81" s="4" t="n"/>
       <c r="F81" s="4" t="n"/>
       <c r="G81" s="4" t="n"/>
@@ -2306,7 +2322,11 @@
           <t>2026-10-13 | Issue button checked against the employee's branch.</t>
         </is>
       </c>
-      <c r="D84" s="4" t="n"/>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke next to Issued (SALARY R).</t>
+        </is>
+      </c>
       <c r="E84" s="4" t="n"/>
       <c r="F84" s="4" t="n"/>
       <c r="G84" s="4" t="n"/>
@@ -2327,7 +2347,11 @@
           <t>2026-10-13 | Issue button checked against the employee's branch.</t>
         </is>
       </c>
-      <c r="D85" s="4" t="n"/>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke next to Issued (SALARY R) - salary set to not issued, its accounts entry removed, Issue shows again.</t>
+        </is>
+      </c>
       <c r="E85" s="4" t="n"/>
       <c r="F85" s="4" t="n"/>
       <c r="G85" s="4" t="n"/>
@@ -2348,7 +2372,11 @@
           <t>2026-10-13 | Issue button checked against the employee's branch.</t>
         </is>
       </c>
-      <c r="D86" s="4" t="n"/>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke next to Issued (SALARY R).</t>
+        </is>
+      </c>
       <c r="E86" s="4" t="n"/>
       <c r="F86" s="4" t="n"/>
       <c r="G86" s="4" t="n"/>
@@ -2381,7 +2409,11 @@
           <t>2026-10-13 | Approve / reject for approvers in Task Settings (DC A) - was admin or the DC's branch.</t>
         </is>
       </c>
-      <c r="C88" s="4" t="n"/>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke (DC R) on an approved DC - back to draft; refused once invoiced.</t>
+        </is>
+      </c>
       <c r="D88" s="4" t="n"/>
       <c r="E88" s="4" t="n"/>
       <c r="F88" s="4" t="n"/>
@@ -2767,7 +2799,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (SALES_RECEIPT W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C110" s="4" t="n"/>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke next to a confirmed payment (SALES_RECEIPT R).</t>
+        </is>
+      </c>
       <c r="D110" s="4" t="n"/>
       <c r="E110" s="4" t="n"/>
       <c r="F110" s="4" t="n"/>
@@ -2827,7 +2863,11 @@
           <t>2026-10-13 | Tile mode: pending suppliers of the user's approver branches; status filter cast to int.</t>
         </is>
       </c>
-      <c r="D113" s="4" t="n"/>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Approve page link also for Revokers on approved suppliers.</t>
+        </is>
+      </c>
       <c r="E113" s="4" t="n"/>
       <c r="F113" s="4" t="n"/>
       <c r="G113" s="4" t="n"/>
@@ -3042,7 +3082,11 @@
           <t>2026-10-13 | Approve / reject for approvers in Task Settings (PURCHASE_ORDER A) - was admin.</t>
         </is>
       </c>
-      <c r="C125" s="4" t="n"/>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke for Revokers (PURCHASE_ORDER R) on an approved PO - back to draft; refused once a GRN is made. Last revoke shown.</t>
+        </is>
+      </c>
       <c r="D125" s="4" t="n"/>
       <c r="E125" s="4" t="n"/>
       <c r="F125" s="4" t="n"/>
@@ -3059,7 +3103,11 @@
           <t>2026-10-13 | Approve / reject for approvers in Task Settings (QUOTATION A) - was admin or the quotation's branch.</t>
         </is>
       </c>
-      <c r="C126" s="4" t="n"/>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke (QUOTATION R) on an approved quotation - back to draft; refused once a sales order / invoice / proforma / requote is made.</t>
+        </is>
+      </c>
       <c r="D126" s="4" t="n"/>
       <c r="E126" s="4" t="n"/>
       <c r="F126" s="4" t="n"/>
@@ -3081,7 +3129,11 @@
           <t>2026-10-13 | Approve / reject buttons follow Sales Order approver - they showed to every user (every user holds it to begin with).</t>
         </is>
       </c>
-      <c r="D127" s="4" t="n"/>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke (SALES_ORDER R) on an approved sales order - back to in approval (credit sales back to credit approved); refused once a DC / invoice is made.</t>
+        </is>
+      </c>
       <c r="E127" s="4" t="n"/>
       <c r="F127" s="4" t="n"/>
       <c r="G127" s="4" t="n"/>
@@ -3114,7 +3166,11 @@
           <t>2026-10-13 | Approve / reject only for approvers in Task Settings (PURCHASE_RETURN A) - was anyone opening the page.</t>
         </is>
       </c>
-      <c r="C129" s="4" t="n"/>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke (PURCHASE_RETURN R) on an approved return - back to draft (a rejected return cannot be edited).</t>
+        </is>
+      </c>
       <c r="D129" s="4" t="n"/>
       <c r="E129" s="4" t="n"/>
       <c r="F129" s="4" t="n"/>
@@ -3153,7 +3209,11 @@
           <t>2026-10-13 | Buttons checked against the repair's branch (company_id).</t>
         </is>
       </c>
-      <c r="D131" s="4" t="n"/>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoke under send for approval (back to draft) and approve (back to in approval) - SALES_REPAIR R.</t>
+        </is>
+      </c>
       <c r="E131" s="4" t="n"/>
       <c r="F131" s="4" t="n"/>
       <c r="G131" s="4" t="n"/>
@@ -3212,7 +3272,11 @@
           <t>2026-10-13 | Unknown user / branch ids refused; Item and Stock Location rows always All branches.</t>
         </is>
       </c>
-      <c r="D134" s="4" t="n"/>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | Revoker role (R) - role tick, user rows and a Revoker column on the list.</t>
+        </is>
+      </c>
       <c r="E134" s="4" t="n"/>
       <c r="F134" s="4" t="n"/>
       <c r="G134" s="4" t="n"/>
@@ -3411,6 +3475,91 @@
       <c r="E145" s="4" t="n"/>
       <c r="F145" s="4" t="n"/>
       <c r="G145" s="4" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>db/post_upload_151026.sql</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | New. Revoker role (R) on 10 tasks - mst_task.task_roles widened to 10, notes extended; new table tbl_revoke_log. No user rows: admin only until Revokers are given in Task Settings. Run after post_upload_131026.sql. Safe to run again.</t>
+        </is>
+      </c>
+      <c r="C146" s="4" t="n"/>
+      <c r="D146" s="4" t="n"/>
+      <c r="E146" s="4" t="n"/>
+      <c r="F146" s="4" t="n"/>
+      <c r="G146" s="4" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>inc/common/revoke.php</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | New. One entry per form: state it must be in, what blocks it (GRN / sales order / DC / invoice / proforma / requote made on top), state it goes back to. Revoke + log in one transaction, button and last-revoke note helpers.</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="n"/>
+      <c r="D147" s="4" t="n"/>
+      <c r="E147" s="4" t="n"/>
+      <c r="F147" s="4" t="n"/>
+      <c r="G147" s="4" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_revoke.php</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | New. The revoke call for every form - login, csrf, Revoker for the document's branch, reason needed; 409 with the reason when refused.</t>
+        </is>
+      </c>
+      <c r="C148" s="4" t="n"/>
+      <c r="D148" s="4" t="n"/>
+      <c r="E148" s="4" t="n"/>
+      <c r="F148" s="4" t="n"/>
+      <c r="G148" s="4" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>js/revoke.js</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | New. Revoke button: asks the reason, calls the revoke, reloads or shows why it was refused.</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="n"/>
+      <c r="D149" s="4" t="n"/>
+      <c r="E149" s="4" t="n"/>
+      <c r="F149" s="4" t="n"/>
+      <c r="G149" s="4" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>attendance_report_epf_txt.php</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | EPF text file only takes issued salaries - a revoked one stays in the table with status 0.</t>
+        </is>
+      </c>
+      <c r="C150" s="4" t="n"/>
+      <c r="D150" s="4" t="n"/>
+      <c r="E150" s="4" t="n"/>
+      <c r="F150" s="4" t="n"/>
+      <c r="G150" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3423,7 +3572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3519,7 +3668,11 @@
           <t>2026-10-13 | (new table) | One row per task: code checked by the screens, name, module, roles used (C V A W), note, status.</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | task_roles | VARCHAR(4) widened to VARCHAR(10); R (Revoker) added to PURCHASE_ORDER, SUPPLIER, PURCHASE_RETURN, QUOTATION, SALES_ORDER, CREDIT_SALES, DC, SALES_RECEIPT, SALES_REPAIR, SALARY.</t>
+        </is>
+      </c>
       <c r="D2" s="4" t="n"/>
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
@@ -3547,7 +3700,11 @@
           <t>2026-10-13 | (rows) | Sales order approver and payment verifier: every user (head office all branches, others own branch). New task SO_CANCEL for cancel (admin).</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | task_role | New value R (Revoker). No rows added - admin only to begin with.</t>
+        </is>
+      </c>
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
@@ -4156,6 +4313,75 @@
       <c r="L25" s="4" t="n"/>
       <c r="M25" s="4" t="n"/>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>tbl_revoke_log</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | (new table) | One row per revoke: form, task, document id / ref, branch, old values (json), reason, who, when.</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="4" t="n"/>
+      <c r="J26" s="4" t="n"/>
+      <c r="K26" s="4" t="n"/>
+      <c r="L26" s="4" t="n"/>
+      <c r="M26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>tbl_emp_monthly_salary</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | salary_status | Revoke sets 0 (not issued); the reports already count only 1, the EPF text file now too.</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
+      <c r="J27" s="4" t="n"/>
+      <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="n"/>
+      <c r="M27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>tbl_accounts</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | (rows) | Revoking a salary deletes its entry (emp_sal_id).</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="n"/>
+      <c r="M28" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
SPAC items: item discount 28% to 30% - cost price and margin per branch, price history rows (db/spac_discount_30_151026.sql)
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G150"/>
+  <dimension ref="A1:G151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3530,12 +3530,12 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>js/revoke.js</t>
+          <t>db/spac_discount_30_151026.sql</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15 | New. Revoke button: asks the reason, calls the revoke, reloads or shows why it was refused.</t>
+          <t>2026-10-15 | New. SPAC items discount 28% -&gt; 30%: cost price and margin per branch and in the item master, item / selling price unchanged, price history row per item per branch. Safe to run again.</t>
         </is>
       </c>
       <c r="C149" s="4" t="n"/>
@@ -3547,12 +3547,12 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>attendance_report_epf_txt.php</t>
+          <t>js/revoke.js</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15 | EPF text file only takes issued salaries - a revoked one stays in the table with status 0.</t>
+          <t>2026-10-15 | New. Revoke button: asks the reason, calls the revoke, reloads or shows why it was refused.</t>
         </is>
       </c>
       <c r="C150" s="4" t="n"/>
@@ -3560,6 +3560,23 @@
       <c r="E150" s="4" t="n"/>
       <c r="F150" s="4" t="n"/>
       <c r="G150" s="4" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>attendance_report_epf_txt.php</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | EPF text file only takes issued salaries - a revoked one stays in the table with status 0.</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="n"/>
+      <c r="D151" s="4" t="n"/>
+      <c r="E151" s="4" t="n"/>
+      <c r="F151" s="4" t="n"/>
+      <c r="G151" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3572,7 +3589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4316,12 +4333,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>tbl_revoke_log</t>
+          <t>tbl_itemprice_history</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15 | (new table) | One row per revoke: form, task, document id / ref, branch, old values (json), reason, who, when.</t>
+          <t>2026-10-15 | (rows) | One per SPAC item per branch for the 28% -&gt; 30% discount change.</t>
         </is>
       </c>
       <c r="C26" s="4" t="n"/>
@@ -4339,12 +4356,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>tbl_emp_monthly_salary</t>
+          <t>tbl_revoke_log</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15 | salary_status | Revoke sets 0 (not issued); the reports already count only 1, the EPF text file now too.</t>
+          <t>2026-10-15 | (new table) | One row per revoke: form, task, document id / ref, branch, old values (json), reason, who, when.</t>
         </is>
       </c>
       <c r="C27" s="4" t="n"/>
@@ -4362,12 +4379,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>tbl_accounts</t>
+          <t>tbl_item_stock / tbl_item_details (SPAC)</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15 | (rows) | Revoking a salary deletes its entry (emp_sal_id).</t>
+          <t>2026-10-15 | (rows) | SPAC items: discount 30, cost price and margin recalculated; item and selling price unchanged.</t>
         </is>
       </c>
       <c r="C28" s="4" t="n"/>
@@ -4382,6 +4399,52 @@
       <c r="L28" s="4" t="n"/>
       <c r="M28" s="4" t="n"/>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>tbl_emp_monthly_salary</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | salary_status | Revoke sets 0 (not issued); the reports already count only 1, the EPF text file now too.</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="n"/>
+      <c r="J29" s="4" t="n"/>
+      <c r="K29" s="4" t="n"/>
+      <c r="L29" s="4" t="n"/>
+      <c r="M29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>tbl_accounts</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15 | (rows) | Revoking a salary deletes its entry (emp_sal_id).</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="n"/>
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
+      <c r="J30" s="4" t="n"/>
+      <c r="K30" s="4" t="n"/>
+      <c r="L30" s="4" t="n"/>
+      <c r="M30" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Item prices: margin on cost everywhere, Bulk Discount / Margin and Item Price Update screens
- js/price_calc.js: cost = price less discount, margin % on cost; selling changes only from margin or
  selling. Used by the item form, Item Price History (was margin on item price) and the new screens
- Item Masters > Bulk Discount / Margin: filter by principal / brand / division / item type, branches,
  one discount or margin % for all listed rows, remove rows, one save (set-based, history per row)
- Item Masters > Item Price Update: one branch, price / discount / margin / selling boxes, save per row
- Both for Item creators (ITEM C) or admin; Head Office values copied to the item master
- db/post_upload_161026.sql: menus + rights, index on tbl_item_stock.item_id (10,740-row save 145 s ->
  0.7 s), stored margins recalculated on cost
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G151"/>
+  <dimension ref="A1:H158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -473,6 +473,7 @@
     <col width="62" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
     <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -509,6 +510,11 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Change 6</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Change 7</t>
         </is>
       </c>
     </row>
@@ -528,6 +534,7 @@
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -549,6 +556,7 @@
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -566,6 +574,7 @@
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="4" t="n"/>
       <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -587,6 +596,7 @@
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -616,6 +626,7 @@
       </c>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -649,6 +660,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -682,6 +694,7 @@
         </is>
       </c>
       <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -715,6 +728,7 @@
         </is>
       </c>
       <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -752,6 +766,11 @@
           <t>2026-10-13 | updated_by from _user_id (was empty).</t>
         </is>
       </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | Margin on cost (was on item price), branch and multi-UOM rows; price / discount no longer rewrite the selling price; loaded margin shown on cost.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -784,7 +803,12 @@
           <t>2026-10-13 | Price block check uses Task Settings (ITEM C) - was user 1; both branches show it.</t>
         </is>
       </c>
-      <c r="G11" s="4" t="n"/>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | Price fields use js/price_calc.js - price / discount no longer rewrite the selling price.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -802,6 +826,7 @@
       <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -819,6 +844,7 @@
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -840,6 +866,7 @@
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -857,6 +884,7 @@
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
       <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -874,6 +902,7 @@
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -899,6 +928,7 @@
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
+      <c r="H17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -916,6 +946,7 @@
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -933,6 +964,7 @@
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -950,6 +982,7 @@
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -967,6 +1000,7 @@
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
       <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -984,6 +1018,7 @@
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
       <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1005,6 +1040,7 @@
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
       <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1038,6 +1074,7 @@
         </is>
       </c>
       <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1059,6 +1096,7 @@
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1088,6 +1126,7 @@
       </c>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1113,6 +1152,7 @@
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
       <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1146,6 +1186,7 @@
         </is>
       </c>
       <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1171,6 +1212,7 @@
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
       <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1200,6 +1242,7 @@
       </c>
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1229,6 +1272,7 @@
       </c>
       <c r="F31" s="4" t="n"/>
       <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1250,6 +1294,7 @@
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
       <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1271,6 +1316,7 @@
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
       <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1288,6 +1334,7 @@
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
       <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1305,6 +1352,7 @@
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
       <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1334,6 +1382,7 @@
       </c>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1355,6 +1404,7 @@
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="n"/>
       <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1372,6 +1422,7 @@
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="n"/>
       <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1407,6 +1458,11 @@
       <c r="G39" s="3" t="inlineStr">
         <is>
           <t>2026-10-15 | Loads js/revoke.js.</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | Loads js/price_calc.js.</t>
         </is>
       </c>
     </row>
@@ -1426,6 +1482,7 @@
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
       <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1443,6 +1500,7 @@
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="4" t="n"/>
       <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1460,6 +1518,7 @@
       <c r="E42" s="4" t="n"/>
       <c r="F42" s="4" t="n"/>
       <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1481,6 +1540,7 @@
       <c r="E43" s="4" t="n"/>
       <c r="F43" s="4" t="n"/>
       <c r="G43" s="4" t="n"/>
+      <c r="H43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1498,6 +1558,7 @@
       <c r="E44" s="4" t="n"/>
       <c r="F44" s="4" t="n"/>
       <c r="G44" s="4" t="n"/>
+      <c r="H44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1519,6 +1580,7 @@
       <c r="E45" s="4" t="n"/>
       <c r="F45" s="4" t="n"/>
       <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1536,6 +1598,7 @@
       <c r="E46" s="4" t="n"/>
       <c r="F46" s="4" t="n"/>
       <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1553,6 +1616,7 @@
       <c r="E47" s="4" t="n"/>
       <c r="F47" s="4" t="n"/>
       <c r="G47" s="4" t="n"/>
+      <c r="H47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1570,6 +1634,7 @@
       <c r="E48" s="4" t="n"/>
       <c r="F48" s="4" t="n"/>
       <c r="G48" s="4" t="n"/>
+      <c r="H48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1591,6 +1656,7 @@
       <c r="E49" s="4" t="n"/>
       <c r="F49" s="4" t="n"/>
       <c r="G49" s="4" t="n"/>
+      <c r="H49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1608,6 +1674,7 @@
       <c r="E50" s="4" t="n"/>
       <c r="F50" s="4" t="n"/>
       <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1629,6 +1696,7 @@
       <c r="E51" s="4" t="n"/>
       <c r="F51" s="4" t="n"/>
       <c r="G51" s="4" t="n"/>
+      <c r="H51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1646,6 +1714,7 @@
       <c r="E52" s="4" t="n"/>
       <c r="F52" s="4" t="n"/>
       <c r="G52" s="4" t="n"/>
+      <c r="H52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1675,6 +1744,7 @@
       </c>
       <c r="F53" s="4" t="n"/>
       <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1692,6 +1762,7 @@
       <c r="E54" s="4" t="n"/>
       <c r="F54" s="4" t="n"/>
       <c r="G54" s="4" t="n"/>
+      <c r="H54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1709,6 +1780,7 @@
       <c r="E55" s="4" t="n"/>
       <c r="F55" s="4" t="n"/>
       <c r="G55" s="4" t="n"/>
+      <c r="H55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1738,6 +1810,7 @@
       </c>
       <c r="F56" s="4" t="n"/>
       <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1767,6 +1840,7 @@
       </c>
       <c r="F57" s="4" t="n"/>
       <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1792,6 +1866,7 @@
       <c r="E58" s="4" t="n"/>
       <c r="F58" s="4" t="n"/>
       <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1809,6 +1884,7 @@
       <c r="E59" s="4" t="n"/>
       <c r="F59" s="4" t="n"/>
       <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1830,6 +1906,7 @@
       <c r="E60" s="4" t="n"/>
       <c r="F60" s="4" t="n"/>
       <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1847,6 +1924,7 @@
       <c r="E61" s="4" t="n"/>
       <c r="F61" s="4" t="n"/>
       <c r="G61" s="4" t="n"/>
+      <c r="H61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1864,6 +1942,7 @@
       <c r="E62" s="4" t="n"/>
       <c r="F62" s="4" t="n"/>
       <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1881,6 +1960,7 @@
       <c r="E63" s="4" t="n"/>
       <c r="F63" s="4" t="n"/>
       <c r="G63" s="4" t="n"/>
+      <c r="H63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1898,6 +1978,7 @@
       <c r="E64" s="4" t="n"/>
       <c r="F64" s="4" t="n"/>
       <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1915,6 +1996,7 @@
       <c r="E65" s="4" t="n"/>
       <c r="F65" s="4" t="n"/>
       <c r="G65" s="4" t="n"/>
+      <c r="H65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1932,6 +2014,7 @@
       <c r="E66" s="4" t="n"/>
       <c r="F66" s="4" t="n"/>
       <c r="G66" s="4" t="n"/>
+      <c r="H66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1949,6 +2032,7 @@
       <c r="E67" s="4" t="n"/>
       <c r="F67" s="4" t="n"/>
       <c r="G67" s="4" t="n"/>
+      <c r="H67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1970,6 +2054,7 @@
       <c r="E68" s="4" t="n"/>
       <c r="F68" s="4" t="n"/>
       <c r="G68" s="4" t="n"/>
+      <c r="H68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1987,6 +2072,7 @@
       <c r="E69" s="4" t="n"/>
       <c r="F69" s="4" t="n"/>
       <c r="G69" s="4" t="n"/>
+      <c r="H69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2004,6 +2090,7 @@
       <c r="E70" s="4" t="n"/>
       <c r="F70" s="4" t="n"/>
       <c r="G70" s="4" t="n"/>
+      <c r="H70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2021,6 +2108,7 @@
       <c r="E71" s="4" t="n"/>
       <c r="F71" s="4" t="n"/>
       <c r="G71" s="4" t="n"/>
+      <c r="H71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2050,6 +2138,7 @@
       </c>
       <c r="F72" s="4" t="n"/>
       <c r="G72" s="4" t="n"/>
+      <c r="H72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2075,6 +2164,7 @@
       <c r="E73" s="4" t="n"/>
       <c r="F73" s="4" t="n"/>
       <c r="G73" s="4" t="n"/>
+      <c r="H73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2100,6 +2190,7 @@
       <c r="E74" s="4" t="n"/>
       <c r="F74" s="4" t="n"/>
       <c r="G74" s="4" t="n"/>
+      <c r="H74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2125,6 +2216,7 @@
       <c r="E75" s="4" t="n"/>
       <c r="F75" s="4" t="n"/>
       <c r="G75" s="4" t="n"/>
+      <c r="H75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2150,6 +2242,7 @@
       <c r="E76" s="4" t="n"/>
       <c r="F76" s="4" t="n"/>
       <c r="G76" s="4" t="n"/>
+      <c r="H76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2175,6 +2268,7 @@
       <c r="E77" s="4" t="n"/>
       <c r="F77" s="4" t="n"/>
       <c r="G77" s="4" t="n"/>
+      <c r="H77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2200,6 +2294,7 @@
       <c r="E78" s="4" t="n"/>
       <c r="F78" s="4" t="n"/>
       <c r="G78" s="4" t="n"/>
+      <c r="H78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2221,6 +2316,7 @@
       <c r="E79" s="4" t="n"/>
       <c r="F79" s="4" t="n"/>
       <c r="G79" s="4" t="n"/>
+      <c r="H79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2242,6 +2338,7 @@
       <c r="E80" s="4" t="n"/>
       <c r="F80" s="4" t="n"/>
       <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2267,6 +2364,7 @@
       <c r="E81" s="4" t="n"/>
       <c r="F81" s="4" t="n"/>
       <c r="G81" s="4" t="n"/>
+      <c r="H81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2288,6 +2386,7 @@
       <c r="E82" s="4" t="n"/>
       <c r="F82" s="4" t="n"/>
       <c r="G82" s="4" t="n"/>
+      <c r="H82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -2305,6 +2404,7 @@
       <c r="E83" s="4" t="n"/>
       <c r="F83" s="4" t="n"/>
       <c r="G83" s="4" t="n"/>
+      <c r="H83" s="4" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2330,6 +2430,7 @@
       <c r="E84" s="4" t="n"/>
       <c r="F84" s="4" t="n"/>
       <c r="G84" s="4" t="n"/>
+      <c r="H84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -2355,6 +2456,7 @@
       <c r="E85" s="4" t="n"/>
       <c r="F85" s="4" t="n"/>
       <c r="G85" s="4" t="n"/>
+      <c r="H85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2380,6 +2482,7 @@
       <c r="E86" s="4" t="n"/>
       <c r="F86" s="4" t="n"/>
       <c r="G86" s="4" t="n"/>
+      <c r="H86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -2397,6 +2500,7 @@
       <c r="E87" s="4" t="n"/>
       <c r="F87" s="4" t="n"/>
       <c r="G87" s="4" t="n"/>
+      <c r="H87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2418,6 +2522,7 @@
       <c r="E88" s="4" t="n"/>
       <c r="F88" s="4" t="n"/>
       <c r="G88" s="4" t="n"/>
+      <c r="H88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -2435,6 +2540,7 @@
       <c r="E89" s="4" t="n"/>
       <c r="F89" s="4" t="n"/>
       <c r="G89" s="4" t="n"/>
+      <c r="H89" s="4" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -2452,6 +2558,7 @@
       <c r="E90" s="4" t="n"/>
       <c r="F90" s="4" t="n"/>
       <c r="G90" s="4" t="n"/>
+      <c r="H90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -2469,6 +2576,7 @@
       <c r="E91" s="4" t="n"/>
       <c r="F91" s="4" t="n"/>
       <c r="G91" s="4" t="n"/>
+      <c r="H91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -2486,6 +2594,7 @@
       <c r="E92" s="4" t="n"/>
       <c r="F92" s="4" t="n"/>
       <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2503,6 +2612,7 @@
       <c r="E93" s="4" t="n"/>
       <c r="F93" s="4" t="n"/>
       <c r="G93" s="4" t="n"/>
+      <c r="H93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -2528,6 +2638,7 @@
       <c r="E94" s="4" t="n"/>
       <c r="F94" s="4" t="n"/>
       <c r="G94" s="4" t="n"/>
+      <c r="H94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -2545,6 +2656,7 @@
       <c r="E95" s="4" t="n"/>
       <c r="F95" s="4" t="n"/>
       <c r="G95" s="4" t="n"/>
+      <c r="H95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -2562,6 +2674,7 @@
       <c r="E96" s="4" t="n"/>
       <c r="F96" s="4" t="n"/>
       <c r="G96" s="4" t="n"/>
+      <c r="H96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2579,6 +2692,7 @@
       <c r="E97" s="4" t="n"/>
       <c r="F97" s="4" t="n"/>
       <c r="G97" s="4" t="n"/>
+      <c r="H97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2596,6 +2710,7 @@
       <c r="E98" s="4" t="n"/>
       <c r="F98" s="4" t="n"/>
       <c r="G98" s="4" t="n"/>
+      <c r="H98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -2617,6 +2732,7 @@
       <c r="E99" s="4" t="n"/>
       <c r="F99" s="4" t="n"/>
       <c r="G99" s="4" t="n"/>
+      <c r="H99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -2634,6 +2750,7 @@
       <c r="E100" s="4" t="n"/>
       <c r="F100" s="4" t="n"/>
       <c r="G100" s="4" t="n"/>
+      <c r="H100" s="4" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -2651,6 +2768,7 @@
       <c r="E101" s="4" t="n"/>
       <c r="F101" s="4" t="n"/>
       <c r="G101" s="4" t="n"/>
+      <c r="H101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -2668,6 +2786,7 @@
       <c r="E102" s="4" t="n"/>
       <c r="F102" s="4" t="n"/>
       <c r="G102" s="4" t="n"/>
+      <c r="H102" s="4" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -2685,6 +2804,7 @@
       <c r="E103" s="4" t="n"/>
       <c r="F103" s="4" t="n"/>
       <c r="G103" s="4" t="n"/>
+      <c r="H103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -2702,6 +2822,7 @@
       <c r="E104" s="4" t="n"/>
       <c r="F104" s="4" t="n"/>
       <c r="G104" s="4" t="n"/>
+      <c r="H104" s="4" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -2719,6 +2840,7 @@
       <c r="E105" s="4" t="n"/>
       <c r="F105" s="4" t="n"/>
       <c r="G105" s="4" t="n"/>
+      <c r="H105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -2736,6 +2858,7 @@
       <c r="E106" s="4" t="n"/>
       <c r="F106" s="4" t="n"/>
       <c r="G106" s="4" t="n"/>
+      <c r="H106" s="4" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -2753,6 +2876,7 @@
       <c r="E107" s="4" t="n"/>
       <c r="F107" s="4" t="n"/>
       <c r="G107" s="4" t="n"/>
+      <c r="H107" s="4" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -2770,6 +2894,7 @@
       <c r="E108" s="4" t="n"/>
       <c r="F108" s="4" t="n"/>
       <c r="G108" s="4" t="n"/>
+      <c r="H108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -2787,6 +2912,7 @@
       <c r="E109" s="4" t="n"/>
       <c r="F109" s="4" t="n"/>
       <c r="G109" s="4" t="n"/>
+      <c r="H109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -2808,6 +2934,7 @@
       <c r="E110" s="4" t="n"/>
       <c r="F110" s="4" t="n"/>
       <c r="G110" s="4" t="n"/>
+      <c r="H110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -2829,6 +2956,7 @@
       <c r="E111" s="4" t="n"/>
       <c r="F111" s="4" t="n"/>
       <c r="G111" s="4" t="n"/>
+      <c r="H111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -2846,6 +2974,7 @@
       <c r="E112" s="4" t="n"/>
       <c r="F112" s="4" t="n"/>
       <c r="G112" s="4" t="n"/>
+      <c r="H112" s="4" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -2871,6 +3000,7 @@
       <c r="E113" s="4" t="n"/>
       <c r="F113" s="4" t="n"/>
       <c r="G113" s="4" t="n"/>
+      <c r="H113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -2888,6 +3018,7 @@
       <c r="E114" s="4" t="n"/>
       <c r="F114" s="4" t="n"/>
       <c r="G114" s="4" t="n"/>
+      <c r="H114" s="4" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -2905,6 +3036,7 @@
       <c r="E115" s="4" t="n"/>
       <c r="F115" s="4" t="n"/>
       <c r="G115" s="4" t="n"/>
+      <c r="H115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -2922,6 +3054,7 @@
       <c r="E116" s="4" t="n"/>
       <c r="F116" s="4" t="n"/>
       <c r="G116" s="4" t="n"/>
+      <c r="H116" s="4" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -2943,6 +3076,7 @@
       <c r="E117" s="4" t="n"/>
       <c r="F117" s="4" t="n"/>
       <c r="G117" s="4" t="n"/>
+      <c r="H117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -2960,6 +3094,7 @@
       <c r="E118" s="4" t="n"/>
       <c r="F118" s="4" t="n"/>
       <c r="G118" s="4" t="n"/>
+      <c r="H118" s="4" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -2977,6 +3112,7 @@
       <c r="E119" s="4" t="n"/>
       <c r="F119" s="4" t="n"/>
       <c r="G119" s="4" t="n"/>
+      <c r="H119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -2994,6 +3130,7 @@
       <c r="E120" s="4" t="n"/>
       <c r="F120" s="4" t="n"/>
       <c r="G120" s="4" t="n"/>
+      <c r="H120" s="4" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -3011,6 +3148,7 @@
       <c r="E121" s="4" t="n"/>
       <c r="F121" s="4" t="n"/>
       <c r="G121" s="4" t="n"/>
+      <c r="H121" s="4" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -3028,6 +3166,7 @@
       <c r="E122" s="4" t="n"/>
       <c r="F122" s="4" t="n"/>
       <c r="G122" s="4" t="n"/>
+      <c r="H122" s="4" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -3053,6 +3192,7 @@
       <c r="E123" s="4" t="n"/>
       <c r="F123" s="4" t="n"/>
       <c r="G123" s="4" t="n"/>
+      <c r="H123" s="4" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -3070,6 +3210,7 @@
       <c r="E124" s="4" t="n"/>
       <c r="F124" s="4" t="n"/>
       <c r="G124" s="4" t="n"/>
+      <c r="H124" s="4" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -3091,6 +3232,7 @@
       <c r="E125" s="4" t="n"/>
       <c r="F125" s="4" t="n"/>
       <c r="G125" s="4" t="n"/>
+      <c r="H125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -3112,6 +3254,7 @@
       <c r="E126" s="4" t="n"/>
       <c r="F126" s="4" t="n"/>
       <c r="G126" s="4" t="n"/>
+      <c r="H126" s="4" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -3137,6 +3280,7 @@
       <c r="E127" s="4" t="n"/>
       <c r="F127" s="4" t="n"/>
       <c r="G127" s="4" t="n"/>
+      <c r="H127" s="4" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -3154,6 +3298,7 @@
       <c r="E128" s="4" t="n"/>
       <c r="F128" s="4" t="n"/>
       <c r="G128" s="4" t="n"/>
+      <c r="H128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -3175,6 +3320,7 @@
       <c r="E129" s="4" t="n"/>
       <c r="F129" s="4" t="n"/>
       <c r="G129" s="4" t="n"/>
+      <c r="H129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -3192,6 +3338,7 @@
       <c r="E130" s="4" t="n"/>
       <c r="F130" s="4" t="n"/>
       <c r="G130" s="4" t="n"/>
+      <c r="H130" s="4" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -3217,6 +3364,7 @@
       <c r="E131" s="4" t="n"/>
       <c r="F131" s="4" t="n"/>
       <c r="G131" s="4" t="n"/>
+      <c r="H131" s="4" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -3234,6 +3382,7 @@
       <c r="E132" s="4" t="n"/>
       <c r="F132" s="4" t="n"/>
       <c r="G132" s="4" t="n"/>
+      <c r="H132" s="4" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -3255,6 +3404,7 @@
       <c r="E133" s="4" t="n"/>
       <c r="F133" s="4" t="n"/>
       <c r="G133" s="4" t="n"/>
+      <c r="H133" s="4" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -3280,6 +3430,7 @@
       <c r="E134" s="4" t="n"/>
       <c r="F134" s="4" t="n"/>
       <c r="G134" s="4" t="n"/>
+      <c r="H134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -3301,6 +3452,7 @@
       <c r="E135" s="4" t="n"/>
       <c r="F135" s="4" t="n"/>
       <c r="G135" s="4" t="n"/>
+      <c r="H135" s="4" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -3322,6 +3474,7 @@
       <c r="E136" s="4" t="n"/>
       <c r="F136" s="4" t="n"/>
       <c r="G136" s="4" t="n"/>
+      <c r="H136" s="4" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -3339,6 +3492,7 @@
       <c r="E137" s="4" t="n"/>
       <c r="F137" s="4" t="n"/>
       <c r="G137" s="4" t="n"/>
+      <c r="H137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -3356,6 +3510,7 @@
       <c r="E138" s="4" t="n"/>
       <c r="F138" s="4" t="n"/>
       <c r="G138" s="4" t="n"/>
+      <c r="H138" s="4" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -3373,6 +3528,7 @@
       <c r="E139" s="4" t="n"/>
       <c r="F139" s="4" t="n"/>
       <c r="G139" s="4" t="n"/>
+      <c r="H139" s="4" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -3390,6 +3546,7 @@
       <c r="E140" s="4" t="n"/>
       <c r="F140" s="4" t="n"/>
       <c r="G140" s="4" t="n"/>
+      <c r="H140" s="4" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -3407,6 +3564,7 @@
       <c r="E141" s="4" t="n"/>
       <c r="F141" s="4" t="n"/>
       <c r="G141" s="4" t="n"/>
+      <c r="H141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -3424,6 +3582,7 @@
       <c r="E142" s="4" t="n"/>
       <c r="F142" s="4" t="n"/>
       <c r="G142" s="4" t="n"/>
+      <c r="H142" s="4" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -3441,6 +3600,7 @@
       <c r="E143" s="4" t="n"/>
       <c r="F143" s="4" t="n"/>
       <c r="G143" s="4" t="n"/>
+      <c r="H143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -3458,6 +3618,7 @@
       <c r="E144" s="4" t="n"/>
       <c r="F144" s="4" t="n"/>
       <c r="G144" s="4" t="n"/>
+      <c r="H144" s="4" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -3475,6 +3636,7 @@
       <c r="E145" s="4" t="n"/>
       <c r="F145" s="4" t="n"/>
       <c r="G145" s="4" t="n"/>
+      <c r="H145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -3492,6 +3654,7 @@
       <c r="E146" s="4" t="n"/>
       <c r="F146" s="4" t="n"/>
       <c r="G146" s="4" t="n"/>
+      <c r="H146" s="4" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -3509,6 +3672,7 @@
       <c r="E147" s="4" t="n"/>
       <c r="F147" s="4" t="n"/>
       <c r="G147" s="4" t="n"/>
+      <c r="H147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -3526,6 +3690,7 @@
       <c r="E148" s="4" t="n"/>
       <c r="F148" s="4" t="n"/>
       <c r="G148" s="4" t="n"/>
+      <c r="H148" s="4" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -3543,6 +3708,7 @@
       <c r="E149" s="4" t="n"/>
       <c r="F149" s="4" t="n"/>
       <c r="G149" s="4" t="n"/>
+      <c r="H149" s="4" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -3560,6 +3726,7 @@
       <c r="E150" s="4" t="n"/>
       <c r="F150" s="4" t="n"/>
       <c r="G150" s="4" t="n"/>
+      <c r="H150" s="4" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -3577,6 +3744,133 @@
       <c r="E151" s="4" t="n"/>
       <c r="F151" s="4" t="n"/>
       <c r="G151" s="4" t="n"/>
+      <c r="H151" s="4" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>js/price_calc.js</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | New. One price rule for every screen: cost = price less discount, margin % on cost; selling changes only from margin or selling.</t>
+        </is>
+      </c>
+      <c r="C152" s="4" t="n"/>
+      <c r="D152" s="4" t="n"/>
+      <c r="E152" s="4" t="n"/>
+      <c r="F152" s="4" t="n"/>
+      <c r="G152" s="4" t="n"/>
+      <c r="H152" s="4" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>item_bulk_discount.php</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | New screen Item Masters &gt; Bulk Discount / Margin - one discount or margin % for a filtered item set in chosen branches, one save, history per row.</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="n"/>
+      <c r="D153" s="4" t="n"/>
+      <c r="E153" s="4" t="n"/>
+      <c r="F153" s="4" t="n"/>
+      <c r="G153" s="4" t="n"/>
+      <c r="H153" s="4" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>item_price_list.php</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | New screen Item Masters &gt; Item Price Update - filtered list of one branch, price / discount / margin / selling boxes, save per row.</t>
+        </is>
+      </c>
+      <c r="C154" s="4" t="n"/>
+      <c r="D154" s="4" t="n"/>
+      <c r="E154" s="4" t="n"/>
+      <c r="F154" s="4" t="n"/>
+      <c r="G154" s="4" t="n"/>
+      <c r="H154" s="4" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>inc/common/item_price_filters.php</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | New. Principal / brand / division / item type / search filters shared by the two screens.</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="n"/>
+      <c r="D155" s="4" t="n"/>
+      <c r="E155" s="4" t="n"/>
+      <c r="F155" s="4" t="n"/>
+      <c r="G155" s="4" t="n"/>
+      <c r="H155" s="4" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>inc/common/item_price.php</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | New. Price list, one-row save and set-based bulk save per branch; history rows; Head Office copied to the item master.</t>
+        </is>
+      </c>
+      <c r="C156" s="4" t="n"/>
+      <c r="D156" s="4" t="n"/>
+      <c r="E156" s="4" t="n"/>
+      <c r="F156" s="4" t="n"/>
+      <c r="G156" s="4" t="n"/>
+      <c r="H156" s="4" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_item_price.php</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | New. List / save row / bulk calls - login, csrf, ITEM C or admin; cost and margin worked out on the server.</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="n"/>
+      <c r="D157" s="4" t="n"/>
+      <c r="E157" s="4" t="n"/>
+      <c r="F157" s="4" t="n"/>
+      <c r="G157" s="4" t="n"/>
+      <c r="H157" s="4" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>db/post_upload_161026.sql</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | New. Two menus + rights for Item creators, index on tbl_item_stock.item_id and tbl_itemprice_history (item_id, branch_id), stored margins recalculated on cost.</t>
+        </is>
+      </c>
+      <c r="C158" s="4" t="n"/>
+      <c r="D158" s="4" t="n"/>
+      <c r="E158" s="4" t="n"/>
+      <c r="F158" s="4" t="n"/>
+      <c r="G158" s="4" t="n"/>
+      <c r="H158" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3589,7 +3883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4103,8 +4397,16 @@
           <t>2026-09-22 | (no schema change) | Qty columns are now only written through fnApplyStockMovement(), never directly.</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | item_id | Index added - lookups by item scanned the whole table.</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | ho / kl / rjpm _item_margin | Recalculated on cost: (selling - cost) / cost x 100, 0 without cost or selling. Prices untouched.</t>
+        </is>
+      </c>
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
@@ -4318,7 +4620,11 @@
           <t>2026-09-22 | item_curr_stock | No change. Noted as dead - every write to it was already commented out. Branch columns in tbl_item_stock are the live balance.</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | margin_percent | Recalculated on cost, same rule. Head Office price changes from the new screens are copied here.</t>
+        </is>
+      </c>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
@@ -4341,8 +4647,16 @@
           <t>2026-10-15 | (rows) | One per SPAC item per branch for the 28% -&gt; 30% discount change.</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | item_branch | Index (item_id, branch_id) added.</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | (rows) | One per item per branch for every change from Bulk Discount / Margin and Item Price Update.</t>
+        </is>
+      </c>
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
@@ -4445,6 +4759,29 @@
       <c r="L30" s="4" t="n"/>
       <c r="M30" s="4" t="n"/>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>mst_sub_menu / tbl_user_rights</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | (rows) | Item Masters &gt; Bulk Discount / Margin and Item Price Update; rights for Item creators (ITEM C).</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="n"/>
+      <c r="K31" s="4" t="n"/>
+      <c r="L31" s="4" t="n"/>
+      <c r="M31" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Price screens: loader while loading / saving, branches on their own line; item list: principal filter, brand / search values made safe in the list query
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H158"/>
+  <dimension ref="A1:H159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2817,7 +2817,11 @@
           <t>2026-10-13 | Edit / price / branch / delete links for creators in Task Settings (ITEM C) - was admin at head office.</t>
         </is>
       </c>
-      <c r="C104" s="4" t="n"/>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | Principal filter; brand / principal as numbers and search text quoted - they went into the sql as typed.</t>
+        </is>
+      </c>
       <c r="D104" s="4" t="n"/>
       <c r="E104" s="4" t="n"/>
       <c r="F104" s="4" t="n"/>
@@ -3757,7 +3761,11 @@
           <t>2026-10-16 | New. One price rule for every screen: cost = price less discount, margin % on cost; selling changes only from margin or selling.</t>
         </is>
       </c>
-      <c r="C152" s="4" t="n"/>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | fnPrice.busy() - small please-wait loader over the page, calls can overlap.</t>
+        </is>
+      </c>
       <c r="D152" s="4" t="n"/>
       <c r="E152" s="4" t="n"/>
       <c r="F152" s="4" t="n"/>
@@ -3775,7 +3783,11 @@
           <t>2026-10-16 | New screen Item Masters &gt; Bulk Discount / Margin - one discount or margin % for a filtered item set in chosen branches, one save, history per row.</t>
         </is>
       </c>
-      <c r="C153" s="4" t="n"/>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | Loader while loading / redrawing / saving; preview redraws 300 ms after typing; branches on their own line.</t>
+        </is>
+      </c>
       <c r="D153" s="4" t="n"/>
       <c r="E153" s="4" t="n"/>
       <c r="F153" s="4" t="n"/>
@@ -3793,7 +3805,11 @@
           <t>2026-10-16 | New screen Item Masters &gt; Item Price Update - filtered list of one branch, price / discount / margin / selling boxes, save per row.</t>
         </is>
       </c>
-      <c r="C154" s="4" t="n"/>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | Loader while loading and saving a row.</t>
+        </is>
+      </c>
       <c r="D154" s="4" t="n"/>
       <c r="E154" s="4" t="n"/>
       <c r="F154" s="4" t="n"/>
@@ -3871,6 +3887,24 @@
       <c r="F158" s="4" t="n"/>
       <c r="G158" s="4" t="n"/>
       <c r="H158" s="4" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>lst_item_details.php</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | Principal filter (name - code) next to Brand.</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="n"/>
+      <c r="D159" s="4" t="n"/>
+      <c r="E159" s="4" t="n"/>
+      <c r="F159" s="4" t="n"/>
+      <c r="G159" s="4" t="n"/>
+      <c r="H159" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
GRN payment: status in the list, bill amount edit, multiple GRN bills
- Multiple GRN bill: picked GRNs linked by supplier and branch (were only linked on the same PO,
  so they stayed Not Yet though paid on the main GRN); dropdown leaves out GRNs on another bill;
  main GRN lists only the GRNs actually linked; un-picking releases them
- Bill amount save: status and balance from the payments made (was reset to Pending and kept the
  old balance); bill below the paid amount refused on the server. Payment save: balance on the server
- Payments table balance takes all payments (was the first one only), paise kept
- GRN payment list: status as saved, paid 0.00 when none; filters / sort as numbers, search quoted;
  list page sets its status filter before use (PHP 8 warning broke the page script)
- db/grn_pay_status_fix_221026.sql: links GRNs of old multiple bills, recalculates status and
  balance, lists GRNs billed twice for review
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H159"/>
+  <dimension ref="A1:H160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1742,7 +1742,11 @@
           <t>2026-10-13 | Edit paid amount for approvers in Task Settings (GRN_PAYMENT A) - was admin.</t>
         </is>
       </c>
-      <c r="F53" s="4" t="n"/>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | Bill save: status and balance from payments made (was reset to Pending, old balance kept); bill below paid refused. Payment save: balance worked out on the server. Multiple GRN linked by supplier and branch (was same PO only); payments table balance uses all payments.</t>
+        </is>
+      </c>
       <c r="G53" s="4" t="n"/>
       <c r="H53" s="4" t="n"/>
     </row>
@@ -2607,7 +2611,11 @@
           <t>2026-10-13 | Branch filter for viewers in Task Settings (GRN_PAYMENT W) - was head office.</t>
         </is>
       </c>
-      <c r="C93" s="4" t="n"/>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | Status filter and page number set before use - PHP 8 warning broke the page script.</t>
+        </is>
+      </c>
       <c r="D93" s="4" t="n"/>
       <c r="E93" s="4" t="n"/>
       <c r="F93" s="4" t="n"/>
@@ -2781,7 +2789,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (GRN_PAYMENT W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C102" s="4" t="n"/>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | Status from the saved status, paid 0.00 when none; filters / sort as numbers and column names, search quoted.</t>
+        </is>
+      </c>
       <c r="D102" s="4" t="n"/>
       <c r="E102" s="4" t="n"/>
       <c r="F102" s="4" t="n"/>
@@ -3905,6 +3917,24 @@
       <c r="F159" s="4" t="n"/>
       <c r="G159" s="4" t="n"/>
       <c r="H159" s="4" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>db/grn_pay_status_fix_221026.sql</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | New. Links GRNs of old multiple bills, recalculates GRN payment status and balance, lists GRNs billed twice for review.</t>
+        </is>
+      </c>
+      <c r="C160" s="4" t="n"/>
+      <c r="D160" s="4" t="n"/>
+      <c r="E160" s="4" t="n"/>
+      <c r="F160" s="4" t="n"/>
+      <c r="G160" s="4" t="n"/>
+      <c r="H160" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3917,7 +3947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4796,12 +4826,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>mst_sub_menu / tbl_user_rights</t>
+          <t>tbl_grn (GRN payment)</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>2026-10-16 | (rows) | Item Masters &gt; Bulk Discount / Margin and Item Price Update; rights for Item creators (ITEM C).</t>
+          <t>2026-10-22 | grn_pay_finished_status / grn_bal_value | Recalculated from the payments; pay_type / grn_ids set on GRNs covered by another GRN's multiple bill.</t>
         </is>
       </c>
       <c r="C31" s="4" t="n"/>
@@ -4816,6 +4846,29 @@
       <c r="L31" s="4" t="n"/>
       <c r="M31" s="4" t="n"/>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>mst_sub_menu / tbl_user_rights</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16 | (rows) | Item Masters &gt; Bulk Discount / Margin and Item Price Update; rights for Item creators (ITEM C).</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="n"/>
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="4" t="n"/>
+      <c r="K32" s="4" t="n"/>
+      <c r="L32" s="4" t="n"/>
+      <c r="M32" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
GRN payment: no-bill check by amount, not the text '0.000' (bill amount was locked with a 2-decimal amount); Multiple rows open the main GRN's payment
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -1747,7 +1747,11 @@
           <t>2026-10-22 | Bill save: status and balance from payments made (was reset to Pending, old balance kept); bill below paid refused. Payment save: balance worked out on the server. Multiple GRN linked by supplier and branch (was same PO only); payments table balance uses all payments.</t>
         </is>
       </c>
-      <c r="G53" s="4" t="n"/>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | No bill yet checked as amount 0, not the text '0.000' - with a 2-decimal amount the bill amount was locked and Save hidden.</t>
+        </is>
+      </c>
       <c r="H53" s="4" t="n"/>
     </row>
     <row r="54">
@@ -2794,7 +2798,11 @@
           <t>2026-10-22 | Status from the saved status, paid 0.00 when none; filters / sort as numbers and column names, search quoted.</t>
         </is>
       </c>
-      <c r="D102" s="4" t="n"/>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | Multiple rows: edit icon opens the main GRN's payment page.</t>
+        </is>
+      </c>
       <c r="E102" s="4" t="n"/>
       <c r="F102" s="4" t="n"/>
       <c r="G102" s="4" t="n"/>

</xml_diff>

<commit_message>
Sales Order Report: Partial opens the SO's items and their stage (pending by default, show all); status counts dispatched qty, not the ordered qty repeated per DC
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3929,12 +3929,12 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>db/grn_pay_status_fix_221026.sql</t>
+          <t>rpt_sales_order.php</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>2026-10-22 | New. Links GRNs of old multiple bills, recalculates GRN payment status and balance, lists GRNs billed twice for review.</t>
+          <t>2026-10-22 | Partial opens a popup with the SO's items and their stage (linked to a page that does not exist); dispatched qty from dc_dispatch_qty (dc_qty repeats the ordered qty per DC); dead fnValidate() call removed.</t>
         </is>
       </c>
       <c r="C160" s="4" t="n"/>
@@ -3943,6 +3943,42 @@
       <c r="F160" s="4" t="n"/>
       <c r="G160" s="4" t="n"/>
       <c r="H160" s="4" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_so_item_status.php</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | New. SO items with ordered / DC / invoiced / pending qty, stock, stage, DC and invoice numbers - login + csrf.</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="n"/>
+      <c r="D161" s="4" t="n"/>
+      <c r="E161" s="4" t="n"/>
+      <c r="F161" s="4" t="n"/>
+      <c r="G161" s="4" t="n"/>
+      <c r="H161" s="4" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>db/grn_pay_status_fix_221026.sql</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | New. Links GRNs of old multiple bills, recalculates GRN payment status and balance, lists GRNs billed twice for review.</t>
+        </is>
+      </c>
+      <c r="C162" s="4" t="n"/>
+      <c r="D162" s="4" t="n"/>
+      <c r="E162" s="4" t="n"/>
+      <c r="F162" s="4" t="n"/>
+      <c r="G162" s="4" t="n"/>
+      <c r="H162" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Purchase Order Report with status and items popup; items popup centred in the existing modal style; indexes on PO / GRN / SO / DC / invoice link columns
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H162"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3937,7 +3937,11 @@
           <t>2026-10-22 | Partial opens a popup with the SO's items and their stage (linked to a page that does not exist); dispatched qty from dc_dispatch_qty (dc_qty repeats the ordered qty per DC); dead fnValidate() call removed.</t>
         </is>
       </c>
-      <c r="C160" s="4" t="n"/>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | Items popup now the shared centred one (was a full-width popup at the top).</t>
+        </is>
+      </c>
       <c r="D160" s="4" t="n"/>
       <c r="E160" s="4" t="n"/>
       <c r="F160" s="4" t="n"/>
@@ -3955,7 +3959,11 @@
           <t>2026-10-22 | New. SO items with ordered / DC / invoiced / pending qty, stock, stage, DC and invoice numbers - login + csrf.</t>
         </is>
       </c>
-      <c r="C161" s="4" t="n"/>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | Rows marked for the shared popup.</t>
+        </is>
+      </c>
       <c r="D161" s="4" t="n"/>
       <c r="E161" s="4" t="n"/>
       <c r="F161" s="4" t="n"/>
@@ -3979,6 +3987,54 @@
       <c r="F162" s="4" t="n"/>
       <c r="G162" s="4" t="n"/>
       <c r="H162" s="4" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>inc/common/doc_items_modal.php</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | New. Centred popup in the existing modal style (bg-modal header / footer, Show all items in the footer) shared by the sales order and purchase order reports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>rpt_purchase_order.php</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | New. Report &gt; Purchase Order Report: approved POs, GRNs, items fully received, status Pending / Partial / Completed from accepted qty on finalised GRNs; status opens the items popup. PO viewers pick any branch, others their own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_po_item_status.php</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | New. PO items with ordered / received / accepted / rejected / returned / to receive, stock, stage, GRN and return numbers - login + csrf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>db/post_upload_221026.sql</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | New. Report &gt; Purchase Order Report menu (rights as Sales Order Report); indexes on the PO / GRN / SO / DC / invoice link columns.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3991,7 +4047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4901,7 +4957,11 @@
           <t>2026-10-16 | (rows) | Item Masters &gt; Bulk Discount / Margin and Item Price Update; rights for Item creators (ITEM C).</t>
         </is>
       </c>
-      <c r="C32" s="4" t="n"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | (rows) | Report &gt; Purchase Order Report (rpt_purchase_order.php); rights for users who have the Sales Order Report.</t>
+        </is>
+      </c>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
@@ -4913,6 +4973,30 @@
       <c r="L32" s="4" t="n"/>
       <c r="M32" s="4" t="n"/>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>tbl_grn / tbl_grn_details / tbl_purchase_order_details</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | po_id, (grn_id, grn_item_id), po_id | Indexes added - the reports and GRN screens scanned whole tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>tbl_dc / tbl_dc_details / tbl_invoice / tbl_invoice_details / tbl_sales_order_details / tbl_grn_pay_receipt</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 | so_id, (dc_id, dc_item_id), so_id, inv_id, so_id, grn_id | Indexes added on the link columns.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Principal All option on the price screens; item count on principal / brand masters, delete only when unused; principal-brand pairs sync script
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H166"/>
+  <dimension ref="A1:I169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -474,6 +474,7 @@
     <col width="62" customWidth="1" min="6" max="6"/>
     <col width="62" customWidth="1" min="7" max="7"/>
     <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -515,6 +516,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Change 7</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Change 8</t>
         </is>
       </c>
     </row>
@@ -1465,6 +1471,11 @@
           <t>2026-10-16 | Loads js/price_calc.js.</t>
         </is>
       </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | datatable-col4 setup (4 columns, actions not sortable) for the principal / brand masters.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3601,7 +3612,11 @@
           <t>2026-10-13 | CRITICAL: login + csrf, only the 24 table / column pairs the delete links use, status forced to 0, id bound - it took table, column and value from the post with no login.</t>
         </is>
       </c>
-      <c r="C142" s="4" t="n"/>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | A principal or brand still used by items is refused (409 with the item count).</t>
+        </is>
+      </c>
       <c r="D142" s="4" t="n"/>
       <c r="E142" s="4" t="n"/>
       <c r="F142" s="4" t="n"/>
@@ -3847,7 +3862,11 @@
           <t>2026-10-16 | New. Principal / brand / division / item type / search filters shared by the two screens.</t>
         </is>
       </c>
-      <c r="C155" s="4" t="n"/>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | Principal dropdown without data-placeholder - the --- All --- option was taken as the placeholder and hidden on Bulk Discount / Margin and Item Price Update.</t>
+        </is>
+      </c>
       <c r="D155" s="4" t="n"/>
       <c r="E155" s="4" t="n"/>
       <c r="F155" s="4" t="n"/>
@@ -4033,6 +4052,42 @@
       <c r="B166" s="3" t="inlineStr">
         <is>
           <t>2026-10-22 | New. Report &gt; Purchase Order Report menu (rights as Sales Order Report); indexes on the PO / GRN / SO / DC / invoice link columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>mst_principal.php</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | Items column (active items mapped); delete icon only when no item uses the principal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>mst_brand.php</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | Items column (active items mapped); delete icon only when no item uses the brand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>db/principal_brand_sync_231026.sql</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | New. Stanley / Taparia / Chicago Pneumatic / Shree Prayag: brand created when missing, items with the principal get the brand and items with the brand get the principal where the other side is empty or Not Applicable; items with a different real principal / brand listed, not changed.</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4789,7 +4844,11 @@
           <t>2026-10-16 | margin_percent | Recalculated on cost, same rule. Head Office price changes from the new screens are copied here.</t>
         </is>
       </c>
-      <c r="D25" s="4" t="n"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | item_principal / item_brand_make | The four principal-brand pairs filled in where one side was empty or Not Applicable.</t>
+        </is>
+      </c>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="4" t="n"/>
@@ -4997,6 +5056,18 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>mst_brand</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | (rows) | SHREE PRAYAG (SPAC) created; CHICAGO PNEUMATIC / STANLEY / TAPARIA only when missing.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Principal-brand sync: find principals by name too (live codes STANELY / TAPARIA were missed), Chicago uses brand CP, drop unused duplicate brand; optional override for items with another principal
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I169"/>
+  <dimension ref="A1:I170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -4088,6 +4088,23 @@
       <c r="B169" s="3" t="inlineStr">
         <is>
           <t>2026-10-23 | New. Stanley / Taparia / Chicago Pneumatic / Shree Prayag: brand created when missing, items with the principal get the brand and items with the brand get the principal where the other side is empty or Not Applicable; items with a different real principal / brand listed, not changed.</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | Second version: principals found by name as well as code (live codes STANELY / TAPARIA were missed, so Stanley and Taparia were skipped); Chicago uses the existing brand CP; the duplicate CHICAGO PNEUMATIC brand removed when unused; a pair not found is shown, not skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>db/principal_brand_override_231026.sql</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | New, optional. Items with a STANLEY / TAPARIA / CP brand but another real principal (Customize, MULTIBRAND, HONDA, YAMAHA - 45 on live) get the brand's company as principal; lists the changes first.</t>
         </is>
       </c>
     </row>
@@ -5067,6 +5084,11 @@
           <t>2026-10-23 | (rows) | SHREE PRAYAG (SPAC) created; CHICAGO PNEUMATIC / STANLEY / TAPARIA only when missing.</t>
         </is>
       </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 | (rows) | CHICAGO PNEUMATIC (made by the first sync version, unused) set to status 0 - Chicago Pneumatics uses brand CP.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Reports: read lookups once per report instead of once per row
Stock lists, branch wise stock, SO stock list, item details check and the
sales order report ran one query per row for names, units, GST, stock and
DC / invoice figures (up to 21,000 queries per click). Each lookup is now one
query for the whole report (20-40 queries in all); output is unchanged.
New dbhandler GetMap / MapValue helpers.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I170"/>
+  <dimension ref="A1:I174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1720,7 +1720,11 @@
           <t>2026-10-06 | Branch columns driven from mst_branch. The header looped the branch table but the rows wrote only ho_stock and kl_stock, so Rajapalayam had a header and no cells. An item with no tbl_item_stock row now reads 0.000 instead of dropping its cells, the item lookup is bound, and the empty-state colspan follows the branch count.</t>
         </is>
       </c>
-      <c r="C52" s="4" t="n"/>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Units, GST, stock rows and selling price read once for the whole report (14,035 -&gt; 26 queries). Output unchanged.</t>
+        </is>
+      </c>
       <c r="D52" s="4" t="n"/>
       <c r="E52" s="4" t="n"/>
       <c r="F52" s="4" t="n"/>
@@ -3368,7 +3372,11 @@
           <t>2026-10-13 | Update location for creators in Task Settings (STOCK_LOCATION C) - was users 1 and 9.</t>
         </is>
       </c>
-      <c r="C130" s="4" t="n"/>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Branch stock and open SO qty read once for the whole report (16,845 -&gt; 28 queries, 13.9 s -&gt; 0.4 s on 8,900 items). Output unchanged.</t>
+        </is>
+      </c>
       <c r="D130" s="4" t="n"/>
       <c r="E130" s="4" t="n"/>
       <c r="F130" s="4" t="n"/>
@@ -3961,7 +3969,11 @@
           <t>2026-10-22 | Items popup now the shared centred one (was a full-width popup at the top).</t>
         </is>
       </c>
-      <c r="D160" s="4" t="n"/>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | SO qty, DC / invoice lists and counts, totals, customer names read once for all SOs listed (5,891 -&gt; 39 queries); unused per-DC lookups removed. Output unchanged.</t>
+        </is>
+      </c>
       <c r="E160" s="4" t="n"/>
       <c r="F160" s="4" t="n"/>
       <c r="G160" s="4" t="n"/>
@@ -4105,6 +4117,54 @@
       <c r="B170" s="3" t="inlineStr">
         <is>
           <t>2026-10-23 | New, optional. Items with a STANLEY / TAPARIA / CP brand but another real principal (Customize, MULTIBRAND, HONDA, YAMAHA - 45 on live) get the brand's company as principal; lists the changes first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>rpt_branch_wise_stock.php</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Units and branch stock read once for the whole report (21,049 -&gt; 27 queries). Output unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>rpt_store_stock_list.php</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Descriptions and units read once for the whole report (12,623 -&gt; 21 queries). Output unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>rpt_item_details_check.php</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Units and HSN codes read once for the whole report (12,621 -&gt; 20 queries). Output unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>inc/common/dbhandler.php</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | New GetMap (whole lookup in one query) and MapValue (value per key, same as GetSingleReconrd gives).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sales Order list and GRN Payments pending: read lookups once per page
Both looked up DC / invoice / quotation figures and supplier details with
one query per row. Now one query per lookup for the rows shown
(392 -> 33 and 1,512 -> 21 queries); output unchanged.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -2991,7 +2991,11 @@
           <t>2026-10-13 | Cancel link moved to its own task SO_CANCEL (admin) - approve and cancel are different people.</t>
         </is>
       </c>
-      <c r="D111" s="4" t="n"/>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Item count, qty, DC, dispatched qty, invoice and quotation lookups read once for the page's SOs (392 -&gt; 33 queries per page). Output unchanged.</t>
+        </is>
+      </c>
       <c r="E111" s="4" t="n"/>
       <c r="F111" s="4" t="n"/>
       <c r="G111" s="4" t="n"/>
@@ -3602,7 +3606,11 @@
           <t>2026-10-13 | List limited to the branches the user approves for, same rule as the tile.</t>
         </is>
       </c>
-      <c r="C141" s="4" t="n"/>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Supplier name / credit days and paid amount read once for the list, not 3 queries per GRN (1,512 -&gt; 21 queries). Output unchanged.</t>
+        </is>
+      </c>
       <c r="D141" s="4" t="n"/>
       <c r="E141" s="4" t="n"/>
       <c r="F141" s="4" t="n"/>

</xml_diff>

<commit_message>
Big reports: show 100 rows a page with search, exports keep every row
The stock / item reports drew every row (up to 38,000 cells and 2,000
photos) on load. Rows now sit in a template and are paged by
js/report_rows.js; Excel, PDF and Print still take all rows in their
original order.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I174"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1725,7 +1725,11 @@
           <t>2026-10-26 | Units, GST, stock rows and selling price read once for the whole report (14,035 -&gt; 26 queries). Output unchanged.</t>
         </is>
       </c>
-      <c r="D52" s="4" t="n"/>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Rows shown 100 a page with search; photos load only for the rows shown (5.5 s -&gt; 1.4 s). Exports unchanged.</t>
+        </is>
+      </c>
       <c r="E52" s="4" t="n"/>
       <c r="F52" s="4" t="n"/>
       <c r="G52" s="4" t="n"/>
@@ -3381,7 +3385,11 @@
           <t>2026-10-26 | Branch stock and open SO qty read once for the whole report (16,845 -&gt; 28 queries, 13.9 s -&gt; 0.4 s on 8,900 items). Output unchanged.</t>
         </is>
       </c>
-      <c r="D130" s="4" t="n"/>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Rows shown 100 a page with search (js/report_rows.js); 8.9 s -&gt; 1.0 s to usable page. Exports unchanged.</t>
+        </is>
+      </c>
       <c r="E130" s="4" t="n"/>
       <c r="F130" s="4" t="n"/>
       <c r="G130" s="4" t="n"/>
@@ -4139,6 +4147,11 @@
           <t>2026-10-26 | Units and branch stock read once for the whole report (21,049 -&gt; 27 queries). Output unchanged.</t>
         </is>
       </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Rows shown 100 a page with search (4.3 s -&gt; 1.0 s). Exports unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -4151,6 +4164,11 @@
           <t>2026-10-26 | Descriptions and units read once for the whole report (12,623 -&gt; 21 queries). Output unchanged.</t>
         </is>
       </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Rows shown 100 a page with search (1.9 s -&gt; 1.0 s). Exports unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -4163,6 +4181,11 @@
           <t>2026-10-26 | Units and HSN codes read once for the whole report (12,621 -&gt; 20 queries). Output unchanged.</t>
         </is>
       </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Rows shown 100 a page with search (2.1 s -&gt; 0.5 s).</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -4173,6 +4196,30 @@
       <c r="B174" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 | New GetMap (whole lookup in one query) and MapValue (value per key, same as GetSingleReconrd gives).</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>js/report_rows.js</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | New. Report rows held in &lt;template id="rpt_rows"&gt; shown 100 a page with search; Excel / PDF / Print get every row for that click.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>rpt_item_discount.php</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Rows shown 100 a page with search (3.5 s -&gt; 0.7 s). Exports unchanged.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Every page: sidebar and menu lookup in fewer queries, one shared dbhandler connection
Sidebar read sub menus (and user rights) once per main menu; now one query.
The current page's menu took two lookups; now one. dbhandler objects share
one connection per request. Quotation list proforma lookup read once per
page. Output unchanged.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I176"/>
+  <dimension ref="A1:I178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2950,7 +2950,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (QUOTATION W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C109" s="4" t="n"/>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Proforma per quotation read once for the page (was one query per row).</t>
+        </is>
+      </c>
       <c r="D109" s="4" t="n"/>
       <c r="E109" s="4" t="n"/>
       <c r="F109" s="4" t="n"/>
@@ -4198,6 +4202,11 @@
           <t>2026-10-26 | New GetMap (whole lookup in one query) and MapValue (value per key, same as GetSingleReconrd gives).</t>
         </is>
       </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | One connection shared by all dbhandler objects of a request (was a new connection each); new GetRow (prepared, first row).</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -4220,6 +4229,30 @@
       <c r="B176" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 | Rows shown 100 a page with search (3.5 s -&gt; 0.7 s). Exports unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>inc/common/sidebar.php</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | All visible sub menus in one query grouped per main menu (was 1-2 queries per main menu). Same menus and HTML.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>inc/common/active_menu.php</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Page's sub menu and main menu in one prepared query (was two).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Indexes on link columns that pages look rows up by (db/post_upload_261026.sql)
Found by opening every menu page with the query log on and running EXPLAIN
on each query: lookups by quo_id, si_id, inv_id, supp_id, item_id etc. read
the whole table each time. 24 indexes, no data changes, safe to re-run.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I178"/>
+  <dimension ref="A1:I179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -4256,6 +4256,18 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>db/post_upload_261026.sql</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | New. 24 indexes on link columns found by EXPLAIN on every menu page; only indexes, safe to run again.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4267,7 +4279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4595,7 +4607,11 @@
           <t>2026-10-05 | cgst_per, sgst_per, igst_per, cgst_val, sgst_val, igst_val | Optional tidy on the same 111 rows only.</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | item_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
@@ -5238,6 +5254,258 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>tbl_quotation_details</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | quo_id, item_id - lookups by these columns were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>tbl_quo_pack_details</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | quo_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>tbl_invoice_pack_details</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | inv_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>tbl_sales_order_pack_dts</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | so_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>tbl_store_indent_details</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | si_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>tbl_po_prepare_dets</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | po_prepare_id, si_id - lookups by these columns were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>tbl_po_prepare</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | si_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>tbl_po_print_details</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | po_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>tbl_package_box_details</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | dc_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>tbl_item_group_details</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | item_group_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>tbl_attendance</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | emp_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>tbl_quotation</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | supp_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>tbl_purchase_order</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | supp_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>tbl_grn</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | supp_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>tbl_invoice</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | supp_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>tbl_sales_order</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | quo_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>tbl_receipt</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | so_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>tbl_dc</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | dc_inv_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>tbl_sales_order_details</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | item_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>tbl_purchase_order_details</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | item_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>tbl_spare_mapping</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | (index) | item_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Quotation branch report, invoice report, PO prepare list: read lookups once
Same per-row lookup fix as the other reports (3,606 -> 17, 901 -> 19 and
about 450 -> 22 queries); output unchanged. COUNT defaults in the lookup
helpers are the number 0, as the old per-row counts returned.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I179"/>
+  <dimension ref="A1:I180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2914,7 +2914,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (PO_PREPARE W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C107" s="4" t="n"/>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | PO prepare / indent lookups read once for the page's indents (about 450 -&gt; 22 queries); unused lookups removed. Output unchanged.</t>
+        </is>
+      </c>
       <c r="D107" s="4" t="n"/>
       <c r="E107" s="4" t="n"/>
       <c r="F107" s="4" t="n"/>
@@ -3004,7 +3008,11 @@
           <t>2026-10-26 | Item count, qty, DC, dispatched qty, invoice and quotation lookups read once for the page's SOs (392 -&gt; 33 queries per page). Output unchanged.</t>
         </is>
       </c>
-      <c r="E111" s="4" t="n"/>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Item count for an SO with no lines is the number 0, as the old count gave.</t>
+        </is>
+      </c>
       <c r="F111" s="4" t="n"/>
       <c r="G111" s="4" t="n"/>
       <c r="H111" s="4" t="n"/>
@@ -3680,7 +3688,11 @@
           <t>2026-10-14 | Customer branch read from cus_branch_id - it used branch_id (our branch), so every invoice showed customer branch 1 or 2, even for customers without a branch.</t>
         </is>
       </c>
-      <c r="C144" s="4" t="n"/>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Customer names and invoice / pack totals read once for the report (901 -&gt; 19 queries). Output unchanged.</t>
+        </is>
+      </c>
       <c r="D144" s="4" t="n"/>
       <c r="E144" s="4" t="n"/>
       <c r="F144" s="4" t="n"/>
@@ -3994,7 +4006,11 @@
           <t>2026-10-26 | SO qty, DC / invoice lists and counts, totals, customer names read once for all SOs listed (5,891 -&gt; 39 queries); unused per-DC lookups removed. Output unchanged.</t>
         </is>
       </c>
-      <c r="E160" s="4" t="n"/>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | DC / invoice counts for an SO with none are the number 0, as the old count gave.</t>
+        </is>
+      </c>
       <c r="F160" s="4" t="n"/>
       <c r="G160" s="4" t="n"/>
       <c r="H160" s="4" t="n"/>
@@ -4207,6 +4223,11 @@
           <t>2026-10-26 | One connection shared by all dbhandler objects of a request (was a new connection each); new GetRow (prepared, first row).</t>
         </is>
       </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | MapValue note: COUNT default is 0 (number).</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -4265,6 +4286,18 @@
       <c r="B179" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 | New. 24 indexes on link columns found by EXPLAIN on every menu page; only indexes, safe to run again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>quotation_branch_rept.php</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 | Customer names and item counts read once for the report (3,606 -&gt; 17 queries). Output unchanged.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GRN pending bill due date from the party bill date; Item Discount max column
Bill Due Date added the credit days to an unset variable, so it showed today
+ credit days. Max Discount checked the min value and showed '-' whenever the
min was 0.
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -3631,7 +3631,11 @@
           <t>2026-10-26 | Supplier name / credit days and paid amount read once for the list, not 3 queries per GRN (1,512 -&gt; 21 queries). Output unchanged.</t>
         </is>
       </c>
-      <c r="D141" s="4" t="n"/>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Bill Due Date = party bill date + supplier credit days (was today + credit days - unset variable); badge follows it.</t>
+        </is>
+      </c>
       <c r="E141" s="4" t="n"/>
       <c r="F141" s="4" t="n"/>
       <c r="G141" s="4" t="n"/>
@@ -4250,6 +4254,11 @@
       <c r="B176" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 | Rows shown 100 a page with search (3.5 s -&gt; 0.7 s). Exports unchanged.</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Max Discount shown whenever a max is set (it checked the min, so showed '-' when min was 0).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix defects confirmed from the 27-10 list / report audit
- search / sort input made safe for SQL on all list endpoints and three
  reports (an apostrophe in a search box broke 23 pages)
- all-branches stock list no longer stops at row 2,001 on PHP 8
- stock reports list each item once (extra stock join removed)
- broken sorts fixed: customer #, GRN payment supplier, PO prepare status;
  item price history search / sort on real columns, no reused stock values
- invoice report keeps the chosen dates, Print / PDF area exists
- delete cancel script error, DC sales popup id, spare mapping item link,
  active menu for URLs stored with a line break
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I180"/>
+  <dimension ref="A1:I206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -965,7 +965,11 @@
           <t>2026-09-23 | New. Rows for the stock list. One stock column per active branch, read from mst_branch.</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
@@ -1730,7 +1734,11 @@
           <t>2026-10-26 | Rows shown 100 a page with search; photos load only for the rows shown (5.5 s -&gt; 1.4 s). Exports unchanged.</t>
         </is>
       </c>
-      <c r="E52" s="4" t="n"/>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Missing price / GST count as 0 - PHP 8 type error stopped the report at row 2,001.</t>
+        </is>
+      </c>
       <c r="F52" s="4" t="n"/>
       <c r="G52" s="4" t="n"/>
       <c r="H52" s="4" t="n"/>
@@ -1929,7 +1937,11 @@
           <t>2026-10-14 | fnIsLoggedIn(); isAdmin also needs the user id and branch - a session with only _user=crm_user (another app on the server) opened pages with no user or branch.</t>
         </is>
       </c>
-      <c r="D60" s="4" t="n"/>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | New fnSqlText / fnSqlColumn / fnSqlDir - search and sort input safe in SQL.</t>
+        </is>
+      </c>
       <c r="E60" s="4" t="n"/>
       <c r="F60" s="4" t="n"/>
       <c r="G60" s="4" t="n"/>
@@ -2682,7 +2694,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (DC W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C95" s="4" t="n"/>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Sales Details popup given the SO id (was DC id); search / sort input safe.</t>
+        </is>
+      </c>
       <c r="D95" s="4" t="n"/>
       <c r="E95" s="4" t="n"/>
       <c r="F95" s="4" t="n"/>
@@ -2700,7 +2716,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C96" s="4" t="n"/>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D96" s="4" t="n"/>
       <c r="E96" s="4" t="n"/>
       <c r="F96" s="4" t="n"/>
@@ -2718,7 +2738,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C97" s="4" t="n"/>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D97" s="4" t="n"/>
       <c r="E97" s="4" t="n"/>
       <c r="F97" s="4" t="n"/>
@@ -2736,7 +2760,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C98" s="4" t="n"/>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D98" s="4" t="n"/>
       <c r="E98" s="4" t="n"/>
       <c r="F98" s="4" t="n"/>
@@ -2759,7 +2787,11 @@
           <t>2026-10-13 | Own branch only without the Employee viewer role - every branch showed.</t>
         </is>
       </c>
-      <c r="D99" s="4" t="n"/>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="E99" s="4" t="n"/>
       <c r="F99" s="4" t="n"/>
       <c r="G99" s="4" t="n"/>
@@ -2776,7 +2808,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C100" s="4" t="n"/>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D100" s="4" t="n"/>
       <c r="E100" s="4" t="n"/>
       <c r="F100" s="4" t="n"/>
@@ -2794,7 +2830,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (GRN W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C101" s="4" t="n"/>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D101" s="4" t="n"/>
       <c r="E101" s="4" t="n"/>
       <c r="F101" s="4" t="n"/>
@@ -2822,7 +2862,11 @@
           <t>2026-10-22 | Multiple rows: edit icon opens the main GRN's payment page.</t>
         </is>
       </c>
-      <c r="E102" s="4" t="n"/>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Supplier column sorts by supplier name (supp_id ambiguous); sort input checked.</t>
+        </is>
+      </c>
       <c r="F102" s="4" t="n"/>
       <c r="G102" s="4" t="n"/>
       <c r="H102" s="4" t="n"/>
@@ -2838,7 +2882,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (INVOICE W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C103" s="4" t="n"/>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D103" s="4" t="n"/>
       <c r="E103" s="4" t="n"/>
       <c r="F103" s="4" t="n"/>
@@ -2861,7 +2909,11 @@
           <t>2026-10-16 | Principal filter; brand / principal as numbers and search text quoted - they went into the sql as typed.</t>
         </is>
       </c>
-      <c r="D104" s="4" t="n"/>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="E104" s="4" t="n"/>
       <c r="F104" s="4" t="n"/>
       <c r="G104" s="4" t="n"/>
@@ -2878,7 +2930,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C105" s="4" t="n"/>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D105" s="4" t="n"/>
       <c r="E105" s="4" t="n"/>
       <c r="F105" s="4" t="n"/>
@@ -2896,7 +2952,11 @@
           <t>2026-10-13 | Edit links for creators in Task Settings (PURCHASE_ORDER C) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C106" s="4" t="n"/>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D106" s="4" t="n"/>
       <c r="E106" s="4" t="n"/>
       <c r="F106" s="4" t="n"/>
@@ -2919,7 +2979,11 @@
           <t>2026-10-26 | PO prepare / indent lookups read once for the page's indents (about 450 -&gt; 22 queries); unused lookups removed. Output unchanged.</t>
         </is>
       </c>
-      <c r="D107" s="4" t="n"/>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Status filter on the PO prepare rows; search / sort input safe.</t>
+        </is>
+      </c>
       <c r="E107" s="4" t="n"/>
       <c r="F107" s="4" t="n"/>
       <c r="G107" s="4" t="n"/>
@@ -2936,7 +3000,11 @@
           <t>2026-10-13 | GRN cancel link for approvers in Task Settings (GRN A) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C108" s="4" t="n"/>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D108" s="4" t="n"/>
       <c r="E108" s="4" t="n"/>
       <c r="F108" s="4" t="n"/>
@@ -2959,7 +3027,11 @@
           <t>2026-10-26 | Proforma per quotation read once for the page (was one query per row).</t>
         </is>
       </c>
-      <c r="D109" s="4" t="n"/>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="E109" s="4" t="n"/>
       <c r="F109" s="4" t="n"/>
       <c r="G109" s="4" t="n"/>
@@ -2981,7 +3053,11 @@
           <t>2026-10-15 | Revoke next to a confirmed payment (SALES_RECEIPT R).</t>
         </is>
       </c>
-      <c r="D110" s="4" t="n"/>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="E110" s="4" t="n"/>
       <c r="F110" s="4" t="n"/>
       <c r="G110" s="4" t="n"/>
@@ -3013,7 +3089,11 @@
           <t>2026-10-26 | Item count for an SO with no lines is the number 0, as the old count gave.</t>
         </is>
       </c>
-      <c r="F111" s="4" t="n"/>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="G111" s="4" t="n"/>
       <c r="H111" s="4" t="n"/>
     </row>
@@ -3028,7 +3108,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (EMPLOYEE W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C112" s="4" t="n"/>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D112" s="4" t="n"/>
       <c r="E112" s="4" t="n"/>
       <c r="F112" s="4" t="n"/>
@@ -3056,7 +3140,11 @@
           <t>2026-10-15 | Approve page link also for Revokers on approved suppliers.</t>
         </is>
       </c>
-      <c r="E113" s="4" t="n"/>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="F113" s="4" t="n"/>
       <c r="G113" s="4" t="n"/>
       <c r="H113" s="4" t="n"/>
@@ -3072,7 +3160,11 @@
           <t>2026-10-13 | All branches for viewers in Task Settings (STORE_INDENT W) - was admin or head office.</t>
         </is>
       </c>
-      <c r="C114" s="4" t="n"/>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
       <c r="D114" s="4" t="n"/>
       <c r="E114" s="4" t="n"/>
       <c r="F114" s="4" t="n"/>
@@ -3264,7 +3356,11 @@
           <t>2026-10-13 | Branch filter for viewers in Task Settings (PO_PREPARE W) - was head office.</t>
         </is>
       </c>
-      <c r="C124" s="4" t="n"/>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Status not sortable (no column), date sortable.</t>
+        </is>
+      </c>
       <c r="D124" s="4" t="n"/>
       <c r="E124" s="4" t="n"/>
       <c r="F124" s="4" t="n"/>
@@ -3402,7 +3498,11 @@
           <t>2026-10-26 | Rows shown 100 a page with search (js/report_rows.js); 8.9 s -&gt; 1.0 s to usable page. Exports unchanged.</t>
         </is>
       </c>
-      <c r="E130" s="4" t="n"/>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | No stock join (items with 2 stock rows listed twice); no stock row shows 0.000.</t>
+        </is>
+      </c>
       <c r="F130" s="4" t="n"/>
       <c r="G130" s="4" t="n"/>
       <c r="H130" s="4" t="n"/>
@@ -3697,7 +3797,11 @@
           <t>2026-10-26 | Customer names and invoice / pack totals read once for the report (901 -&gt; 19 queries). Output unchanged.</t>
         </is>
       </c>
-      <c r="D144" s="4" t="n"/>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Chosen dates kept; Print / PDF area rpt_division; 5-column spans; search quoted.</t>
+        </is>
+      </c>
       <c r="E144" s="4" t="n"/>
       <c r="F144" s="4" t="n"/>
       <c r="G144" s="4" t="n"/>
@@ -4015,7 +4119,11 @@
           <t>2026-10-26 | DC / invoice counts for an SO with none are the number 0, as the old count gave.</t>
         </is>
       </c>
-      <c r="F160" s="4" t="n"/>
+      <c r="F160" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search text quoted, branch as number (a ' broke the report).</t>
+        </is>
+      </c>
       <c r="G160" s="4" t="n"/>
       <c r="H160" s="4" t="n"/>
     </row>
@@ -4118,6 +4226,11 @@
           <t>2026-10-23 | Items column (active items mapped); delete icon only when no item uses the principal.</t>
         </is>
       </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -4130,6 +4243,11 @@
           <t>2026-10-23 | Items column (active items mapped); delete icon only when no item uses the brand.</t>
         </is>
       </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -4176,6 +4294,11 @@
           <t>2026-10-26 | Rows shown 100 a page with search (4.3 s -&gt; 1.0 s). Exports unchanged.</t>
         </is>
       </c>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | No stock join (items with 2 stock rows listed twice, descriptions lost); no stock row shows 0.000.</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -4261,6 +4384,11 @@
           <t>2026-10-27 | Max Discount shown whenever a max is set (it checked the min, so showed '-' when min was 0).</t>
         </is>
       </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Item's first stock row only (items with 2 stock rows listed twice).</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -4285,6 +4413,11 @@
           <t>2026-10-26 | Page's sub menu and main menu in one prepared query (was two).</t>
         </is>
       </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Line breaks in stored menu URLs ignored (those menus never showed active).</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -4307,6 +4440,323 @@
       <c r="B180" s="3" t="inlineStr">
         <is>
           <t>2026-10-26 | Customer names and item counts read once for the report (3,606 -&gt; 17 queries). Output unchanged.</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search text quoted, branch as number (a ' broke the report).</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_modal_stock_det.php</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxCostWorkSheet.php</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxCustomerList.php</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxIndentList.php</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxItemGroupingList.php</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxItemPriceHistoryList.php</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | One joined query: search on existing columns, sort by shown values, no stock row shows blanks (showed previous row).</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxMappingList.php</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Item name opens the item details popup (linked to a missing page); search / sort input safe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxSalaryPackageList.php</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>inc/datatable/ajaxStoreStockList.php</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Search / sort input through fnSqlText / fnSqlColumn / fnSqlDir (a ' in a search box broke the query).</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>lst_customers.php</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | # column not sortable (sorting by it failed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>lst_item_grouping.php</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>mst_boxtype.php</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>mst_branch.php</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>mst_category.php</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>mst_city.php</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>mst_color.php</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>mst_department.php</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>mst_designation.php</t>
+        </is>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>mst_district.php</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>mst_division.php</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>mst_hsn.php</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>mst_labour.php</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>mst_state.php</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>mst_uom.php</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>mst_user.php</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Delete cancel uses return false (return false() threw a script error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>spare_mapping_list.php</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-27 | Item details popup added for the item name link.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Index file: move the information_schema check into its own file
phpMyAdmin ran the whole batch against information_schema because of the
check query at the end and stopped at the first CREATE INDEX (#1044).
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I206"/>
+  <dimension ref="A1:I207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -4430,6 +4430,11 @@
           <t>2026-10-26 | New. 24 indexes on link columns found by EXPLAIN on every menu page; only indexes, safe to run again.</t>
         </is>
       </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28 | Check query moved out (phpMyAdmin ran the batch against information_schema, #1044).</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -4757,6 +4762,18 @@
       <c r="B206" s="3" t="inlineStr">
         <is>
           <t>2026-10-27 | Item details popup added for the item name link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>db/post_upload_261026_check.sql</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28 | New. Read-only index check for post_upload_261026.sql - run on its own.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Invoice: items can be sold in part quantity (0.2, 0.5, 1.25)
inv_qty was an int, so 0.5 was saved as 1 and 0.2 as 0. It becomes
DECIMAL(12,3) (db/post_upload_301026.sql), the invoice Quantity box takes
up to 3 decimals, and quantities are shown without trailing zeros on the
invoice pages and prints (fnQty).
</commit_message>
<xml_diff>
--- a/docs/BIE_Change_Log.xlsx
+++ b/docs/BIE_Change_Log.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I207"/>
+  <dimension ref="A1:I211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,11 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
-      <c r="G7" s="4" t="n"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30 | Quantity takes decimals (above 0, at most 3 decimals); total qty keeps decimals; rows shown with fnQty.</t>
+        </is>
+      </c>
       <c r="H7" s="4" t="n"/>
     </row>
     <row r="8">
@@ -699,7 +703,11 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="n"/>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30 | Invoice qty and total shown with fnQty.</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="n"/>
     </row>
     <row r="9">
@@ -733,7 +741,11 @@
           <t>2026-10-07 | Posted row counts via fnRowCount() - count() on a single value is fatal on PHP 8. Package dropdown renamed pack_pick so it cannot replace the pack_id[] rows.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="n"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30 | Invoice qty and total shown with fnQty.</t>
+        </is>
+      </c>
       <c r="H9" s="4" t="n"/>
     </row>
     <row r="10">
@@ -1942,7 +1954,11 @@
           <t>2026-10-27 | New fnSqlText / fnSqlColumn / fnSqlDir - search and sort input safe in SQL.</t>
         </is>
       </c>
-      <c r="E60" s="4" t="n"/>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30 | New fnQty() - qty shown up to 3 decimals without trailing zeros.</t>
+        </is>
+      </c>
       <c r="F60" s="4" t="n"/>
       <c r="G60" s="4" t="n"/>
       <c r="H60" s="4" t="n"/>
@@ -4774,6 +4790,54 @@
       <c r="B207" s="3" t="inlineStr">
         <is>
           <t>2026-10-28 | New. Read-only index check for post_upload_261026.sql - run on its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>db/post_upload_301026.sql</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30 | New. tbl_invoice_details.inv_qty to DECIMAL(12,3) - items sold in part qty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>inc/cis_ajax/jquery_po_inv_details.php</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30 | Invoice row qty shown with fnQty (part qty).</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>invoice_print.php</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30 | Qty shown with fnQty (0.5 / 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>quo_invoice_print.php</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30 | Qty shown with fnQty (0.5 / 2).</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5185,11 @@
           <t>2026-10-26 | (index) | item_id - lookups by this column were full table scans. db/post_upload_261026.sql</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-30 | inv_qty int(11) -&gt; DECIMAL(12,3) NOT NULL (part qty). db/post_upload_301026.sql</t>
+        </is>
+      </c>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="n"/>

</xml_diff>